<commit_message>
feat(appraiser): wire live Vertex AI engine into sourcing pipeline and cloud run server
</commit_message>
<xml_diff>
--- a/data/BlueToad_2026-08-22_BidSheet.xlsx
+++ b/data/BlueToad_2026-08-22_BidSheet.xlsx
@@ -438,7 +438,7 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="58" customWidth="1" min="3" max="3"/>
+    <col width="187" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
@@ -491,392 +491,392 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BT-001</t>
+          <t>BT-066</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>vintage cards</t>
+          <t>vintage toys</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Vintage Topps Baseball Cards (1959-69 Golden Era Stars)</t>
+          <t>Lot of six handheld electronic LCD games including Radica titles, late 1990s to 2000s.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>$250-$500</t>
+          <t>$26-$32</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>35</v>
+        <v>5</v>
       </c>
       <c r="F2" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="G2" t="n">
-        <v>115</v>
+        <v>11.5</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>APPROVED</t>
+          <t>AUTO-SEND</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BT-041</t>
+          <t>BT-016</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>phonograph / records</t>
+          <t>vintage cards</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Edison rolls (11-12 canisters + bare roll)</t>
+          <t>Bulk lot of sports trading cards in a multi-row cardboard storage box, predominantly late 20th-century/1980s–2000s issues.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>$100-$160</t>
+          <t>$38-$48</t>
         </is>
       </c>
       <c r="E3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F3" t="n">
         <v>15</v>
       </c>
-      <c r="F3" t="n">
-        <v>40</v>
-      </c>
       <c r="G3" t="n">
-        <v>46</v>
+        <v>17.25</v>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>APPROVED</t>
+          <t>AUTO-SEND</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BT-002</t>
+          <t>BT-030</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>jewelry</t>
+          <t>vintage cards</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Estate Costume Jewelry (Tray 12/14/16: 50-70 pcs)</t>
+          <t>Assorted lot of non-sport trading cards, including MAD Magazine, pop culture, automobile, and entertainment cards, c. 1970s-1990s</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>$80-$160</t>
+          <t>$38-$48</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F4" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="G4" t="n">
-        <v>28.75</v>
+        <v>17.25</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>APPROVED</t>
+          <t>AUTO-SEND</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BT-087</t>
+          <t>BT-235</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>jewelry</t>
+          <t>advertising / bottles</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>costume jewelry (Tray Lot 2)</t>
+          <t>1933 Chicago World's Fair 'A Century of Progress' embossed clear glass commemorative bottle</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>$80-$160</t>
+          <t>$38-$48</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F5" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="G5" t="n">
-        <v>28.75</v>
+        <v>17.25</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>APPROVED</t>
+          <t>AUTO-SEND</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BT-181</t>
+          <t>BT-021</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>jewelry</t>
+          <t>vintage electronics</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>estate costume jewelry (Tray Lot 3)</t>
+          <t>Vintage Bell System / Western Electric pink Touch-Tone Princess telephone in original box, c. 1970s.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>$80-$160</t>
+          <t>$52-$62</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F6" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="G6" t="n">
-        <v>28.75</v>
+        <v>23</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>APPROVED</t>
+          <t>AUTO-SEND</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BT-050</t>
+          <t>BT-048</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>vintage toys</t>
+          <t>vintage smalls</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Lionel building set</t>
+          <t>Vintage E.T. The Extra-Terrestrial ceramic nightlight figure, likely Universal City Studios licensed or craft mold, c. 1982</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>$50-$120</t>
+          <t>$52-$62</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F7" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="G7" t="n">
-        <v>28.75</v>
+        <v>23</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>APPROVED</t>
+          <t>AUTO-SEND</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BT-021</t>
+          <t>BT-002</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>vintage electronics</t>
+          <t>jewelry</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>princess phone</t>
+          <t>Assortment of vintage estate costume jewelry, including beaded necklaces, brooches, chains, pendants, and faux pearls arranged in auction trays.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>$40-$100</t>
+          <t>$65-$75</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F8" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="G8" t="n">
-        <v>23</v>
+        <v>28.75</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>APPROVED</t>
+          <t>AUTO-SEND</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BT-048</t>
+          <t>BT-050</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>vintage smalls</t>
+          <t>vintage toys</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ET nightlight</t>
+          <t>Vintage Lionel metal construction set in fitted wooden carrying case, circa late 1930s.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>$40-$100</t>
+          <t>$65-$75</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F9" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="G9" t="n">
-        <v>23</v>
+        <v>28.75</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>APPROVED</t>
+          <t>AUTO-SEND</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>BT-235</t>
+          <t>BT-087</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>advertising / bottles</t>
+          <t>jewelry</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Century Progress bottle</t>
+          <t>Assorted bulk lot of vintage and modern costume jewelry in a plastic storage bin, including faux pearl strands, beaded necklaces, pins, brooches, and bagged smalls.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>$30-$80</t>
+          <t>$65-$75</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F10" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="G10" t="n">
-        <v>17.25</v>
+        <v>28.75</v>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>APPROVED</t>
+          <t>AUTO-SEND</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>BT-016</t>
+          <t>BT-181</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>vintage cards</t>
+          <t>jewelry</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>trading cards</t>
+          <t>Assorted estate costume jewelry lot including rhinestone brooches (such as Christmas tree pins), faux pearl and beaded necklaces, pendants, and cuff bracelet, mid to late 20th century.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>$30-$80</t>
+          <t>$65-$75</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F11" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="G11" t="n">
-        <v>17.25</v>
+        <v>28.75</v>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>APPROVED</t>
+          <t>AUTO-SEND</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>BT-030</t>
+          <t>BT-041</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>vintage cards</t>
+          <t>phonograph / records</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>non-sport trading cards</t>
+          <t>Group of Edison phonograph cylinder records and containers, Thomas A. Edison, Inc., circa 1902–1929.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>$30-$80</t>
+          <t>$100-$130</t>
         </is>
       </c>
       <c r="E12" t="n">
         <v>10</v>
       </c>
       <c r="F12" t="n">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="G12" t="n">
-        <v>17.25</v>
+        <v>46</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
@@ -887,32 +887,32 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>BT-066</t>
+          <t>BT-001</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>vintage toys</t>
+          <t>vintage cards</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>hand held video games (5 Radica/LCD units)</t>
+          <t>Group of vintage baseball trading cards including Topps and Bowman releases featuring various Major League Baseball players</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>$25-$45</t>
+          <t>$250-$320</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>5</v>
+        <v>35</v>
       </c>
       <c r="F13" t="n">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="G13" t="n">
-        <v>11.5</v>
+        <v>115</v>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat(pipeline): fresh live Vertex AI appraisal run and archive previous run
</commit_message>
<xml_diff>
--- a/data/BlueToad_2026-08-22_BidSheet.xlsx
+++ b/data/BlueToad_2026-08-22_BidSheet.xlsx
@@ -438,7 +438,7 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="187" customWidth="1" min="3" max="3"/>
+    <col width="219" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
@@ -501,7 +501,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Lot of six handheld electronic LCD games including Radica titles, late 1990s to 2000s.</t>
+          <t>Lot of handheld LCD electronic games, including Radica and electronic handheld game titles, c. 1990s-2000s</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -537,7 +537,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Bulk lot of sports trading cards in a multi-row cardboard storage box, predominantly late 20th-century/1980s–2000s issues.</t>
+          <t>Bulk collection of loose sports trading cards (hockey, football, baseball) housed in a multi-row cardboard monster storage box.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -573,7 +573,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Assorted lot of non-sport trading cards, including MAD Magazine, pop culture, automobile, and entertainment cards, c. 1970s-1990s</t>
+          <t>Assorted vintage non-sport trading card collection in plastic cases and top loaders, featuring Garbage Pail Kids, MAD Magazine, classic automobiles, and entertainment sets, Topps and other publishers, c. 1980s-1990s.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -609,7 +609,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1933 Chicago World's Fair 'A Century of Progress' embossed clear glass commemorative bottle</t>
+          <t>1933 Chicago World's Fair 'A Century of Progress' embossed glass souvenir bottle</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -645,7 +645,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Vintage Bell System / Western Electric pink Touch-Tone Princess telephone in original box, c. 1970s.</t>
+          <t>Vintage Western Electric pink Princess push-button (Touch-Tone) telephone with original box, Bell System, c. 1965-1975.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -681,7 +681,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Vintage E.T. The Extra-Terrestrial ceramic nightlight figure, likely Universal City Studios licensed or craft mold, c. 1982</t>
+          <t>Vintage E.T. The Extra-Terrestrial ceramic figure nightlight, likely Universal City Studios licensed or ceramic craft mold, c. 1982.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -717,7 +717,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Assortment of vintage estate costume jewelry, including beaded necklaces, brooches, chains, pendants, and faux pearls arranged in auction trays.</t>
+          <t>Assorted vintage and contemporary estate costume jewelry including beaded necklaces, brooches, chains, pendants, and bracelets in three black jewelry trays (labeled 12, 14, 16)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -753,7 +753,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Vintage Lionel metal construction set in fitted wooden carrying case, circa late 1930s.</t>
+          <t>Vintage metal construction set in wooden case, attributed as Lionel, c. 1930s-1940s</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -789,7 +789,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Assorted bulk lot of vintage and modern costume jewelry in a plastic storage bin, including faux pearl strands, beaded necklaces, pins, brooches, and bagged smalls.</t>
+          <t>Bulk lot of assorted costume jewelry including faux pearls, beaded necklaces, pins, and loose components in a plastic bin</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -825,7 +825,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Assorted estate costume jewelry lot including rhinestone brooches (such as Christmas tree pins), faux pearl and beaded necklaces, pendants, and cuff bracelet, mid to late 20th century.</t>
+          <t>Tray lot of vintage costume jewelry, including rhinestone brooches (notably holiday/Christmas tree designs), beaded multi-strand necklaces, cabochon pendant, and charm elements, mid-to-late 20th century.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -861,7 +861,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Group of Edison phonograph cylinder records and containers, Thomas A. Edison, Inc., circa 1902–1929.</t>
+          <t>Lot of vintage Edison phonograph cylinder record containers and cylinders, Thomas A. Edison, Inc., circa 1900-1920s</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -897,7 +897,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Group of vintage baseball trading cards including Topps and Bowman releases featuring various Major League Baseball players</t>
+          <t>Assortment of vintage baseball trading cards including 1950s and 1960s Topps and Bowman issues in protective top loaders</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">

</xml_diff>

<commit_message>
feat(appraiser): ground truth caption authority eliminates redundant mark questions
</commit_message>
<xml_diff>
--- a/data/BlueToad_2026-08-22_BidSheet.xlsx
+++ b/data/BlueToad_2026-08-22_BidSheet.xlsx
@@ -438,7 +438,7 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="219" customWidth="1" min="3" max="3"/>
+    <col width="173" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
@@ -501,7 +501,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Lot of handheld LCD electronic games, including Radica and electronic handheld game titles, c. 1990s-2000s</t>
+          <t>Collection of vintage electronic handheld LCD games including Radica titles, c. 1990s-2000s</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -537,7 +537,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Bulk collection of loose sports trading cards (hockey, football, baseball) housed in a multi-row cardboard monster storage box.</t>
+          <t>Multi-row cardboard storage box containing large collection of sports trading cards, c. 1980s-2000s</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -573,7 +573,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Assorted vintage non-sport trading card collection in plastic cases and top loaders, featuring Garbage Pail Kids, MAD Magazine, classic automobiles, and entertainment sets, Topps and other publishers, c. 1980s-1990s.</t>
+          <t>Assorted vintage non-sport trading card collection in protective sleeves, including MAD Magazine, automotive, and pop culture cards, c. 1970s-1990s</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -609,7 +609,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1933 Chicago World's Fair 'A Century of Progress' embossed glass souvenir bottle</t>
+          <t>1933 Chicago World's Fair Century of Progress embossed clear glass souvenir bottle</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -645,7 +645,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Vintage Western Electric pink Princess push-button (Touch-Tone) telephone with original box, Bell System, c. 1965-1975.</t>
+          <t>Vintage pink push-button Princess telephone by Western Electric / Bell System in original box, circa 1970s</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -681,7 +681,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Vintage E.T. The Extra-Terrestrial ceramic figure nightlight, likely Universal City Studios licensed or ceramic craft mold, c. 1982.</t>
+          <t>E.T. The Extra-Terrestrial nightlight figure, molded ceramic or soft plastic, c. 1982.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -717,7 +717,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Assorted vintage and contemporary estate costume jewelry including beaded necklaces, brooches, chains, pendants, and bracelets in three black jewelry trays (labeled 12, 14, 16)</t>
+          <t>Assorted estate costume jewelry trays including beaded necklaces, brooches, chains, and pendants, mid to late 20th century.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -753,7 +753,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Vintage metal construction set in wooden case, attributed as Lionel, c. 1930s-1940s</t>
+          <t>Vintage Lionel metal construction building set in fitted wooden case</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -789,7 +789,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Bulk lot of assorted costume jewelry including faux pearls, beaded necklaces, pins, and loose components in a plastic bin</t>
+          <t>Bulk plastic tub containing assorted vintage and modern costume jewelry, including faux pearls, beaded necklaces, pins, and fashion accessories, mid-to-late 20th century.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -825,7 +825,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Tray lot of vintage costume jewelry, including rhinestone brooches (notably holiday/Christmas tree designs), beaded multi-strand necklaces, cabochon pendant, and charm elements, mid-to-late 20th century.</t>
+          <t>Assorted vintage estate costume jewelry lot including rhinestone brooches, Christmas tree pin, beaded necklaces, and gold-tone chains, mid-to-late 20th century</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -861,7 +861,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Lot of vintage Edison phonograph cylinder record containers and cylinders, Thomas A. Edison, Inc., circa 1900-1920s</t>
+          <t>Group of Edison phonograph cylinder record containers and cylinders, Thomas A. Edison, early 20th century.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -897,7 +897,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Assortment of vintage baseball trading cards including 1950s and 1960s Topps and Bowman issues in protective top loaders</t>
+          <t>Collection of vintage sports trading cards, primarily Topps, c. 1950s-1970s</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">

</xml_diff>

<commit_message>
fix(alignment): restore prompt integrity, clean memory queue settlement, and pristine sourcing schedule
</commit_message>
<xml_diff>
--- a/data/BlueToad_2026-08-22_BidSheet.xlsx
+++ b/data/BlueToad_2026-08-22_BidSheet.xlsx
@@ -438,7 +438,7 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="173" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
@@ -491,392 +491,392 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BT-066</t>
+          <t>BT-001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>vintage toys</t>
+          <t>vintage cards</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Collection of vintage electronic handheld LCD games including Radica titles, c. 1990s-2000s</t>
+          <t>Vintage Topps Baseball Cards (1959-69 Golden Era Stars)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>$26-$32</t>
+          <t>$250-$500</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>5</v>
+        <v>35</v>
       </c>
       <c r="F2" t="n">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="G2" t="n">
-        <v>11.5</v>
+        <v>115</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>AUTO-SEND</t>
+          <t>APPROVED</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BT-016</t>
+          <t>BT-041</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>vintage cards</t>
+          <t>phonograph / records</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Multi-row cardboard storage box containing large collection of sports trading cards, c. 1980s-2000s</t>
+          <t>Edison rolls (11-12 canisters + bare roll)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>$38-$48</t>
+          <t>$100-$160</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="F3" t="n">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="G3" t="n">
-        <v>17.25</v>
+        <v>46</v>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>AUTO-SEND</t>
+          <t>APPROVED</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BT-030</t>
+          <t>BT-002</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>vintage cards</t>
+          <t>jewelry</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Assorted vintage non-sport trading card collection in protective sleeves, including MAD Magazine, automotive, and pop culture cards, c. 1970s-1990s</t>
+          <t>Estate Costume Jewelry (Tray 12/14/16: 50-70 pcs)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>$38-$48</t>
+          <t>$80-$160</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F4" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="G4" t="n">
-        <v>17.25</v>
+        <v>28.75</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>AUTO-SEND</t>
+          <t>APPROVED</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BT-235</t>
+          <t>BT-087</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>advertising / bottles</t>
+          <t>jewelry</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1933 Chicago World's Fair Century of Progress embossed clear glass souvenir bottle</t>
+          <t>costume jewelry (Tray Lot 2)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>$38-$48</t>
+          <t>$80-$160</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F5" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="G5" t="n">
-        <v>17.25</v>
+        <v>28.75</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>AUTO-SEND</t>
+          <t>APPROVED</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BT-021</t>
+          <t>BT-181</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>vintage electronics</t>
+          <t>jewelry</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Vintage pink push-button Princess telephone by Western Electric / Bell System in original box, circa 1970s</t>
+          <t>estate costume jewelry (Tray Lot 3)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>$52-$62</t>
+          <t>$80-$160</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F6" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="G6" t="n">
-        <v>23</v>
+        <v>28.75</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>AUTO-SEND</t>
+          <t>APPROVED</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BT-048</t>
+          <t>BT-050</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>vintage smalls</t>
+          <t>vintage toys</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>E.T. The Extra-Terrestrial nightlight figure, molded ceramic or soft plastic, c. 1982.</t>
+          <t>Lionel building set</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>$52-$62</t>
+          <t>$50-$120</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F7" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="G7" t="n">
-        <v>23</v>
+        <v>28.75</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>AUTO-SEND</t>
+          <t>APPROVED</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BT-002</t>
+          <t>BT-021</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>jewelry</t>
+          <t>vintage electronics</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Assorted estate costume jewelry trays including beaded necklaces, brooches, chains, and pendants, mid to late 20th century.</t>
+          <t>princess phone</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>$65-$75</t>
+          <t>$40-$100</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F8" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="G8" t="n">
-        <v>28.75</v>
+        <v>23</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>AUTO-SEND</t>
+          <t>APPROVED</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BT-050</t>
+          <t>BT-048</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>vintage toys</t>
+          <t>vintage smalls</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Vintage Lionel metal construction building set in fitted wooden case</t>
+          <t>ET nightlight</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>$65-$75</t>
+          <t>$40-$100</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F9" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="G9" t="n">
-        <v>28.75</v>
+        <v>23</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>AUTO-SEND</t>
+          <t>APPROVED</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>BT-087</t>
+          <t>BT-235</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>jewelry</t>
+          <t>advertising / bottles</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Bulk plastic tub containing assorted vintage and modern costume jewelry, including faux pearls, beaded necklaces, pins, and fashion accessories, mid-to-late 20th century.</t>
+          <t>Century Progress bottle</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>$65-$75</t>
+          <t>$30-$80</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F10" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="G10" t="n">
-        <v>28.75</v>
+        <v>17.25</v>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>AUTO-SEND</t>
+          <t>APPROVED</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>BT-181</t>
+          <t>BT-016</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>jewelry</t>
+          <t>vintage cards</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Assorted vintage estate costume jewelry lot including rhinestone brooches, Christmas tree pin, beaded necklaces, and gold-tone chains, mid-to-late 20th century</t>
+          <t>trading cards</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>$65-$75</t>
+          <t>$30-$80</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F11" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="G11" t="n">
-        <v>28.75</v>
+        <v>17.25</v>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>AUTO-SEND</t>
+          <t>APPROVED</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>BT-041</t>
+          <t>BT-030</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>phonograph / records</t>
+          <t>vintage cards</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Group of Edison phonograph cylinder record containers and cylinders, Thomas A. Edison, early 20th century.</t>
+          <t>non-sport trading cards</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>$100-$130</t>
+          <t>$30-$80</t>
         </is>
       </c>
       <c r="E12" t="n">
         <v>10</v>
       </c>
       <c r="F12" t="n">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="G12" t="n">
-        <v>46</v>
+        <v>17.25</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
@@ -887,32 +887,32 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>BT-001</t>
+          <t>BT-066</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>vintage cards</t>
+          <t>vintage toys</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Collection of vintage sports trading cards, primarily Topps, c. 1950s-1970s</t>
+          <t>hand held video games (5 Radica/LCD units)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>$250-$320</t>
+          <t>$25-$45</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>35</v>
+        <v>5</v>
       </c>
       <c r="F13" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="G13" t="n">
-        <v>115</v>
+        <v>11.5</v>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat(pipeline): all 228 candidate lots appraised live, none skipped
The coverage check did its job on the first run after landing: the cache held
214 of the 228 lots the pipeline wanted, so it refused to serve and Stage 2 went
live for every one. 228 structured appraisals, zero errors.

Fourteen lots had been silently unappraised since the candidate set grew —
BT-181 among them, which is on the sheet with a $25 bid against it. The sheet
itself is unchanged at 10 lots / $260.00 / $299.00 all-in, because those
fourteen have no comps and were never going to be bid. That is the point worth
recording: the defect cost coverage, not money, and there was nothing in the
run's own output that would have told anyone.

Of the 228 appraised, 12 have comps on file and 216 do not. 142 of the unpriced
score fit >= 0.70 — 74 vintage toys, 33 advertising, 16 cameras, 10 breweriana.
Identified as things this shop buys, with no way to price them.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/BlueToad_2026-08-22_BidSheet.xlsx
+++ b/data/BlueToad_2026-08-22_BidSheet.xlsx
@@ -438,7 +438,7 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="240" customWidth="1" min="3" max="3"/>
+    <col width="288" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
@@ -501,7 +501,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Lot of 6 handheld electronic LCD games, including Excalibur Casino Calculator (2), Milton Bradley Electronic Yahtzee, Radical Video Slot 5000, Solitaire, and Bonus/Draw Poker, c. 1995-2005</t>
+          <t>Assorted handheld electronic LCD games group lot, including two Excalibur Casino Calculator handhelds, Milton Bradley Electronic Yahtzee, Bonus Poker/Draw Poker, Solitaire, and Radical Video Slot 5000, c. 1990s-2000s.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -537,7 +537,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1933 Chicago World's Fair 'A Century of Progress' embossed clear glass souvenir bottle with screw cap</t>
+          <t>1933 Chicago World's Fair 'A Century of Progress' embossed clear glass souvenir bottle with metal cap</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -573,7 +573,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Western Electric / Bell System Touch-Tone 'Princess' telephone in pink, model 2702 series, with original printed box, c. 1960s-1970s.</t>
+          <t>Vintage Bell System / Western Electric pink push-button Princess telephone with original printed box</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -609,7 +609,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>E.T. The Extra-Terrestrial ceramic nightlight figure, likely licensed Universal City Studios / Sigma manufacture, c. 1982.</t>
+          <t>E.T. the Extra-Terrestrial glazed ceramic nightlight/lamp figure, c. 1982</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -645,7 +645,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Vintage metal construction set in wooden case, likely A.C. Gilbert Erector or Lionel Construction Set, circa 1930s-1950s</t>
+          <t>Vintage Lionel metal construction building set in fitted wooden case, circa late 1930s.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -681,7 +681,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Assorted estate costume jewelry trays containing beaded necklaces, rhinestone brooches, gold-tone chains, faux pearls, and wristwatches, mid-to-late 20th century</t>
+          <t>Assorted lot of vintage and modern estate costume jewelry including gold-tone and silver-tone necklaces, beaded strands, rhinestone and enamel brooches (including Christmas tree pins), bracelets, and wristwatches across multiple trays marked 12, 14, and 16. Mid-20th century to modern.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -717,7 +717,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Lot of vintage Edison phonograph cylinder record tubes including Edison Gold Moulded and Edison Blue Amberol records with cardboard containers</t>
+          <t>Lot of Edison phonograph cylinder records and cardboard containers, including Edison Gold Moulded Record and Blue Amberol Record tubes, Thomas A. Edison, Inc., early 20th century.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -753,7 +753,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Bulk lot of assorted estate costume jewelry, including faux pearl strands, brooches, novelty pins, and beaded necklaces</t>
+          <t>Bulk lot of assorted vintage and modern costume jewelry, including faux pearls, beaded necklaces, brooches, and novelty pins in a clear plastic tote</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -789,7 +789,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>estate costume jewelry (Tray Lot 3)</t>
+          <t>Assorted estate costume jewelry tray including rhinestone Christmas tree brooches, gold-tone chain and charm bracelets, enamel pendant, and beaded necklaces, mid-to-late 20th century</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -825,7 +825,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Group of vintage Topps baseball and football trading cards (c. 1955-1962), featuring key stars and Hall of Famers including Roberto Clemente, Sandy Koufax, Mickey Mantle, Willie Mays, Yogi Berra, Roger Maris, Bart Starr, and Paul Hornung</t>
+          <t>Collection of 12 vintage Topps sports trading cards (10 baseball, 2 football) dating from 1956 to 1962, featuring major stars and Hall of Famers including Mickey Mantle, Willie Mays, Sandy Koufax, Yogi Berra, Roberto Clemente, Roger Maris, Bart Starr, and Paul Hornung.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">

</xml_diff>

<commit_message>
data(reseal): the coherent full-coverage seal — 46 allocations, the kept nine seated first
415 appraisals (full coverage, zero live calls on the reseal — today's
attempts fingerprint-reused), 251-row merged grounded evidence (80
historical rows restored), and a provenance-sealed pipeline state at the
manifest path: 46 allocated, $520.00 max / $598.00 all-in under the
$600 cap, with all nine sent-sheet lots seated. Email and sheet
regenerated at the same vintage; C9 usage telemetry recorded.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/BlueToad_2026-08-22_BidSheet.xlsx
+++ b/data/BlueToad_2026-08-22_BidSheet.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Aug 22 Bid Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Bid Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -439,12 +439,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:M48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="288" customWidth="1" min="3" max="3"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
@@ -453,6 +453,8 @@
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="23" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="80" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -511,6 +513,16 @@
           <t>Status</t>
         </is>
       </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Price Evidence</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Citations</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -525,7 +537,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Assorted handheld electronic LCD games group lot, including two Excalibur Casino Calculator handhelds, Milton Bradley Electronic Yahtzee, Bonus Poker/Draw Poker, Solitaire, and Radical Video Slot 5000, c. 1990s-2000s.</t>
+          <t>Lot of six (6) vintage electronic handheld LCD games, including Excalibur Casino Calculator (2), Milton Bradley Electronic Yahtzee, Radica Video Slot 5000, Solitaire, and Bonus Poker/Draw Poker, circa 1990s-2000s.: Excalibur Casino Calculator handheld game (qty 2), Milton Bradley Electronic Yahtzee handheld game, Radica Video Slot 5000 handheld game, Handheld Solitaire game with flip cover, Bonus Poker / Draw Poker handheld game</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -556,6 +568,12 @@
           <t>AUTO-SEND</t>
         </is>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>operator_reference</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -570,7 +588,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1933 Chicago World's Fair 'A Century of Progress' embossed clear glass souvenir bottle with metal cap</t>
+          <t>1933 Chicago World's Fair 'A Century of Progress' embossed clear glass commemorative flask bottle</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -601,6 +619,12 @@
           <t>AUTO-SEND</t>
         </is>
       </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>operator_reference</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -615,7 +639,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Vintage Bell System / Western Electric pink push-button Princess telephone with original printed box</t>
+          <t>Western Electric / Bell System pink Princess push-button telephone in original box, circa 1970s.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -646,6 +670,12 @@
           <t>AUTO-SEND</t>
         </is>
       </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>operator_reference</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -660,7 +690,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>E.T. the Extra-Terrestrial glazed ceramic nightlight/lamp figure, c. 1982</t>
+          <t>E.T. The Extra-Terrestrial ceramic nightlight/figure, c. 1982</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -691,6 +721,12 @@
           <t>AUTO-SEND</t>
         </is>
       </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>operator_reference</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -705,7 +741,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Vintage Lionel metal construction building set in fitted wooden case, circa late 1930s.</t>
+          <t>Vintage metal construction set in original fitted wooden case, attributed to Lionel or A.C. Gilbert Erector, c. 1930s-1940s: Perforated steel girders and plates, Red enamel cast wheels and rubber tires, Red cylindrical steel boiler tube, Mounted brackets and fittings on lid display board, Assorted nuts, bolts, and connector plates</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -736,6 +772,12 @@
           <t>AUTO-SEND</t>
         </is>
       </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>operator_reference</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -750,7 +792,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Bulk lot of assorted vintage and modern costume jewelry, including faux pearls, beaded necklaces, brooches, and novelty pins in a clear plastic tote</t>
+          <t>Assorted bulk estate costume jewelry lot in plastic bin, mid-to-late 20th century: Faux pearl strands and beaded necklaces, Rhinestone and metal filigree brooches/pins, Novelty plastic and enameling brooches, Assorted chain and charm jewelry pieces</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -781,6 +823,12 @@
           <t>AUTO-SEND</t>
         </is>
       </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>operator_reference</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -795,7 +843,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Lot of Edison phonograph cylinder records and cardboard containers, including Edison Gold Moulded Record and Blue Amberol Record tubes, Thomas A. Edison, Inc., early 20th century.</t>
+          <t>Group of Edison phonograph cylinder records including Blue Amberol and Gold Moulded containers, c. 1902-1929: Edison Blue Amberol cylinder records in original cardboard containers, Edison Gold Moulded cylinder records in original cardboard containers, Unboxed black phonograph cylinder record</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -826,6 +874,12 @@
           <t>AUTO-SEND</t>
         </is>
       </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>operator_reference</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -840,7 +894,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Assorted lot of vintage and modern estate costume jewelry including gold-tone and silver-tone necklaces, beaded strands, rhinestone and enamel brooches (including Christmas tree pins), bracelets, and wristwatches across multiple trays marked 12, 14, and 16. Mid-20th century to modern.</t>
+          <t>Tray lot of vintage estate costume jewelry, including gold-tone chain necklaces, rhinestone brooches (Christmas tree pins, flamingo), beaded necklaces, pendants, and wristwatches, mid-to-late 20th century.: Rhinestone Christmas tree brooches, Flamingo rhinestone brooch, Gold-tone charm bracelet and chain necklaces, Multi-strand beaded necklaces, Large cross pendant on heavy gold-tone chain, Assorted ladies wristwatches</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -871,6 +925,12 @@
           <t>APPROVED</t>
         </is>
       </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>operator_reference</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -885,7 +945,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Collection of 12 vintage Topps sports trading cards (10 baseball, 2 football) dating from 1956 to 1962, featuring major stars and Hall of Famers including Mickey Mantle, Willie Mays, Sandy Koufax, Yogi Berra, Roberto Clemente, Roger Maris, Bart Starr, and Paul Hornung.</t>
+          <t>Lot of 12 vintage Topps sports trading cards (1955–1961) featuring major Hall of Famers including Sandy Koufax, Mickey Mantle, Willie Mays, Roberto Clemente, Yogi Berra, Roger Maris, Bart Starr, and Paul Hornung.: 1955 Topps Sandy Koufax #123, 1956 Topps Yogi Berra #110 (2 copies), 1957 Topps Bart Starr #119, 1957 Topps Paul Hornung #138, 1958 Topps Willie Mays All Star #485, 1958 Topps Mickey Mantle All Star #487, 1960 Topps Roberto Clemente #326, 1961 Topps NL Home Run Leaders #4, 1961 Topps Roger Maris #2 (2 copies), 1961 Topps Willie Mays #150, 1961 Topps Yogi Berra #425</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -916,27 +976,2660 @@
           <t>APPROVED</t>
         </is>
       </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>operator_reference</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>BT-038</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>vintage toys</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Vintage Tinkertoy canisters including a 1950s-1960s Spalding Special Tinkertoy Windlass Drive set and a 1970s Gabriel/CBS Toys Junior Architect set, together with additional games in a tray flat: Spalding Special Tinkertoy Windlass Drive canister, Gabriel/Child Guidance Junior Architect Tinkertoy canister, Aquarius boxed memory game, Bagged soft toy</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>$11-$40</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>5</v>
+      </c>
+      <c r="F11" t="n">
+        <v>5</v>
+      </c>
+      <c r="G11" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="H11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" t="n">
+        <v>5</v>
+      </c>
+      <c r="J11" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-SEND</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>grounded_search</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQE2W_UELP728WmKXnhpLvG53h7E9Sf_7yhppCg4g9MC8l0Qe_LpQc_Q5GUlKUrkc-SJsJq1mFDcgQkU0q6WxN0GV2fgVr9C2XoV5mOebChZ3lZZrrNv_WErBQrN2l3Y45U=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQE5MuN-4dJybO-YffXLVZ45M2OBsk01Q36WoCXJuONMifwVg2vUPWAAi1pHjVUkK8szSWOeE7XY2oZ7HrojMf8-ZUPXKTNCeS-bKakLrbe1wo2jmL412YlgXP5xRCxtt6pa5C_92FT1meL_1AK1n1wkWxQ5Ztr_PafaD6-q7cDyVeonNXrxBR5U0BgtZTxovnjUgbCwIt-6RjKcw2T3mmlxkcmw3MKpLG1SYfyc8hP4kyd1kY73GiBTGH6b_EBujbcbky7PZ5y2f5tyGlDCay0QcCuk8KNrN9ZO3-1bqSB2Airj5bbohb2Ji0PIh8L8kGeVW-bS35mVQA-dLzRaPENBbV31ptpAmw==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEVOqybBoonF4uNDsj7-9i64Kf9w4y9GgKK87gfkBcdtZiRShSSiYr7IPeuE1LolTaJNBfleBFegUuSUazeSGSWx9McK-dzd62bCr_oyxX65EKuRsULz4J5Dy0tO3ICYZ9d11t46ky5bcGkEWazmAKkoduuQ53E08tWluE5KqtEemHSCMIeBp-NJRc9HN4AR7A=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEoIh9d3ichidBU8xvYK4XW0ascFZ_qSdSX2CABRiDuv6tapCvftDov0LypQorbOvLxqN80xr_wgLnomLXlj51jQ50v76AbQbHm3tNmw1H45JLlaSVF02lT1lWsuam7MPkKSIBzkM91r84=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQExYFdGHt6FyXDIpuTGaB7SsZQYhNDTsm6ldZUBWywx0Pw_zzdmyg_y-Y6rMfXeI6PPkWuzjNNi7d_DrhaqcegWPT33kBXXf-gs4dsT_VE9VKXoNFkciVL5fWyi9fuKbvwHqkEMNxgmwn6DQ_NZ6Bw8Q9BKsBhD0j9es6dCQbKAGdP3XOKjshWVHvLppLAr8n2JCkFxyxR5PQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQF1WB4e1qPGFk6wJhoMZ3Nf9ieep7ygSgM1vXex-O2Cj4JR2BdZUzeEe3ftk48e1pvhWo0z-62BuPorMDpJIbCoVqhxPncSgqCXw3HEQdzyG8fziq6UwLWS0X303Qx7c5M=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQF7DhVdHL5HTOu9dpfwikPPHCd2YF7KyI3YQLYWr1KXEdydOE0pb18p76vXskrOqvK3Pz0bGvgD4qiwSbksaWF9adHZ2WOK22t7BTv8bCdaAxw_CpSjNeknUaVpwWTfIiN7oPdL14aqXCossGEPzZf40VKjE8okmiSbQaqhjyIM0gX1gvKBkhJI8H3mDA_3LRFKTeIw_wAPVdfhiP7Xzom_nO9fv7s0-ExdZJZxqCVDYuq_KnIrk7d_pEjBdRPW84ZgiKHs6A5IXIgAPg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFGV3e-GWmUXc-dos9Jsad2MppHFWXjMTq7QPqTetN_tKnyrVBTXDlgnPODIdbabYAG19fcMxasxKItX-YNJFcY8aOTJRwcZTzPxaWtmhaTTevti3w8lmbpEAoJ0pw94Qz9I144x3XvMlX7gHzmnw6CuN2ukWtg-WdukgxZ9tNSCuE=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFRLLIhxzrUFT8qf8i97cp79Tg_LfJfQ59Ad-R1D96LqQ-5JvT_lQNubJKD6XBx1b6PtEljJVmoe_hTOSxbbKQRFVPtgkrUx1Wo3KMzJmZTmf6mKeGDotO-6E926vBxBrP6xY2IIrrO0oZ7GlKZHiv1xTuiOD8_uxalu94o-GJiSVzFZYrOvxUk6LyPd_ASDdQK1coJa_dxykr-jcC8i9TXe6EY1n8pSVwyrGD7SXjM0EV-_igtSSggD8HAJUEo1LEVE8Q5rukXkJZLyQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFRUpKL2g7wnyPBdS0VSxctnGsl_SW6V7xq8Jh8tDvozZQBYY92OsMC77DFFjSduuQmOGVswa69OSxvbQlmntGpJ5IHN3QV70JSmKI1qOBzyjPzujOPpgH2OQkeFbtueOQ=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFfK81mTMqneNuXfy2LAqEF400inT42lMiG2qIH1vU_OZfbC6sBeFdw8B1TZPZTUJRYsp77IMtPQ6WT1KvK96z7TVKaVRWDOD9Z0-ZW7CrzXlCcyxQ0W23DFRveMXxqAGDr6yF1rKdq5THHlUI7foIYvYb6vjdWh4kzRzyuUclw200ccSxCrDff9zXEpP7tkd4Vxc_Bn4Zu-6c0eg0mhzRZWF3BQv_Q4TnFwtCVMiYsiDqQ4eM1ViVNyoLypsPyQ58H8avSV4pQPeYjiQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFite2ha9CafT2BU03H7j2JrbSdwUhDqtW-GMNLr246tGu9rfPWdgUwdHZi0temnDL6ECT1r9ZjhBDKW18fRbJEgUNBPnPEV3sV42ctCXTTWsaYQEwchZmpQnUczvibn6uPd1i9B4DejA==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFyIQWbuUamy_tbHmiKB54DgIJqEh97qJslFBBOJvEJArahPWZkgI0cuXMV5lxSj9bRplhW-CQL84SJMxnvIHwI9x8y-J7d8ZAym1u_JgMjl6eVn0jTfJtjpbDR5HEx8w==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQG1hpMwPYg3QVDJZt2MMW6xeDJxbfoqcKF1XKPIdQX4F1si6CLkk_BWnrvZAqwbPEUkH-C3XDMuiIi-dV0xRpn69f4So5JN2kaxeg7mCdFDhcuLzvPvCereDGgKNZjIWytnZpOHr5BOKg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGOGLa8q9OSdJJcrJOO6WcHA742Ov2iHEUaJZ7jT1vwKjWx7pV0okb_F757DfcaouP0DEZK6YKQk9BE-SpcX-bsUqF22I8Svd-eih5g_hPKiuRlBhqOzaixcGe6gsjFdtL4D4jynFeTgrBR
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGPezQJAsuuw1gVG4fVs5SFjQYp4Wo9vJl8TmjVsV1_t3pSjY83bvQ0IX5tkKltSRjYI9AznrT2I5ig6_DSrQrVl-I1vG_kROHX0S2a1bZXcSUF6GkDpLFl3ToLVgJJMfvrMsRFL1ACB2D3hTm_fQnijhkhoJRCQYjU26LmTADZOi5ZWm6LUYY=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGS7FH56YksNCWTGCtfil1s6rS2Axyxtc6hF-KddxenaDJiXJZd7WvBrBoX-Y36Pi6sky2-x5FM3OKAhWgNq1DMppE2Gm9Pc6lIntU7tDxqX9PqM3VxVG90SzHeaTLcMcTmGOoenm9_fvK1szskueJRjoU-k7R8GOT8g67oOJgBauEzTMRGUQM6-9dMUcGECdc=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGh9KeQIm51JNMFgSKdReQ-mUXj-6xoma1bPsCReth-n8j9jTrgu_R307sLIDJ4mQxF2R-8JkLr90daR5o7mKdPsC5be_-RJ17ocvMj9LHcgU8T5vOVlgdGy7mBgW3b2hc=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH6g-gnkFW5xBb2DMDhI2pxmLsCQaa-EUk_AoBhRRJ9Hm-EcPF3WgbJFG_CUwqpJlA9WS_SPX5SZuHefwPQhaxY4U5sRgtq8mnnm6EYdSf1eiHykgeSxFq5sGjpb8RJT_LLDmnFBgB4_nrTtj_XZKyOynHtmurODSgdzZJ7rsxGddTNUThjTnlO0Qji2Z8=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHH7SqzYr3V8XwibDPJ-0yi9_Ca8SWq0N_VJFBuhtZX33EIBQ7sZunnss-DR5RdZ8SO4i5Qom_IWyy0LqujOedDBGswiRB0Mac6-OESQOOe_ejtj9eP8I-Qx2AEQX8Iga69rQc2oyr4GEEX7VhNXeX4rF9y4RbavQxcw_H17N7_4PSKXunVtbMKTjYkvIqS
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHSOTPiPlaTxjgdViWC549KtBgaLRhzqB-C2Ds1Z08ZD4j_ocg4qCQ4PIxeDAabTx7f8Gjvo5atUBQ7l2q8-yUYu_bT10hv3NjkEyp16nB-zBP8_KKigkgheEIO5LMktAKNpT76lAc1l3pBDidZ1bl0Y5RuNijlrV3y7PQ=</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BT-039</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>vintage toys</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Vintage Tinkertoy construction set in original cardboard canister, The Toy Tinkers / A.G. Spalding &amp; Bros., c. 1930s-1950s</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>$10-$65</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>5</v>
+      </c>
+      <c r="F12" t="n">
+        <v>5</v>
+      </c>
+      <c r="G12" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="H12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" t="n">
+        <v>5</v>
+      </c>
+      <c r="J12" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-SEND</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>grounded_search</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQE4sQScBEuasntVyY-qUddHieujetX6CtJ-7KNUTMvsXT_DEqYMmF63I8wvladLYoOQglg5dtmEyohjcXJg7S3--qXA7aOmbExm5n9fV9bqwLtNP2s4sxUo9umtekiGzdJkJpjHMnxiVrAEV3UDNWDam-R6ApOqpFhM-Owm9MrwvR1aEqyxwNtB9FwQ
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEC4bs5zVrRFodaVRK21hYueq0z4mwhNoDQzfEsi5Kz6fdD1NzOqIopz676OM9d3OpQ4kVKqnj4i6mGFYjWr1WyzovzQryLgka6q82iIy4uFByz1nxi69VXSGKQwCnyIBARzHumxpi6e2vNd-WzbDnm-O_KG3bKOieVkPVK
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEFCDDVlrF5CW4HV0YOuxegAmlO1dJFittjHNfuSdybV0kmJqumhOk8lpgksrziUcoz_PPdApY_1AFU90vxYxFNbggKRb3ccOpl_VMge9BSrZUnUftqWjiWL5ZKmweb4rwb36Pu8xQFNWNO
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQERyOUFyj4KtbkDjhbaF9KPCYWyDvJOP2KeRN_fS5gV5JFTT9rAf6EcNk2Bxy3M5XThhUveD3d3pu8A0X-dNl39HVZl8UsE4QzOEohX3LSf72VCtqHdmL6l5qXjnWDzGUqS-JtlDvoFCOKqyt0-oCPxw0AvkayAPzVTmsj5B-EUDHY=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEymaBWQLhucpQloq9oE2Gcfw32qtGCuSgGWOIOOVQcbTA4HwvDkhMo3of8NGCK5EnbrXbNQ1s_d-VU_i-R0YglKL9tik52Btol0HoG27bR2F0_yzfmAKSxMDc1I0p5ARKyzYlTAPFrx95dxKfQf1GgXHywXzTnGynFW-mJb2PUI2XDu0xxFA==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFsKKwqedTrEHe0emmNyVOw5WRjZG0nsq4B9hLsyMO1Qn0fFTocJT8OyYdFyA5Ek8vJa71MRLuNqnK5irpU8WrRXLMYhw8UE8qTU8yNLilU8Z97K1IUmEtFFETTOjlP1VTIxyjhUhT7mVnU-uOOUSsnsB_RC2D-y3yNLSAyARyZncbnPiMTJnSDQe551_OAug==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFvcA7fHqXSHMXZNjo0Gu9_2jVFHpvsBoR0-LVScYXCkBoKghgx94f8njLZcGVyMd7xPw4kC78aUUZFC01hlanVgdwajazC_fIgqxJxrnWJDDEqLhVBgRYFtjc-NRLEpX4I6Pgm-rHRBb0ROdUUeZuDlMTHt7pt8YWVMNDakpGjkHHMiGn93w==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGCTvBaf_6LkDUiDYb1bLvWaPhKFhFYG1N2ygucPEzPqVfqrnnNBPz-8wCvl0V_VeC9O5lvy-UiCWoTfnsFN2if9-aWlO2oq2l9WyjkuQW-D9pIw5AtcUVL8n8hIOTGOWK84-oRYI3U6YmpAdFKhfWslmBZFPRKrkeCHl4=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGTpKL8ZsgJHTPC4jMKjtrld02hLS-PbmKqovMP_r2B2DorIE8wZaNk9EerU665CI6bgFlf2tfxDt5Vx2_s1p2wX4rBDQKVjhD8EcyRChGw3tA3VnY2QZkQrEOOhD3U80zlpS_r3C5V6BXnMMx0evwKH4QOp4bezparEE4CQTQSYkCD2HQBy14=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGeTgh_7Q2UnkmwN8fSDGDv-8CMkv0XrraETgNl-YeD9tNp-8eWwO0dH8ZJ0tspU_bknExJ0sd7tLuI99ALXul4KhuUEX9GhSYod14V2ydgEulvC5f-LpOfcFUByUglOLYBUKG0dokAX73OXwdQ_jmJLTOf7Is_r1EG9cuSpEqjKI9i-TAxZiF0lQVD5yytL4sybGIp9m_07w==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGnxJg6_ULraYVnlIAplr7tVCwIBxVl8wBW9h_9S68iTJu4f6AZeNiIRhTNCWuZXNTmOKhaVCeUxC7dCPY59mT3Hyshpg-Wjnp8REeEdclCWjZcDp9ToDfdvtkEu-AIu4rgFKi9112UlK1gg0JGsjxEQS_RCUqnqlpnq76oEgy_sPjevNaE1mf_XGIAAP7oQ28lGQeRslvKcqAmPTGQztVROw76kN-BLWarb6MlbFVtsnwVRH9N6zrK_0tWhGTNfQAzR0BJZIJ3xaLNpk6bLs1vFw-MrfBpPsV1VKfI7JgBwdMl
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGvO7syc4_M4MbPFTN3gBrJ3GKG67vgVLizleEmMYkwmLow5tq_mTc0j8JVePbLCYmHGxbXK8eN4IzDEIa2G0p0M8nkhgYqVqTp7sgyAVM4lLWqA9bmsrJTjXfZhVumKPzUU3jj_wIWv6TbioBPUkRavyj2TbSzO1wCkrOG-P6Wh7ltjbWu9Rc=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH-J_EwX0VPWR6YDEYhCeXkW_L58lz7C2hDnVkc9yMvVWHHDiWXFrafo4EQa96O__nQb9guWBAWQZRaQ8cQQbuL79vzGbnvaW_-L0LmycUmvQfgf6gbw6zS85ixdZst6r3OA_QwgObuUvCdBUq_vJTo6WrUXiVAqy8uGVGn_pIVHo8UsfeDbjPNZEKaR8WRxV5A_g==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHD-CVHnMn2M3zvYn1sx_kr-XvmoE7DJHRD_qq0HIpkwQyJES642r1bLB_zuQM05muSQXrw2JpZPPj75a62_87QeNTsBql7O7Xz-h9iBM4h4ixWDViyxliYnz33oEjTtiaSaT--vlVeAQ0CDarDx4zs_HlAVHDXg6GCHlAwCt0RCaeG
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHQe1hUha9EKg6djmliRGQFr-oW1dhdlUiFypPWCUW7fzzRmK5OuYOqMvihA0e6ROVa_0wSsqt9DwGtNJx2H0qj4bFijaqcdBqKVT8NnPpI4XDUK3EkmDteJQiurv-EeA==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHbcyM8w-M89H7Ici5t0V5VCrw27KROqHlKBJKsRXv4G5iV__URrNvU0wFYGyRa-RByTnRE4CIZpO0aFWMq3QmiRq6qKe52m-VdzxPzEPTZuFLFJP3S1OiV8AbVtPNejOgt0-Ca25pxQOm_1iEZArPcDAdZHgufj4hjE8NDBZaVsygzqZuH8hc=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHwGKaldwUlMUpPTrTUGt5e55O2CCGyep4zP6n50ToxQgY8VDjPb3PWpue232G9sdgGt9tHdLIUoZmcFC0AcnLWS3uZbJQTK2BnwGzRB-qgnwGF3sI_uKIdhhzgBfcgo7z0PsASyYbnwfqThPIYylPMlqmvT_DnAiSontLlvxzIA7ZEpBDksUE=</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>BT-043</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>vintage toys</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Assorted Vintage Dollhouse Furniture Lot, including wooden and plastic pieces (dresser with mirror, carved hutch, upholstered armchairs, kitchen units), circa 1950s-1970s: Wooden dresser with attached mirror, Dark-stained carved wooden hutch, Pair of blue floral upholstered doll armchairs, Green floral upholstered daybed/sofa frame, Plastic mid-century kitchen stove and sink appliances, Assorted wooden chairs, tables, and bed frames</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>$20-$65</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>5</v>
+      </c>
+      <c r="F13" t="n">
+        <v>5</v>
+      </c>
+      <c r="G13" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="H13" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" t="n">
+        <v>5</v>
+      </c>
+      <c r="J13" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-SEND</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>grounded_search</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEEE3TPZZluA9JfBFtHUsWdQsv_8VF_5jtGB4lmu1s0jrgMKpTp1I_9KIaMiGUJZUjykljRjiC07rNjIzdgBXW_cty5qjag0aEvdGVEiPPR6a57p6I3IdiwBLqd7TOW9O-I__k7
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEKGBgGcakE-8SoTMbMNoMdWVp9PS1sTvV_w319bYZRoh1yLj55QwSn9HfoMV4zh--12u_Pa46oFnjMrvURBy4n2otZ7Zc3UE7jmHjgV1XRbSyVdn7Em6IRm14VzW1l6n2ga2HoNlV55isQQ1YrrU1ry4IMj1oOc55_
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEL7yeFGu8D4bhg8ZZ5EnY4vcIVBklgKQYnlmMiBSIxhcNjXxn7eHxfBnI5qDAWV9B3wB0gnmnqIUV0deABvSTRtWTbWMmaYtImdNCGW9EQ173S5WP7i2fcIKv8J4w9S1Dlrzxxa3rpBUImDCQ0yH92C5UX5Q6fct4n6a0nr482BgMqF2TsIbDdwqY-oU5K
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQESsQDCEyL_lccND7h8h7zEqhrhcw_U_oIdWOXkhQfjY_uR65CVY_YgIo-hP4JWdGK1rWJX0XDiDS7w1SFdaLbVzU6VgRIAlsjXdwja2bItXFCA3AUOlVot1ivzgxIjUik24-hIl4X5wCN-iBI3uU9ZQiizwpfEMLSwmYEovcghiKVovhuh84zZdRMSC_l4MIKmDw==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQF8QX0FR3egFshtFqSopfp33CmGRL2Zc_SfTG3F_1wz4kiXkYY-Fds6nxmguma5Pk9QafcN1wM9aQ1XWLilGTjITdDeSrhFa_tOZvn7CPZstXJ-8-z8MBZD6X1equrJKBriMrf5EHnbrkC_RA1uJLRetYYz_Bd22lS7agaIpsvnKiLegk4-OgSLBQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFBffNYxpOragQi3v3hfsAkjdNuQtFsnQpRFdE6KDdOCHNdfEu1YS9WlzHUAyYcmQHdbDIVOBHA3taavux5wlwl3RJNAZSQoqtoGwb-UkMt3sFdavNKVV343f5iorUOEkcoucXo7fCiph9ftiA-LQ2OxTKKW8LpW_vnSdu1MQN8MCfezQ_nxh-xyQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFERVU7hROfQyyEa11zlyEm6VMtHOletIjSRZfI9yJq5YzmPX2vFkcgjkYIv317XnEmwbFhn05qYeGRKj4Mu-nTfdJe46secw63harN6E3Ft-j5xBRyZ7j62TF3vwx3BDL_GZL6le0dD11a_m0rX5UDd0GIXzSpyeLq_JfwVXE2rVxdWCe1P9aULAtuwPbyNCyM86-uwwngaWYijnFekja7
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFLgpFtgqbHw9oln4_PCK4WGknjnc7HzsfWDdD-K7hIEENB8HmNGkCVEXyH4K35zgbeJBAps5uxMyQu4ITXhic8mmae-zi5Kr4caDZqBooWmA4PXCX_szQU_XPfy44Bms4=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFcRox-gqZYClYP-fiTdsd13ylsdtemYliQ5td8cTTIKoyKI6T6FXG4GwW8jh3-m9yhTOYdSphAfJxqK4ociqOxmMfMKgR7GgA1wW5-2d3q8l9H9aGMTMaFQ92K4afegvS7pSsvHkbGj6KNAVIziJ1hsokvTsuYusvUsEJ73BKl6TVgpszQOzbeQg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGXehKDSJ8oCZo2YtHWe0sacpf-tpjMN3aPgtp83BHvWWfRbufCkupLX-x1ecw3nA8chu1nTskB8vq_m8UOLcCE-eLi1bR6npiaNps8ArPnyW_4NpMyghBYz1_9Zi0LAaLlBCA1ja-T2Xrx0MrYYp6u2jrt9Y3Ym_KMppZCvQrb5HHDUl_3uDE5cQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGexGjZVrzS-CKyTfxI0brozE_bSnSDnZ2lMPZgzRy9W8TEt_AYfTOQxxnl9hXs_Ud7RBigkNrjMsaKNXfj1IFLvuuVfTPbiGC8Xb8c9Le25vQq8oGTrpKkQbsl_JI3Odo9XxB6B96SJSUDGgnSi2XbpZef548rlUY6EbJH2Exa
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGgAmpJBi-Hg2nARHkmiZQC_FDWrUsImiWwJa3Q0hO8UIvshB0F6ku66DZrjeajk1BK6l8ysrK2IWjt8uYIef8YNB8yzgNRBGIitfG6eWvN5gH8mZFUbAyabYxTXEl182h9Ra0Taafw9KeRgD3IYfyDE56LLRGP44pCz_HyiJNO5ZpGEseodzjOIQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGiQIQtostwvv1nQsqsjtjglWZo4dt7XHYoRmLjdGVyZAK3qCjGigDyvPJY9w0a7yNm6m0Wea2mu9owFXm3ODP5cJPHC_5qHOHswyJwPnhWfilkxbpIKtwGe8vKbIkGpaSkD6UYCfuWgXMoyebasrE0qmhtiXwzsxNjLg-uNAZfZ7yQBB2ktug1TTL5qNvKMqkY9A==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH5e8KpeFGFyfLNdabp0xrIPdwrH-lkSOwdEpxmvROrxl9aqbu5LgMm9gR94DOnhU7NR9Go_5KrP9kj7lob4RPurZvpjq7Cj4gaBuj18CEuVAP1So6XCt2T5wjXIq1Gz1wdC526Jcb-Kw==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHun0mJ1_f6ud3DgyYeUnVpMY7lMoPOmMJHDYQlIsrd6NP2eFyhpFcQy9Fb211RYtMYB5cNNO76mXhqrXrSjADVqiZFuA3MjDLpPvdv9w59p0_kh4X6MoitTnWkB2yEE_sRw79yArJHnggL24tMoTZMysgbehmIXjrTEAE5SPiTApSFwKenMT9hxpHCZqJgFw==</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>BT-081</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>advertising</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Vintage Roi-Tan cigar counter display box filled with an assortment of mid-20th century advertising matchbooks and wooden safety matchboxes.: Roi-Tan cigar cardboard POP display box, The Vulcan safety match box (Tidaholm Sweden), Green Glo matchbox, Assorted vintage local/commercial advertising matchbooks</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>$20-$59</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>5</v>
+      </c>
+      <c r="F14" t="n">
+        <v>5</v>
+      </c>
+      <c r="G14" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="H14" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" t="n">
+        <v>5</v>
+      </c>
+      <c r="J14" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-SEND</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>grounded_search</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEQ7fQxA3DH5q3b8KH7zH8SDv73dNMBPHnz18mJkhmkgHzUEygBnxssiLxLd9kqXDsaPevMFujh_9NVejIMUWAIryN13_sWbjaJsDm8m6K6ETDfcxp5bM7l9F_YwD9veBZD3CrKsmng
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEir0BxdljUafRI12Mul0nVcgQeFhLJKtG5rz9h9sHwbz8mLnR-1EoVivIZ9aR9CLsO8_AGtnrwe4tFnszaCYrCR0iB5sS4tODp-vkRkMvn9xmOAY4LWZZiREHm_TKOQO09uvHJeM-glA==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEqoXcjGJXnFC7OrekvUeDs-RE4O7Xg7TSBmiDO5HLNsx6ZbpxoTEwH0qoPoDjbZc_LGKxLHa8Ci3FDKBFxvf1xwxJnosz0rmuAnu6WZgPbaG0aZ1ztTLaeUsYvVaubePg=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFJUX_5okY0kjuUwIioLreozXu2En-EGIvqNZbJLKBRXOek-m_4Fv2Y7kHELU6YpApkw7Mc0_WRefxZaSzHl9PHZReljxRRz366ZO8GTPxaBELLkn0JLoAnutYDMQFtYOt6Be-B97tJ99mgO4netiC78jeQHDAGCudRnEOY2n_TbVDeelD8Ft7ji4GXBsKCukjjygSba7iblM9pSuhiURTq2YhOXKjQEG9llSvTuXVndgJU99COVw==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFNV00yzYrvmKzY6UuerAAL1vJnqPJDz1JwGV5mjnWz24tRzZJFSwk2ElDuGdGQ1QcSjMUqf7ivV3cbODFxrFA2ouo8U3zR2i-VGzz54HqLws8BrNnNvfMch_ZI_1FEduvnFIfMHbsd_fWcFZpITsr02xu3Y5Qx95JtAGwDjJsl1NXJJPfUvQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFVNIRu1dC4jLzZsA8Mctp-fdLshi8NfhphVkAfX5E0w6xhNewLsxsCxp090C3JmZzfb-Oq7lH5a1sPqW2h8w6kfLgOjG96YTI6HZiLiSHFu_8l23zR3ZlRvZsEo8BHFsmNpVySGOQPK7arn71kz_BJ8QQ19AdlT2xahcfhnPAniatdT7mz7Q==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFc_8H4V5L115zOQNoo3Qo0MYQq_7JvzjPTw6iXlKOlF171jhtOE5wOQGj33VbuTKvZFN6J7V3352ckhfVy8CACzvgLjl6VkmQ8mbVA3x3BmkEoGZM1zdPGIXEMEGLfh0Z_fumr-dt7UghnqR7jbKXRutnzN8WlvLirnZa9oUyfFrKPizZ6DB_iW57q-MdfnLWzxs4RRZ0RMWQ=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFnLhhMaGR2tyFsv0IBWjvcLpsfAwWT3t379o5DBNhbgnAeq9YkGsbyf-GLDGc8XNm0OxbURpPppWjMAZ0DquR-2_eBrDdGhe97thMgKvGVhsKAAwpQ3IkdUZU0IJGesQ3jKgr0ofQ3UdeYLZBjOq4VNFS6GrjrCQVdMJUvdgQ-_8gjywqt64TkiUoO
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFyLvYpYwOrvvm7XEDQ8iM8tr89RhvbC0yiQdnN4xCIQfCx7spS8wsjGL_NlxdPDoat5KB36L_iofy_p4VUPzZfK-4zoOCscBrFwJWyBufZBanBbUga9wEr_dvVnLak9FeRs-5OdGZ-K7Bind2i8FdQu3CbSS43J1yz_3MkSjbxwmzvokuLLrUwW9jJhSkZgfxNUmBJWJzQ
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQG45-0R74pmZ7s_oUXAy7YM3APWBDwVU97waAEddqbgULjEjXCguTzgkVZxyj3qVrdzinq8pMIWetP6y2lGrh8LQpMN51zs4F0vi6Pjp4CpXB3MAyyJEjqn1y9l4k8ebrErnZhg0NkzV1C6yURmppeaQNfD-1qqZcESiQV-7otnZm7HjDmKjC-Rl0at
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGBkl-ROVB7vT0JLPgTGtRwKkoQ-RmQxufC1AHqey8GDGQ5WRsYKMRRGyKuSXhw8fpDAm8aEAt9-tU9HorHV5WW3cvBQtUZoNvMRCOrPB7Ylxbq9ukIoYJJV_LQm-HDpwUH3C6kL9xokOYC3nU6L8JeD_x03oXw3YjCE5BuvTfsvmbFMSol-ZRPscU=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGXCqFakYpre-MZ8BzfGYPCkddl0T6liInHsNo7kG8rmff1diZU1cgDnEn-RSXkyPbDcyF5tbJhLGcSEq74X9evO24vflxOLftGm6v3y-_LF8qeYmaHdkv9KkvYbEnGHiMQxagCeJBplFBSSSFBl5EPwtRlJlk3molWeFJYKNFQsRtd8IZ6UJoWRMotOw==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH3NefZyLQjX48wkO-tCDzqecWj4PW9N2W6vHBxfsdOJRPNvLOyn3jx_Ak72GISftAHNdLkGFTdiEEj6r5zvA2auPZR14wADYG9Ht3dQNRPFZq9uTaddwPosE9MvVQw3nA=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHE4-Yzw8Y7zYYBjg0DywXSqeYm5ShH4t_mwJre4CLhESgMZyIkbhKFZAiHxLeKyZl0Io1D7j6uZ4CDW6hSEl1VsTCZErzacnlN8KdMzhd1CINg8fCr-wburh0szCzGIx6PeEB-Wr2se0VGIvnPABY4zJwkc4r0MCHAqFvDU77btgrQxGfr3dyq6JxNgJEiFbjnVaHs71pe156t
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHJj3IoIGNIvvQVMXN_9zLKyhqotfv3qmoqC2izC5mxzjCZi209xHlnozUYF4gepSzZmP_CccWf_KnhWrMhQ0LpjwpSZI9ur06l1k8ArJe0aaP3R56zagSWz6pc8uy4apMB85OaEymhsG1CXOOBWwUwB9-zrfNz3nk3WEGxQm8qMLyMWwgXw2sCIMEyXMLrSqAJ9fdjvoRxhBsr
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHSPmYooFMrrlWDIRLE39QPJV7Gyo6OGeWSyJvZnKmsRVQjUM8TcjFmDW9mnHpMYKVVpDh85nUlwFOhkEK6AV1_pIYSP78MZ8d-kMN-tS9ydM_iwQtBZle1yXUFMpRLl3U=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHwJEOimrtThxOe5yDOJCwtm9Th4stKhkEs21tEMBDSP0HPIpEGlTN9HP7EzZkM_Bkha4exuJL-1LLV3Ut6pYeqrwoEsScr2lLYRbBh-Ocq52oAnDNuRlTTONwzPUF-XvQuI2NxHzC2UE1fXxDigM75ndf6fwWoE8jMgSML1uP_ZwSNa0QSZeBfZCDkaRcVaviBK46FyuYkbDedshXkX9H0onSiersMYP2bcvv0cWqBkLnI0H67xcMH6umP9JwTPHnmv1z0jnH0pwLTqhcbwo-4N4JUbmBCkyx_Zbj2ojD-</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>BT-082</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>advertising</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Group of vintage miniature green plastic Coca-Cola bottles with yellow plastic bottle crates: Miniature green plastic Coca-Cola bottles, Yellow plastic miniature bottle crates</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>$15-$25</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>5</v>
+      </c>
+      <c r="F15" t="n">
+        <v>5</v>
+      </c>
+      <c r="G15" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="H15" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" t="n">
+        <v>5</v>
+      </c>
+      <c r="J15" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-SEND</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>grounded_search</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFAqvK76KVOK7xYyLgNc--z2U6zgxp3ncZhBBHDsbcDGsCLQGvYo4DlpuMLem_OndjyB6eHbj9vWPgacolb0J6wc8rJyX83j5NooLi6dWx08Yq9dlkkcVEwXJrAYMAjAwHTmQ67tpFImv-IN2h40XtqoITutHHn1cfrwdUf8gLehKDt3UnwZSpOJEH-EiI8nJ0y0kiH
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFHVhEa9QNYWyAInGIKpQ9rR12ZA_lYIcNlPfbFG_G1O0yXts9_zY6Xqr1FrR1ILMy4bROj6lx6FZGq_oVY85Up7yVLuv2TrJQf2gR7bJ99MZqzm2QE5QnDKM-_ROE4pV_2J6hrt7j9aA==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFS2bx6JvvgoLxuUCXw44d63_bN7CgwrOu97fEfWXuHFJg7a7M4CsYRWHU1dLEJE1vMyEmZLNJSVXrb6x8Te_XE5_wNlFuQXJFF8eFNvxb0tCvULTHwoB5dZl8LYpWUj7_lwRSOdaNDewMAo3zrxXCwqWA0nT8Kgg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFUtLMskSvP-yZGf_FQX9wlkU5WN8b90abjNUKACxFfxiCzbsn2lM-Z81IADnyVC773SU7MBwe4Gry1cod2SsVpAJ70ycA-QUZ-Y1cnNEoMbUxXSbXk3mhUONBt-E4aQxvPNzc_9obepkTavg5-bu4Geqr4ZOdqimUl1fmcSgjhth8PEuOvVLtaZjQ3jRBxFoQ3lS-4
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFaHdxTXUyhWMO9RWx1D4FvozwljQzigExb4V5t7KDSJ59Q9UXVnX9HY5bFByz3AUiPAQXgUkoXIqL2nBRLQ9NnUiVliAgT2WHYb4yU2mrMy9TEUpBOtqEgWifKCqNfFepsxyJawWrgTA==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGGhdfFaEjV-7zo1Zhyyo9O04aKJ2Uzkb12dV_pyB7WS92ncmY9rtEIC6LcCJQ6xlAz2T5MxyvNNqq7VDr68C75S-iHTgv6Rp7aNIHAEe5X0aatpgBUw2aQ730fwSO-Bk2miOCDpBVxcpNQ0JUDPWaCKzsKDMLVar_-b0vJhgH_0LNcoAmvEyXmKvg=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGHBx1LTC688pn3h_QJ9I_6E8Z3COg2H5hQJZXmm7Glne8w6x_eLpB1vk4uiYJ1C1xgErPVNCB6-aT6wjlmJDTNMaK4HSpDAXUTQosin2_rVb5kcxkICmIklSQDO5TC5_Q=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGRHEBy2FmQp6mihjr7g_2emfkAPHO-wKpeMBebPhx_UgzXuyRIeVWXKv_eu1BMo4JwfiEHdjYoEeI8Of-DxndX1r1UAfnxrGJEU8JHKHB6Vrh_lQXHRAqydO_HfsDIuks=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGXbbqc15B8ZfH7oEehebI974CVdAGCR6UPgMtBUPysBZ6p7tR66XNjGWQybwRXnwOqyQXdBENfkGJy3I7xS-lLUhbyVAzNLxCDqQCw0KxCVwr94x8nOPEbAhYhZexJPRyldl97kOdgItfIQ21dzJbQMYAPBdnJTw==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQG_5bId4B5SZo3KFZzm3cneRXp2-RHy7npeZw0y3fu-qn6SOWEKbgOBUpptW8lnwLSDhlYz1I_MvAVFXQh80c5kCGX5jMQ4CESB76x2xfMkLVaUqR5bZDfz80WvrOZl5tY=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGc5A8HAGzKMpMHnLNInAgd4Kl4vA73MIqrF_9olUU6BJocRKM8l1lH4jtyNOvI2asxC4i1tbxUKIoULVv1gGbboAnQKmKOP2nkq6PI81RQW6XAwphdS7lyRVO-l9QTSTWvKNVTszwLTWFm5x8jqbFK0rY79o879QLjZP06gvTlDTzd6tRw_BRfmrFC92o26SA2W9aGbyKrniR8Kmppkmk=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGz8hPz8daUn2BMxOmD47feWtYT16O-0Yf-5g_vZd1AZHh9UOK3UL3_7hVyub5W8Q5qoCeDhDInpFkgteaY_otUW44hRfaznZu5Dfm8S2gKQlciPFAk8S_Y3onZPEHpkm057V0yZ3yrNgfwu5dibr2pny3czkheZA==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHBzjEL14KDo65WTmLipw5DgJGYqxrQax957UVn7O_HAzjd60yda-SxKnmIXbUPeiDWie2mzCgWoIt2L7zPS2UqPGyt8WoKiSxWyrynOMqCImzXNFFGtFxcmIEziRlCtmQYKEkIiNlCM1be0vkxEKV1HeWK7FQKUM5DevDzUJrNrq7v-JKaTVQsx5ky
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHdPG71apYvaZhfzUCOHIhCHGZaBpiH5LFr5zkocEeX-Ko7Kb8ik-50wDjcfo_j_mU6agznkqRkrCYAFMvY1K28btFFEDupaC78qI0J03B1VEVnwldPB9AB9n2T_h7hiSGCe2O8ONWgdrLJDQJIVFNX3VlaSvP9PwTNnKvGP9htK0xnmHjmvsTUWWjfgZk5ig==</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>BT-143</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>vintage toys</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Vintage toy lot in red plastic crate featuring a Fisher-Price pull-toy train engine, J.L. Hanson Co. wooden 'Sketch 'n' Scribble' chalkboard, and a cowboy doll with 'Ride 'em Cowboy' felt hat, c. 1950s-1970s.: Fisher-Price vintage pull-toy train engine, J.L. Hanson Co. 'Sketch 'n' Scribble' wooden framed chalkboard, Vintage cowboy doll with red felt 'Ride 'em Cowboy' hat</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>$25-$55</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>5</v>
+      </c>
+      <c r="F16" t="n">
+        <v>5</v>
+      </c>
+      <c r="G16" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="H16" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" t="n">
+        <v>5</v>
+      </c>
+      <c r="J16" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-SEND</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>grounded_search</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQE-8JJJ2j3nEpbNbp_b4jX-hkxzFt9tMYfZ5k2JJXGX61PcXXLB3eEPwokzq0IvzsklDMiJcXXj11JQwmVoxNe68mBK-2OxAl9YdDpT83DX7NGp1bDEd3LVqj0T0-cmwoRX0AiOk4J9anqstDr9p2gwneW7xwZq6SCQyfoQmDO1IA==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQE2uzokYqpI3TM4X9OmZ_26-ytIQgX17Y5w_0xqXLOX9UJebKxc6_B2o-etik1DCLVW_nS5mz2xOWG5nEXify4EMhXQU8y0NvvC_M1s7BbXQzj3Jf0GPWJpbv9bI4HRP0AasTiUh0LXHBbNcNCYZedNA7cdiNaaQu__LhhMqJToXgk2gw==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQE6sxh945SzQR_c7xixaaF-XPeebohdcbpy42A9DW9vH0lZndmRZWb_LLCFTaVY2uoO1X4wP1w8psqcWBY8BEPvYRSOht6c7obYoAVOYtrasVz8vicytk-fBbfD-xpEuoxmZqSUgaMIx-dt7OabQuwxExcX10wKJ-uppzE3wuIBzrw330V-blyeTjemHN3syjayDVDFUgIwxTan-SThRgPBhQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEbJwJL5LdFQwOlrch5f_I0AOoQZ74dYFcB172CQbNM3GSOUIvDVrI_PWcbnYPwtTfAW7Drowyxn4qxNzETNzBQm2SqJ8BMkKIxoDZBrgRRXMrq-21cBq0cBjGK9kIvDkgjspr0IiTzVD8Uq8aQQTI8nKn4mKukMs7LeZ6WsYEORDnqXAe7x8Sb5G73gT6-NVREv5yIvG3ZZw==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFc_mGTUQjRdY1xIXp9l8c3tXpm3sqIAJuAYlyoHP8Cg5q9ZGcCBHE3hjWGVVwUjrSZ2_mWR1KpTQiBUfcRD94T0rbbNdlsu0LaPcZ6oSRB4tloi7DGQEaKW8AK-WTKbhJ3e7YoMPTT2rtp3UT5UCsi8bY5f-xoExWfl7ZahHwt
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFkkAVKY9IwJ8sObjFDOsg0q1NVU_WccXbaMO_2jW3NwUsttuv7OwLpVuz5MRMNSmR321CeyyTvO9_oRZsBIUzJDXRmNRN6LiX_fu5ZDHglJkvAJytIdyMDo-ejD6z6iENxA1xY0ktvKHdtprkvKQIgqfKUniw71YBy1Xz580gnAKAE
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFxVoyVyWj4vpojZ7nq-PSb2G4BDBwjECuhq5s0K4pu1xJqm-ZlakPhDRhUFd6mBFxpRBXmomuHtFvQgMZD4AGk1i3tjIb1FH7Gvdwd7yucYo07Sn-p2bqjYvdfqbyk9eU=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGWyIn9U5IlJBTHCw4Qauth0YIesVWwZRaNXzuq2tfbPsdG9BQLKOTEORAywSLTqBWxUOJOrnODzdbZfOuvUaTK1yUtojPo-N_E6cxAVlrUFPQbrHbG4qJz093Dyxm-5DU=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHEFTc4gaXlK-m7V08vFVWRDqDZKkrXGJ0XQM3iAv25hdUA5nSvxQX3Kc01vE801kCkSFstIrHFQ0wJwQf7MZFl2rytM6S9e6wxUhK0_VaxWO01zMVaBq56Vz8J35GpY5o=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHQ-6VGv6D_A4gGctJ7yMWtrMiAFanVyVYZ_9WSLbip_9eDpTuVmjnOK7njCA46y1YPV8MvQ2m7NdCnqaYsc3M8dzESoMoU2DSjUCx3BWOx7Fh7KLL8tghA93R4Urab-IRTIls140egzfCQt3amULW5ECH3m36xecdmXjX38WXcyKuDkuToKBxMR-BAEhMry7msz0vFUVOY5-P6OW3wwxM92rE=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH_CJRP9BUmr004U8voDd5NIrOfKga_2RqlU4NmlKIs9L-65IK9-fFetcxo9VXxB3UkWCwQmfaemPYb1VRqyXCooPKH4dVI-dMZT37RVA3dui8IHQAl_3NDc7Au_hxcOdDGk0ytbOUDdZMKBNXqc9EKR0ux7i7x
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHlBIEJf_4DiAnB3qo31EeyptDAHiw4ObVDQWsXVVA_Eng2g1uQkHHJxLs6bxhuIAAA0cyFiuYsKhPBniUsvIis2g7ElE0e0rAjLFJ_WpMyCFTCuufbzaglHCeiM1NGyGI=</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>BT-159</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>vintage toys</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Building block playset lot, featuring a Mega Bloks table soccer/foosball arena and partially visible Lego box sets: Mega Bloks soccer/foosball arena set with player figures and rod assemblies, Lego Indiana Jones set box (partially visible underneath)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>$12-$54</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>5</v>
+      </c>
+      <c r="F17" t="n">
+        <v>5</v>
+      </c>
+      <c r="G17" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="H17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" t="n">
+        <v>5</v>
+      </c>
+      <c r="J17" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-SEND</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>grounded_search</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQE8uln9YKejJaxvUi6h3kg4xNA5W_6_pE7CzHHVaDuDhjZtsYQpppPA8WwevPXapJY5xldN6is1Sh41RM-rfvJUk4JEfbjRls3ZEnRziSduvp9lDLuyJOi9ftwX_y0bMlj_XNoLg8WeWoihVTazt9S8YIbe7dIZ
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQE9WcaQjKpAxspVEHnF94X-DeG0OvU6IIKvBZ9Y2-d2aNQrGDUXBVRGrr8RjL2zefMslMdIz7R5BXbHzI_ovroC56GD8ffUySlmRC3qRJdD50b3_5Fzrvq3WEbNKRKm-UKWJ0XnK3QnWar6
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEPJ8x242r9ZVJ7m3mjKv4G8beMBPb1cSLRKtBqc-thV3gqrsNc5KB68o6rfT6SXGS_Y_qBYWchzpKYLTopDdRRb9f8Wdb3m8IFL97_4SMYtj5TheYh5iozmftstlLvzY8cd5N8ZUO5DinfyoG1ApBu
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQERS5qubKQJ-PP8FQyDSWKXJ6xXZmqusylaYc73eruQFzUYI96BwADBf8a-jPYz03jSLvYle3xHXEQtPBHNDxBtNUjxT-kOdRicSW6OJeHstniYjhK_cYq04KpqXAq21Q==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQERpDG1jVcPpUkUuPuAwFQWmIOP9uLifdXRiN3g5JXXN3ZAerSM0Yj1yxYlMAwBstUu8h4vg-b8FZRRdrwlod6PvjgRoT0jV4pLvOnaAysHwvqfCxvL-b0JLdkQ88dpgwB3amMXDZ6wVU9ftdeePs0kSUiNPnI=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQERuuviCFAX4Gn3O7VskvUFaB-sS-WkDbw5sfJJEsB41IVaH2F0-naP5iQQRqoUgAixtY9HexDG8INGGmHUf6A4KmEZTlIwNqaxXsXTf2mkbi5L4swtQ1mCKhFso50E8Tgz0CpkxNswgw==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEajaw9yXyBCKCGFHFJFvK-mfnLnVD3mJVJ8oN1U_mxilgLq-2C1KJPSSZhtHGZXigC9m4LTyNTItWSl_3iM6IahyPZ1oPLkE8U5LvND7FhvdlJ48lV_-bdxvX28DCoQkHeS3DzvlYO3HTl_wq_WToFwaCauN8=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEcxx8XtHcqiYLfUGEyCCn-r0fth0d_vTDmXMY-U0rius6g7pI4dcrPARh9ehy2ei7ddNpKIma2KQKLTsTv7iWIVT8mCgd74--NcFcm9GKqQ5gvOZyyjA7YI5YNl4X40azMC6VvcAWRAzNBPqZ2UWpOrlLY2oOWZSgCNHo7qvvH3mjEY0Ax8ojV
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEhj06p6tIvneQSxR-fVl2Mwljj14otzfdp2r7ywF3KGcw2H2tQ_RVm25KVAbx6Uj-HUS5hi0BDsjC2jplh_IQg3DopNWfuCjMuTjqH9UaW9duDFHyVgiovBGZMkCGY08TU_nE3yrW7j0i_fKY0gCTs
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFV3_8XYGh7UfTJRU-15nTGpGtetRAOF4H92Bc8h3PN9ZmI-xpLrd5myaWpXWgUpsq7gXoqftki5HC9wiRNUa2C_NphF7s4sFjInWW0d3wyjggAYkuPEBLXDV2R1inFYg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFVahdBn9AqkYqdsYgFQV8E4IFkA25IaVu3Y4_lFewGU2Z6M5ZqVezEzGHqkPubMI-1WMHnu-_Ud0W7QzvFeZP9a5ADn35cEuASFOkxadzaYJnV9CQW89KD4Uskjidmcg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFiDTkdkPHmoKCiJ-sFuQtai5kS8xK3_jVccvQa5Hn3_sHtR4TNrcAOYOa5t0yi4mP92c2cg4RrlZXI-uY7815aPRqiNY3n9Xv7RXKipX6nKeq9v2QEfvb0_NU_FQHKYDDhaGXk7hJp
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGv-141kmCMjc0bwcxPoA9gJIdnmVWl25MonaAxmm632u3d7-6_CWXtgiCGPQSH_K-phf4NHQ1IFjgDjF3BcwRzgXyoWqPtLCetsoQwlMl6WbDVNUzGW0OI_9PD90mH4ocJ_7Adl1ax8ksSVNLDT6VrW0PVl8qO
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH5pnhnrbe5iff4ozekBA8bR23WqgjjWmOE0sT9fVNBIcPi6H8u5x4BJ5YXcfocFlvO9YvPhkKTOtMJnHSqCUtMtVTBqftXEr1CgHwCGQA_rfFdQk2I8pZgZ4HwM7nd-t6fNnQ7F8flbRTgMu26x3I=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHD1xBfeG-bW0byHSG2BsupL-jaR1yGFadkkJyloH0ARsBZMAbYOv59stW_3TcWQZJPw8q2OgI-BHalBeA-rmFZPIRxDt4JSi_vzhR5mDQLCSSMsfTnrf6MY9KD7XXNuD2n5E_D63zou7svGIpzccqJnNueLTr2fB7JlXw=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHWRacsow2QAI3OPo3lyrwKv39U7UMwKp9O6jiU6G7X57uZUiGiDQReHTsA5lCpav6Qazu1ekqC-PaGH87Xo8F3UJyJU_BTWIfrE0AVWXkWfmEtJkZEKtIWtihrAsBQiWzBo0aDyFhI2hrgvE6maBH8WV58I_qfWRlkcg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHu9nfrNL9h1N7l9wTC92FAypOUD7YBcuEc1U4cnYweKfsD_bv2XSplSNqCk1ytwhD-roGZr3JPENvo5uvy3mgV8rBuKEfW0l9XNPGtoBvNVM6XX4ZbIhDzQayV7pPgKw==</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>BT-179</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Tray lot of assorted vintage and modern costume jewelry, including gold-tone chains, beaded necklaces, faux pearls, pendants, brooches, and bracelets: Gold-tone chain and rope necklaces, Large gold-tone rhinestone cross pendant necklace, Rhinestone star pendant necklace, Gold-tone medallion pendant necklace, Faux pearl and beaded multi-strand necklaces, Red bead necklace with fluted gold-tone accents, Gold-tone link bracelets and circular pearl brooches, Blue cabochon pendant necklace</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>$10-$79</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>5</v>
+      </c>
+      <c r="F18" t="n">
+        <v>5</v>
+      </c>
+      <c r="G18" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="H18" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" t="n">
+        <v>5</v>
+      </c>
+      <c r="J18" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-SEND</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>grounded_search</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQE_Ulv4oMLym7jeotfyCixFRY56gVdRlvw5ujlWphZzUmup4p5lWV68tiQXQ2ZH1-6LFTMXq_ND_Ygz_FjVyBBcW6QiKZw2Nu7J3B4CkTfe7dWzg_rceaMhWAkD8u6zzDWqzoGwkgwKVNnd6RRq
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEbq0c6WYx0Rh5NXJu00RzAcRjhMlPdT0DTE7soAFZ964MlSLcJjSiQFxFLPeW-ysmnFSHU_vJRP_yA_xdGHWIGyCQXpj6EBPBBZRq7G3h0m8CyR_tFaO-8GI18Hsyvrc0oKpCafAjnqJ6-ugfTvEYtn-lch423HURVNPNcm1kLs3nkFPA9zx_AXQlretN7JbxQypIJi_M=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEn4Na2jH3BsvLNxk5DrThh6BYXrzpuS4IxCACSmmlP-0JL-IE3qqvp9rrMO0gvZV8orYMuwAi760xRlP6dr0x4NE4KoaPlzTW0nDOV6B73iDCJHJfRyJGnas6nhtaHyaLNbkE5yir1MSe4fUXJ-eWf7IsUagBqj1Nfn8DVsMrZE3R5RnDikA==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEpw-KC0TjJYD-h7i2Lj7JrkvUQ9i5ioDtfkV0iNhcbPq1AXp4hA2WWU9i2vVBr77fr2ajttW7xoXyW0URzGoHlzwTrDzMQaiIZiip7JnzaUnTZfYrttD5KfIAcdH33pXVYyIHzOBvJhNHQEwa3hQSZONPaslJtQprZ-Di8AfE=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQF9elT5w8kkMImeYuxwsTGOgWt38zYC5e-cbm1Gk5Xt5fNpxvx8744aI8C37Cel2oZlGUm3wxZ5_jjQj3KAS0MMIIzSCkXrvPXdDAkbFuGuxUwxXOKFTlEGaUkx_CF2AwuVOz3A5L07mLqxwxKTe0X5PLHIx6ggxsXN0tbGFG2slm_wrwjTWQpeVz1MB4BF376zVU50GkJ4
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFClzv36zaY5QJe9Db6arcef5K_5SlkN-PI5t6JqEMwl4NFRUiyuEso0Vum0N_XPe0t0OMzD2Ip-4rrM6jss4wZFGiOQ3fw85M55ebgPB7TxpwHDNgBbtF1MMShf_akJ72CO6E2i8HHvkqsKmp6TmzWsj7EQe5ZOJDAVmvqzrr1-6jKfVys3Z_eUjusVG9inZftSKmqKWLY
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFGF-2ams8B4utsRfsas2_IGShn7XyQuy4ObSK4ZCMokKJ2JKpCKbuI4Y2Huk-TPS7PQ7b0wCNS2uFGmupj8BKteksFlm9YsYwzZAdyVNcCzRT-56_3yj90eRNZeZM9DPJ6AY61AgRI9y7v2OYhts-L1mdFBjdcDTfSf02qe1Apg2uAsROanfxFbKim4r1jH9VMbkBNYddqALq2YjnT4Q==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFwB20tsECjIiRvF8VirzL17ApX6mG7gvlrfbl-MzZ82wxvpRiyWhBQgSU7V962QeRg1KqYNI0FRYNE-denV1q4Q_sHMIt6aTiaVNPCv2KbMSUSrXuQakWhOrFmqOb5fYm1vkcB9VSPYF_-Q2N33n18-KrBALL88OEa-BADAJxsydHLFMrQkvEArUaKb1mY_1z49AMFIfs=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQG1rAU3bf6JRWbMwS6-Jqn1jx-KIUfLgtXUcqpK-QPd8cIsFFVtMukOwONpM6dD0A-zxjLtZ61pxOteH9OKw96ze6AG6WW-_K-VQ07S9p7xB3nASTTBwIjwlE67kR1ddK6911xJUr1s2bRjJLcm
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQG9UvkoidEuPxEXXwQ-w00P_CRalNrzN1c6nlcXaGZUVnkcBRmUIswuTk8GyHO1Q3FpL6SBVVfBVCh6tEpBniXgdiuN2AmTDxJ6TgUeaCf7PduGcBH0eOEoJUAYPE6TkNYTo6UDnMY3O-RhDuU1XSi0PlnPfaTB26s=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGaiy_8Cq8zwHBP8-VlxKTRirwEhQxK5otEQbHvX175Vluz-WrRx3b9EVI8iTIZTpSN5EubgRZtfbhKZD8RD79yUkUDpRjD_bcOJZOmiwTzNwax9iyrrNStRLKEyYkmmNH1jyyT6bgZSvCS4FFaYxSUtzg8JRZ_Hs2HImYAxw9quIHkDA==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH0M4SdtaIUCYHOKEYzF0fVH-bwwj_3W01p5ZwYPujxVCCjwgjMnhV0b6jQN7zezvE3s0B_a09XfLPBkKC9rdOQgpbb3G1vbnZWi8kS-p4bQr6of9HWRp3n20VrzRkVLxb5GoEHnjwC9zimdfY80GDMRcc45kTEGFMLQFlQ0YfKbiSEl7Byyy3AeZ5eAlD4uPC5cwccxM4z
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHGXALsf0CzANihaF5kx7LZZtajKhBiWjBZOZ429RXcDd5JALCg41bP--cEzZsT0jofmnw875HLZ4HlG96rsRNK6RpF7ajAPCQ4JR8puNgK_ojXGEu8Cj2JsUbkc4gVTGqME8qzb4WvLnW7QiR0SyZiS-RftOPZ
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHMDfXE2xaksn2WQxo08uei5UYE2M9c6ngSABvGC3WWzsLzW025NV_ZbbPcoWqBSIEsD3S1dUdcEcSqu2oO0-y2vF0IqhD33FFV0NlYpArRuqTaTCJWOWtJCAs9hFdr62pia7Gm4Oc6NQRdyXSXHNcsPNPrcdE2n01HCg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHTolFZUosEGF8R-pOHEyGgcjZOlMGhtDtIfS_ZGwWlnTVNInUJUT6rLGLXbP_pnVHd8r6Ow1tNRKqG7TaWRRM_kkU5fAH9A0t4hWKuPM529HIq8Nc6QKrcW1NrLFy3qXLMD3vnEwXUfWwi2swdS-H8jVklpnygZN5C3kZEtuQgyxkxB2vlRuaMe6ebkrZQosFoLzzOQr4iR4FkmrCyTA==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHU0i62zFrUAaKzdKkBBsofgBSt7pso6uHSU0tWvz1qqkmZAdjg5dZmxRjG-zAur3-_LNiktwdUhtJX48pSBgKEXmHMpmnqWaMdJ26j6bg84jBnXEhXzrzn5qEf2iU2z0SlIa8JiKTwQ3XV1JEkb0YyARLmcQ7Q1KKZeQBvqPbHltnRC9oxFkbioStNejTisTSx0y6-_p8=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHeTsv6SFWKWzQ0ybwlI5W20qKoGxhyaHDPyD34iSEnUdhiwZrr_4mkOia-VPEwv5_Jn4qC_Ot8IK39brTEKQ2DyWG42weYspTVjMpCcqe2kHiHwodZZ2QkK3kO0Rn4m1Hgpvfv055g8b0Q1hDZKfo=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHy4jCZKXxpNIIPUHCF0WFIgELCZcErxghidY9yfsknq9CdO0XS88jpsZCQZtqruILPWvSKrwQ8h-ISJSAD5fjUIfyMT1i6UnR8YrxaJFgQOZpjj8j7osPn1DT149D_LonqNN2dP3rnJW2HJJuFyv6E4bsVo4ptuHDdziI47tDx0295CO8zCFzW9YMOVmQbDQ==</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>BT-187</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>advertising</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Group of vintage Chicago sports felt pennants, including Chicago Cubs 1988 Wrigley Field 'Let There Be Lights' first night game pennant and Chicago Bears Fan Club mini pennant</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>$20-$55</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>5</v>
+      </c>
+      <c r="F19" t="n">
+        <v>5</v>
+      </c>
+      <c r="G19" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="H19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" t="n">
+        <v>5</v>
+      </c>
+      <c r="J19" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-SEND</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>grounded_search</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQE1RTZOuT58zLgHvS5ZyTujcV2TyWp31qNcVgU5c4XkBT1LAjN-TklV8yRzB7W4e19o7JiXH6IGkb1ST7AqEVUV1Pf8peGUHYvXEdcoWuAtSHvjl26F4ZYLE_Ry3DDsBWxDj5yqRIGe0oVsz6sX8law9jVINCQ4SnZYIz4=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEg4zJkeyQ3ljA6QYdYc16qNQZRBPnoLneXYIyLmQgJiXlW2q6qlGlIo9w6nkB6yeLG5pENnNdakTrusOV8ahs68rUXPokt04xrNihyohRAAXsCGJaZIlCAc0SuLHf5QlFXxj0Ez9cLvsrVk2RwA5vmIXIvzb9K5DHnrcG2K_WjLnZi28TABqCjAVnDnEmLZmvX3C0SPTOJ28SoLkqe9j5y1TYwrg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEo9XR_dfe4vSJydj4c3Qg77CzcmAN1ioC9zaOkdszFbERermgsuTfSXQS8ESlWuzbnXeGnwIds1Lse7_PbtIsfueyYB17gWOCYWm_HGAuSmldVkFd77BMLgaxmGaZhH8LASXXQA0yXoP1klfTj_bDer4pc_8cmGjmIFERYAih22Id9KgOHVTEB-lKL0mBY8XBzlMqUsDw_NAGDRdDg9DwqC2YcKEviAt40hDdWo8xRV1pLxkSmC3rTNCNDcIZVjo3o8mlnCMMDJkybBJDXZvXO0Zlfni1OtIZOpOpN8C6UdKrjJv7tnc_IuMzHSSamcKv_8PVORpv5BVb12XlGnWFt2_KZCBFjBIOszC7onVJyZOqGpKlKb42vbqfj4I5uGnINDBG22VLzT5yBrFJNcASBpA68yAG-4TEklsrlSWtBYFpaEs0p7B2cHd4C9u8GHecIVIjJZoE_M6OgIkqsANSyjugs10vLtGLAq7BNiItRdlJPK83356vw996QqUB73zE24ASSXE0IMLIRguX_MCzhbasRAmynqXT6wfnbyCDIVQtaJ_GkmwatNvqflzFetzYMfJji68yQQ_ACleDdSsx4oMbS6tVqvdSXPN9C-dpTJ2qPOZJkfSmml-tcaej6FOf-jC-o64ng5W7yiNKmcVJWMqsZqrNJ7nPYWTGCqs1q4ANQuxFXxxaT9LphOe90MkuerY3jFXXB5rS2d08=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEvpzZQW7DRD2T1jEITIJSyRdtbdafmz2BdkhP29jTKzPWFKKlUDTxItQDs6ycN80ko6SuyWBKHQJt-5uNe9jqDBOKcpc3_bfcirkaDL2BBak1IrvvJQ8gW9k6JCZZJZnb1-QNs-IC3maoahQa7KL5l0JXLZ_U=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQF-4VflA5ZYltGlgx65-y8eRBVf-Eo8GpAsvrfgxKUfOh_3CaRJAHnVJ5qIkklBNDL3sdTlEySsr0nJvpBPX6MB8U2HMylXENKTgF7WqZZ9ugQkBIaW8OrDs6XIa3H7qNy3fZ_Gl27DAqMdXldJhAnc1j4SzLNuZx0hsALWApBXdXFwoSd_
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQF_OUC-m8oBNjQdyYTQAfFQKpnYZDGfu3T6GsCOEtWIWtfaUUixDXygEpaZPJE11isnN4JRFs6R4f9zryh-R3IPgNgNZmjhe6iEypzwh8ab0VuE3xucpvfprTcyJ3y_pvUAR8ymIm6UaNdie9ejWhOPJnDIZAUlUcNnSpdVZwntIrM4Hn1uAuzy_Ru6pbc66ycF8cgK_0QWGnNhUQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFkh0j4E5JQWYQgY4iPlyWXZV6t2PtdroRzCEiHzrm-7vT_k1kHg20mZfTgxT_0L2ymV2h-VeSMjwwASiSJDXA38UNI3FTynHlb1acudeJSlOSACvWdLSDYEQTvVzZcom4Y1ZX1K601wsUjbhu5ewMzwNVm2vRUB0o7_Cl6WK8Sx6TrPN8=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFwfmumgJOD9mPQ56xtPdiv9xw6ApVDvCPMBQulXFxOhvrisojYNISjxSGO2mJXznnU5Ovj8REEWxwE0nn1lPwZNvXa0BkuEieIUs5qjmsmqNkq4frmZlAzmA3CYPsd68JR_EMlKilyTW89oHBb57Mn8vUt21DslYmkiPlzYN4MzdZ238DUWuOPrdnpxdZuYAC9wZHSfNJd0V7G
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQG4pYGi920lRi8RDEtuO5DQ5ytOL6LrLFZ4uoWWBZqvNnAUVIhsLijtzhpcb5geM28anfBHUnpDpLPyDPe414Dz_aO71MHa_zLyIVrr3Lr3MnUfne-fXcnGxr5Z5WNG8ZYpQgS-p1_RoyqwInNLoHTHu2_w
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH9NHOI1ZUTFsNqa44OMG-Tl44WlDODew9SeXCx3SVanuEkjdkNnj4_QzldKaFGgMVhG-ZwihvF0xDrIWmD03FGXkMyyigL7V_6tbqek63bRADheOCxBDBBQCiKFKmGrD_JS4h9SJYuXNxtoZvSm7Vvi7AXiz6woBHyWcBC
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHFgswZ8riDiwRa_69aAvdfglaa9mndS_qBpxv3qQFG2n-N7t5dVLefFyj_nBBku5BhuLqF1RMaJ0DEyi4eXKcjhLI9JjSqTVjHmXWiJCUxOHnGLbNpU46zt6qLeidpT3yGOigo6BHe_7HUS4_FGQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHI2vIq0ydj1AKQv18hNaA9aHXuUePGKaygf6oXQIx2atNgDWQNmLxYwXo5-lcjMXidZrx7PHOK8moz2xFMweshk5bSLKEBwvGs-86PWRVdARPVyg8S6ScTXV1fB9DBcVnv-35cKAO6zaMBxsV3MeQFj_LJ0ghWlo5f0A==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHIaunPv7Fz9fs7r8_PlawCUGTz-KtmDLu0wSrFkffjC08WChnLA0LadFpgJ7dCrpPJWmaCTb-Xrqp4dHkG1oa0xJCPVETWzbwAnzPBPZwv0gs1RESkUER0j19aIoRHDEw=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHKXzb_44u42JeECuR1LLx9GbvohbEkj6b1U-abuppbNtHTit2ktSusdsPrevh2WbqT4FtJKEnuqYJR2DTKW5RoZzNY47_nAB9zOCjUZglbyJeIpbbzhjLpwWQiZC9-jvs=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHcR2n_Opilkb9zsKItgBWUSJKsxODEBkQPqpEsxVm4zqRMV6_Qkyq5ofQR6LOnfDi_ZIyg6Ojj6JiPsBxCpAoNPnY0HPVg8czKOkIgCe8JJov5-f8vlA4q09q8sy6eoWLrcOPhtNu0dGKV7gZH1oUOXNfb0LmpVNhYYfN_5rkJOAs-oGH6FoBttDer5vOLsti3evVjEvb9wkkiOsFR
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHtkzXIEl4qAD6HgNBeV9v9r_py7EDSPwzZHnQeHLjy_Q0Yg-qAXtl2GVs3qiHmPqVByAbLplYReC88ryFUC58lg5x0LHNZRNkVOkzhy9Kg6Bf5Ljv_Lv1KRP8iCw-Wdw0Tor_Fd5owEAreahnN8AHKCy6LBaLlIKLjBgYOIwlkA3QmtpaRETGCs_GiSqQNhRuyTsA-xiTL5HiXvg9BHg==</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>BT-247</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>breweriana</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Vintage Schlitz Beer Pop Topper woven straw promotional hat, c. 1960s-1970s</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>$25-$35</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>5</v>
+      </c>
+      <c r="F20" t="n">
+        <v>5</v>
+      </c>
+      <c r="G20" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="H20" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" t="n">
+        <v>5</v>
+      </c>
+      <c r="J20" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-SEND</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>grounded_search</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQE3U-ruFdHDgnzd9lA-KX__ysrYchY7diIwcQh9nfRafBUEdm40ektvtdsRLqK_LPoWyw9dY_9lWuN1OkeXP3xbV5i9yAf1HaxawI-5ehXNLCnyoHhFJpxsaa5L7A22h_QilAtu7lzoV0_M81scik99fwQBnlXbSzIhnXloQ-ZlyvtjOhHj
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQENmk8VAhUiz1wcUbN_ZAf3r9MmJl1tbg_HxmSUuCL1iPT1yU1s3LcS_164XlDCNsgo6ATL2BS6X6hOvm1-dB821htLYS5lCE6QnzwYyaAeunkV7F4g0zZzqzDcOFpvry_mXcxecl9W7dPN4w==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEZZK1P1YoFlB-AvXn7y8TXelNbC5DxhSgStZv8dygeZIyU3bwU0-1csNZA1m3rVw59ICBA8cY9niQCKkcS5A1AxFx_-7kPuHA575WpxVCdFCHSO9xE33s2TR8GwhMqobXOlgRQQTnHdXQOe7DNAMTH77ffvqCGPO5IUY5Zj5IluRU1bYSy-6Mdf5Jd
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEulbVNTMAGvyRlMDW0IvuTjgBW2XVwg_9IH6qStliLHAeDaZOH8JO7ptEnreYeQ5QctHinZwVoTb_wnBUZSbwCKGTuKgW0-DVmE8yIvOcXraYHrsoKR6aY4AoqFv9BtuYkTJ6udlEW7U5xE-L_eTM=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFCm9_gffUxwL8BBCMyddD2eOPoK38qyG0ZixdOSf-RKBfH9TrSZeRaIIk1TPuwDxIdMIeUer7ESeRCkeR3ljuQ_c-IojzJlxLXGt_-6A1Y0u71ylzmUAUNWAwysd9Pt9Y=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFCxkkADNEVab5x3aFk8FAeZB6nXhR8Q97c6jVGPex9V75-txIMDGpiZmnIbM5HAIDtppYBxZiuVmz-K8RcXFeL1hjfd-oWPmOM_SaPosbAk_Bxy_OANjxy_ZnTnFrqi5fUP0uBG5LjKwKSKbOHSzbAJJuFC550mBgyYQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFGXi-mdyTBfiaLNhZReBx2Ci3Lh6y-o7WDp4bKcq5mOZieTf4gECffFjLBiNIqwm2bqKrS4YZbzCCKq6_yUZ7yi3jjfiKQuk5duqYgr8FB_Ti70Fz-HPlnH40B900N-I3vkG4Cuayfu4XghQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFRkS4FSwS0Qv0TzJBH_zxt4_4Gp0oOy9Sxj73eCCG61Ukgbbtrx_RUS8uzXkWg8DRK0CxaITKwGXUL0YvsQGmttJayg9OiVdBNYpMrBXmArMXOUieloCgPTutU7zakixG7Cgh5C3VI0SwwuX8clivysKfgXkqbY_z3jz6LxBdA8e8ERZZ0DHvtP1x8MYORbxh06l1wMGc_Hb7PLy_gcNPJouPwb8motd2wGz1a9F_jIx0=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQG1idLUojflhTlx1KZAoxGDxzDTB_yeoI0g8CVURHKhWzogS9QJYvf97ZNPx42lN9RboC-L0guyn1YXLFVjXbD6SWuaiBWtu1Cc0OeklIs5FpulEaBN7dcm2rhtzdh1BKwGpia7nIfP1aJovmXW5uZpcM5RyyMd7fIR5TjLeP0F9DdchvOO0TKGdWORRXcHvAPYS778kZgTJluI9bhYP0Spvy0R-AoahOVnJDuQrnbHMFIM
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQG1rmyZMUwryLemEbX-sIFlmxSMLrGhhO8SBrtUuAKgyRv93ovoTQU_YxVJw_4mV1Y3ht5FL_AC1RpjuT29ZllkZS0ESkIdbJjfWQIO58w689z-OLmRCFpCwcXizPFJjoY=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQG41Se9Xey9BCNV0vXxV9ApJkKf4uat6Z7eSoGpEfEbyJUUFD_ZvIA8AeRe43BoPw-a3btS9SeCFYP7AW0yl6p0ufZf8jjgzAFyWC46oU4c4LFKtcUV8dLAQN-oEhGCrAbnYhvt_DKQ7K_xnso3tB0FigfRT-W3AN4AlsUoY4EaloyC5auolT0HSRMbHki4WzEekgKqIQ3San5SZSiAYi3ijbsuFEc-34sotKe2Nit-Stg_s9eGogcj
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGUSwXcJZ8m6GrPHu3kPntwN0GoMP_4JwXMacfBGhhQkHVqRdsWopDAfO2Mr9z4WMG0W2mN8NS_jx60CMg0_HMOsN6SsAWId3CpLzGKAH9HMnUW3_X_hL-ZHAg9af7RuKbhsxuuSMEctbOIE2uSF-E9w06mTi3LNXU43xbNGno6TzbR5Mrq1ja2X4Y=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQG_pQ9brYdAhx1jYz2J-deBms77oNHnayeIGVVhJTvoBGbTKLMZGBlnyHsN0W1zVfb2Zfk30e8rW250SjAsKMQTbqkXeLMCGaqrSIQ35Fz3x2cANOHovSWwh_363SH_OGgAH3sE9DZJGTnI6RfVKF1RN9B34gO1zsuP_ngSRPQZhkMFUodsxGcq48_M
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH4NRYkHuBQCfkNF_0KjTsFNc9QOuFjiVTU_vEbQaXwC9NuOW4Wolk3GGWYy9MfmALf-p4A_b6ESIgz0Xv7KYBXhnwtBdt9HEz1xbUNjusQmfMRPadNhZ90y6ic68pXc7czbHGdEaCIGn3a-A==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHCvhemFuIIfT0RVrFtUYlGWUdILz0thLVReXH5zWPFMnTiBEyiRKne_0Ez9NSal4kepfwpvjWSCcEABQEuuvpMUvu3Zbeda8gNhOaMmdoydus1vsJoUcI6xTKq-NMbvetH_9SI7vnaqx7nVDcNGvM=</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>BT-256</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>vintage toys</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Collector Barbie doll, 'Barbie as Scarlett O'Hara' (Twelve Oaks Barbecue Dress), Mattel Hollywood Legends Collection, c. 1994</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>$20-$60</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>5</v>
+      </c>
+      <c r="F21" t="n">
+        <v>5</v>
+      </c>
+      <c r="G21" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="H21" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J21" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-SEND</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>grounded_search</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQE02YPeiCUYFHBByWvNu3e-bMn51ZPX3AkgUywFp3IESfbjLD9eRXxGgc1VqjLIt-z9AJt7-z3YE5lR8Wl_YofRAKA0hsSQNzX-yNjSptZpJZJHn6HNLBYtVNrZTM9o67o_f3oNGSyJFU_mVEtbSDmgmCJZ7asScJzr75yS-vTzJVoDyEuz3iPrNrl8rxmqjisX8ahB98PsndO21hQPk-6DsR2AI4gQ0xsPTgchNLP3Lw==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEFbap0X-mdY_kyI1MdH1xSL-U6MfIS6XgjCHgqoVDcRuKI7RhsH53XRtzHWlM0c0KNj5CKNT3Qj9NAbOmp0bqs0i3nqbChN6dCVITCZ6sXcKuhh8Q1T17IU4qw6T1gH5pOejPxGspGO6zz6ETaRYZx25AefqpdwfNcP_yu8yDdu58DtJGXDDsvhtmUVhLPsIyuFcDriVdenMSsWf5pbuEAEqgxdse7hjBngkOMpYwGf_gNI1ip0DWkfkjnwluRAySd-9dbquY5iMSS
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQELQAgKgElkLa8rKAm_-oo0H_thCp9JZeRldirc2yECZzLFtbuFdp17EBSAAkCRmfysIUf6ZKGPxjQqlKmaEKPM6pAPVZb34M-z68TWSe-7axFZtZSXf9D-C_SSv3nUnWzwGdi0_Sv-uA==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEksLlcD4I1nBtsgLeYIz3xS-gL0YPRP5NhWDXfcde7OQi6yQ4jo_fX6ehTE9qQ5fu0coeVPa5kyYwAkvEuTjitawdJm_yBxsKHuzRz1-B4yll_KdG-O93pk8ZMsaXjSJCjaU6A6hCDVi_QRlxhE7AsvAptvEsKvfit7Jc6l5KmopWV3_Ns
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFc3c597ZFtJETXsxA6TZ0xnBlYS8e3qjbUrEZGqk7kK_PH0QweMWWGYDyz0ecNnSsm0HucPFlHNpIBaWhAdH8kZndbDy1VZX4rMsmkf0-IUVKD2eerIAeJ5vwdFTd9i-E1OwRNeZRlnXshD42KmfKjHBye6H7VDW9RkutgHnFVDB6O
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFxZ_rpd2UWgU_8vfkiw_RNEpu94fjr-wLR4_NjiJsn7XYTYJVPpzkMA0jNYPGjX3trM5Rqu1jeSuj-3egmb7qrtx2aQ7K0jpbwbBHeM8tLlrP9CGPfYf0kG0afgTCdcqM0VY7kNwHuSItWBVXlydX117OBSgL_Hmyyp9FIX67cR5dIdgCsVSGyk5Al24cO18SadN9-DsqIi66lSrVe4ibO2oZQLQnuVt68yfJiafY7pRH_x_0=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQG0km35upp-85PDxbFhYNmEZ7vk47WN_29xJLDVRqrV3wYq2MWF5dFYyx3DUbgkDenP2b7XV8HfQ4VjqmWx43dr5cNE5GxsmSjDcNa_tn1lfyuVcIpn4L5pXIBuHltJILTgLVzZhXr1ZnpbrnyEtMoE6m0rz4QULXz5yKXi4rY1dEK029aOIa3PiNyfaalwYXqWNmGFHrkNR9dIVRMyDhdtPTgodqZEGGm1iBt6ipVm8IAhH3I=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGEQveZRivAYGSMUD4iqJckblI_hMrYdrbye_viC_pb7WXkMe5qak-_Me0zLUCCPjoY_6YL1ask3XMYZFhbgC5lr70hZnMOjl3j8zh2eDq0LGZ9IU1hB6U0YwtJOeKjXjg-BeCiQ_A84JCurW8v7oVyH4slLpY5UXDk1fT2yReHXPxSbhCHU03aHe0DBfXSLrDYi9r41lSN6y2Mg5StvA-UoCEB1YslTxISGeH1F0tI5z_zUQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGkp4LbVe3uIw5gdE6pe3bchJ5unSUiL7tl9kMcOxXcg_w1yGtl32OloI1-5QnxiUR4AyriSTdGy58EulYWK0uJ0rR3DtU3b5v3auZOZ_6RVXPLFUdaym3eECF_Sqc_eZ4yhrNgZnomZoUc-8cFQTguc-m-mdPEBEB8czwsjhu8WIU3
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGmluoPxfGMkmsx48HMBECf_AYyfjgtF6wvw6o4tBfTx3n94VW10mpj3KpY9pDqq_XMYwbBAzSH6UEEfP3TIFVtzB_BYZ7PEnuIarWOxdu1ZNyQzXLbfiMaB9xA5Ta9hExoTKKrRDJ2g4UcwNIrCpp-3tELSF_NeEgdtLOJAmE2kg388_qbBw5YQPbrbDmoN9jSagJ8D5fDIo_LfXm7G4hX0Ifac3KC03QDoAaQKki1RIArFfL2WIKrQ4pqWS3j40kL-fwH7WEgGg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH723lcoY8LdlAO1wxubzDsb5f7LEGp91ELZthW_OY6k44PvJAGfaamkVVgDP4kEPSJUWjRSPJ3JK-rQYdTrdJDgZ1qSmetKbKFx63VOrb7QiULZfLpjBj0o6AdwLZ2Kf882i7XlXa3JST6ibnUhp12zmBkPIABtQZL_Jx_YcfI7D0FkGsQFhrLe4ogIYAzLIsFl9wMn0ezWDD_g3-vfNUQodA-NVMSpAar9ydY-V55JrhME-OzLutYVAQ5j6MzJuNOWFaY2B7y8w==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHoD3YN0DdUIt7YFRD_vGNGf6vnmYmL6RYV3Bb6wtPpsALwTA_hjEGL9P35pmCkJA2kO-30rJEi12WvtFlD9WxaWr3QMdlE6xxmpYkBDOtd4ROqKKooshHVQsZXDBWHN0QnDNIOHufPcjig7rDu5UvWjVPaLTk8X39txhzXh3hb_eGt
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHr8a8OyzUPq0d5oZ-0Q8LfUbfogr1u4h4bQ2O9vlfLvQHSwj3YEpFO0Izzm5uWaHr_QjqJ2rwRoJ-MMFobe4tJq9D0GLUNlXU5IfvzrwEJO_C93zJhTIU2d4XoS3Sv_3oJDudE5YQcu5sIlTqjOVZe7HkJjmaqlU7pgNeLlcfKegMhlM3Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>BT-274</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>breweriana</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Group of Budweiser lithographed promotional tin cans featuring baseball graphics and embossed plastic lids, late 20th century.</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>$12-$35</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>5</v>
+      </c>
+      <c r="F22" t="n">
+        <v>5</v>
+      </c>
+      <c r="G22" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="H22" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" t="n">
+        <v>5</v>
+      </c>
+      <c r="J22" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-SEND</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>grounded_search</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEE_bX-ueRRvJt9bI4CIN6HoinytQ3Is6j04fCTdbksoAgchI8kgavX0G9_kI-XwDDz7096wpBZ9SQ98ECM5F-ouRbJN1q4RVXe3dLAvJ1lR6Cw3M6kNLsgmwxg0XEGfWb9OuIGqA==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEPTKigmCriWItB1pzKP9PiIB6k8jIZN3hJBbgY2mPCofhrdeh55VGa7N8UaEOWh5YeZj0GMfPiFDIIIytkYSgq3RqvZu0bkONs3F_lH2OdBPPgdi7BhsnaejdG4z2OOntuOl4F_-wLfg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEVxYcPjnns3GRB6WzX27grQXf0dHRNG_97kRzcOcBIlrwZfqKhhPAH4oGbgeGv6DIxcGuf0-w25i46qpZOavBNYmMujPPI1WihMDz9EJgO3AbN42u7s-epXlXJ70gDqQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEf7BOydqT52zuWokxXoAZW2Na7FarTzEZM9tE_LVr859q7M7meedaXg_UXT8CY5DBltOHddpwfv-pN9XqY-PiYfz2exxXQspNx5jbTjhTYwDVggt6WkZ0aixRqMoBcdb5WGJPVSsde9A==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEpjb5FfOzFfJKJAGyCT1LurGkW-MsxOLPBXad1svtI3HOScjyay67a0FbgpXatoIypPrt82GTokUigGdi7Br4v2jWB-Ovxq9JkIlOFnnJeqDg5lfi1RKmrOPR7Ab0MQWc=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGPGPj7MTGR-KHSvyIZTmP7h1jt0gPbdLMpUxdIHExhXREoxNmvw-BMBeZx0e_6XZIw1JkDwB6x7qMO2xw6Y6nqP0jSg_wdcyS-4y--2KPLJqNodJ-Oh2eMy1sT6rgAqw==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHNW0eygsNN7vJcxSGBnpdn_-3C9ezGOP8uu-Udlh4FBQwHZo0mewuLGviyNtRhEC7OvwKlQBlSu53zFCGVKAWLZt7tVszYMGPLTFwaZwgH4wSvKcYLa5k1uuBU4f22a7uiL2sQczEHeTaXCr-s6h8ZhOS5RHRnvtZQuVo6eaGOocm-
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHVasvANE9O96_SjzFyiNaSgZgSnpW7MIHXkFCVMQjQuANiL6Tl37-9ZmoeRMYSaj4Oj-3WBxFkbGTgrRtQgQrGyZ6Zr3rBOY-NU79mmgGA9Hp8gX6iV8VNNmebev_Wgj37zIxKaa3SA6YeknzAP5tSdz4XnQsDCeCETIy6RO_ituQLj_dmAHrf_n7YDgDGKA_bYB823C3hXY2KLtrIVBHyk7_b0StEEPbVlikqvTNE9gs-MYJbQZJXE509JsLHJw==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHeRMcCl9lO7gE0zne6Ni-12PDuMl8QeJERSuuRQmbLR3psRUPKVctiuxJHUTO2mzoQ0Ocd0ZmtQkvyB9ORUfxeS7sPUphimZmr73SphfReCo2vv2A87HmFYKtLCqyqiZ0nWI1XcaXJ5GMij7aKnENl5u9VVT24glrrMUcFuOsnkmhWn0PLWlmb1CrQ2ZN2To8UVRtX7El7YuTlIB655rc7BE7IhjQuYv97V_Ca2Xx_nALLdDNxEHFSdIWwWtLIkQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHlEND8EGEM8fohy_ZcERpB8NUAmTGpU--UQu-duRYRjdklaFSegfw4SPjy8m-8sI-Bgp_seuJ-2KV96zqqMV-vyia_SqG_IJA2Yr3cbaJxl-gowoOhsYPYg3yhXz2SlEc=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHq3QUvEWgetp5snrnJkW_K_Ym4Hr47FwgGgLWUhlvxNUp91agwUJoV7XGswnaxaOf0bibTjlEQbrEmZQjiBO-ht8P1zAxCPdCqLDV9XTE8ZTQNH_b1bT0ufEJ2fCEyB30=</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>BT-337</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>advertising</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Lot of six vintage tobacco advertising pocket lighters including Camel, Winston, Salem, and a brushed chrome flip-top lighter in box packaging, c. 1950s-1970s.: Two Camel Cigarettes advertising lighters in original cardboard boxes, Two Winston Filter Tipped Cigarettes advertising lighters, One Salem Menthol Fresh Cigarettes advertising lighter, One brushed chrome Zippo-style flip-top lighter in box case lighter in box</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>$12-$50</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>5</v>
+      </c>
+      <c r="F23" t="n">
+        <v>5</v>
+      </c>
+      <c r="G23" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="H23" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" t="n">
+        <v>5</v>
+      </c>
+      <c r="J23" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-SEND</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>grounded_search</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEfL8jI4m9zr72KeMiOdx5FPWEUzn09S0KAwwy3DmDWWSbNN5s4NmHlQ6hDH9kCFSXH0WG-U8Hi8ffLrtsmpr08EpPOGW6I0U0APFSWErPrAMOxJN5ZdHaoxZ3MdiOy6fg-WA_FXduLJ6ggA69Lp6O-PUXRUTNb8iFQoX2oWBFCdUPMSIT7-gSmZyJJJaUv3ydnuQxdeZwcCK28yMGc-dlB_55aIw==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEfm3QPawlhrNRiFV1_bDCFJvVOe7eUcjFSEn1cRW7hJlCTKmvwyqbc6XrmsUIRFbBaPi-bXcobaiwiqEAR9WPlkulYhibJ2DOubAet8GSGigQ_tcXkVYViWjgKjIXOq4s=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQElkyOpXO7jGSGNmcJt8av-lNhNeUO3w1eNC0TFULfMa9is1VyRGWlYWJN3rZlPEgCUUG9Qa9Wu0EeNi_VN-suAO7KrYu5tXMm6TYD-3IzAgET_dFCWQBu1R1MzJupa5dhBHgLPQANVDaFRpabNWIrqHcVwpCBZ
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEmPr99O6p-d3ek2BZsMHEu2WpnS2G2jKED6rl1AMg3kXsp7M26_79GruEzssmwPL1hUl-9Vh51ZkxWDjiEYm7ATTrBgtp7guv-GWQfKzJGXP7nFWvcFoY8FjHM2MU14gWQuY99WsQxZvutQHfE_z7py2NvcST3J53Y4ZkfGA==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFWMeWu3c0YbmWKd83ZCAm799D-3tA-Q2r9uLfqWr-2ZQvG585iIqiN8EdAwHeZK5fYi4GSj9l5Q4jksoCgRyk4aqeAEPSWuqEmNNKexHl2GFNTwqBXaokWExSz3L_N3bylwOmzAMTvw1vhYlQ-GECoJYc5MNWoVFrk2E3v3VkX267brZ4CycRC
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFzqbGzsdM0HmHL_NbNWoiZ3kKBE6sLQjckgx29sqjTk2HN9f7D6D_oZBRUISYaQlLBbPLcbhs3UHx8mgqQQbT2ABVQ47y64k3vM4Lkkpm_Dd6dOvDLkFkplrNpSphTS9KdiibhQKqxz20cUXiSyNDURyyR6TVnba5M-Z3GgfBt1pMCYV1Em3wMfrC4QUoH3uBhB0Q_Ld0HchR2z-vE
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQG83GH5rPgXWJG-4S5QWzGWYKlPkhYKtzySZA1WwsfZ_sERxgzPIon0LGWrXQMA82ZpADJ-PZsL4eYZaCQoOFu20_zLDGO1DtRrXt4LJKUqKBMX5haQIkB7I0PA59Eqn2Y0iIrNT6XB-wF_rsqRwiI1BG_R1jgGYs1qglZuh6-i1u5X1Kp9elOTGRe__M71d6kIk8AW
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGBx3lLREQ7g2zHvFdpSMOJWScG7q3U25SAwsBt1RegrgvYWqID-7qJdTwiK7cglmLA-Izxkec3lNgEvcOS4uByHiXzVc30I-i9ULgvUEt60lNq9Svl4U4y_iQeTbWaZJa4ElY3AyekQyFboQtOPXT2coqQ42Hq31-0snyponRa5U4EWIcvG-ppDCH3zZRfnxGOApUSSqSwYAjjZgKOChCi0iWP
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGLCmPAT2aDmpw1iwHmo_s17mKONk83nxKvmwxYqSmGFTlMCZf7_NbcYZ2wOiKe5BY5p1dtNo4rrDfQ2UzGjuAJ_kl55heyDJehoyL4HgSv3TGFHv59UGVKAYRd9D1QjpWdnB9uKzaI4eai9hICVzQmBD1KmUa0aQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGlv2VCNs-KJY1wfYEolWFaPiNA3kBoJfq8I5grAmIe8GR1XUxW9aG-ZnOiV8y8hIXjlrvzehhFDwjLqeKjuWEl3P1A8ocCpi_CtBVVTvjSZdDaOdPH9FaPmrNGPxCSeBYNhs-q4xMMiIeLJYknlrIRxQOjWkmRAhXbCo7yP5pZFW0DJK_yEJcBdobIfgB_QVgoUpqs
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH2cB5SVN97_BGl1wf60syoXoqKMRe2kQWQHb4GQJAdMfC90HJlxJUwqimW7nply3wWtrx3m0zeDyI62jl4J64mGrBKtgjBvtStbADYLiLItgHygTz-PlDwRBVj_5OQE9K1x9uXtXYcinNoYg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHBTodpYeFlu21DzygHUzSDd1oj_Tkefv0Kh7xxQTdI2lhVBqhz4009X0Mcbj3K8ZIIknrwwLSw4mwdPs8kGMTLyfh5XJer6n5fWK8uYq6rgV6y9ESqFvHM64fbQl7lHgYb1t6wd0fSNGA1XxSPW-vHHt7MRDQiQsfxsxPqPKCezcGRArzdTRWN4WOl1zANakS10nOGyw==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHUSvYas7CSAbNmH_Y56QkWiS7JJkSxXAUNQmkuLV52KPwN6htHK6VmdkLugtw72_3FArGTcueRB6qgdk_O_NIU_3lCGcXqpAzcb82SUjdIqQZludJD_EwUSDb5d1IoTt6yWjTPK9qG6zFPCZbRJQZ5CGalHbELsM4Pza7RBkEAQPfcRr0=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHjc3NWsc4R8jRNMxxBditO-xrL-goWcAkgKPql4fEpJaFmocxhz7g5p0XEAX_HHhq5sIRN9PYKOdKvz2uwacXXDiI8kk0F_IS7ZXiMsdbIGoj6DfnPeTyYeftYIS8tMXKNlBydTDcDjsWYUFNZx61v0bU=</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>BT-362</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>vintage toys</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>1991 Topps Traded Baseball Cards factory-sealed set (132 cards), featuring Team USA, rookies, and traded players</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>$10-$36</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>5</v>
+      </c>
+      <c r="F24" t="n">
+        <v>5</v>
+      </c>
+      <c r="G24" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="H24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I24" t="n">
+        <v>5</v>
+      </c>
+      <c r="J24" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-SEND</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>grounded_search</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQE0k_QwJiNrVYS-Ssj-Zr3N2c1dd1QScDh30zvAzQxGY5fPoe3AuaHfNQ3bY-TRLLbJkKb01JbjvkzppMmCn8ogp9zZ94tsCf4upBcTP3jkHj7XfPxm_JbAbl-fClrpMMlNwCXfwdaXe-zX2ngEOK5NLYe_q-m9eI81nGdjG0QlLiHFQkSQVCeVuE16ffpYrbW86TlnPMKdtkdLcQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQED_lCXktNcEG9Eq_mYdJoYy50WDRTlTb-X31qNjA23S4OB8F4RByTfuVwMKGdUceI_PIENnm7adDjvqldUn9uoYlNcPVFhrgJvO4atQO1kEVu2XVqWtPEMkkR6jTL45Zz-kfpMdfcIwwn8Wfv7Sybk3ORRlZjsabj7Mg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEaG9QRxfejRGlP1TP_NVQZWRHxzDywBpYs8CB7F88ohzJgu4vWGSlyPfuLUpM-rOdQfhNl0mVpnKmtlu8ZumtngEAmUoow_KkGOtKC2ENQStlw0uLyvyhCzE57_iaINjrezBrLigLpkgUSq7mkUyo2UN1hJOI17CYtkwKIDk2c661g
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEhbJISZyVIDHHRWZiVuScLKxkfCZm89kW8ZjqLOG8_qNYDdDzoT3NHELhS9uWpw14CUhYcdw8RPYCRu20ivANPPcYv5g_i5zJdwIX6-RQH-Nng-qa0du-z4Y-fEdP5Ee2RzBgTJ7t16dPaFQhzmSCmoMmSKVvA82XKRGCNbINYDio6LWUCxPPh4w==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQF2g6YVxKPA91oMfe6tlLdlKozZ7yqTi6pO_3971fomM4T0H9kzPrLKQOSRWCj4f8-nWaUC9KId8rFYKjSIxWcJAnhknW8IzwRcG75LmdQMO-z53rAKDWm2do55DxcrFyxVK7iTlwvJHjrO4Ze_Cv2-3muS90j0FZXHEXc=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFAooHV8ivKQa0tZkpBv99-TmxbdZoaxydE-vval19a1f1K2qnwku2m5MDQDqnoeeZP-t_J1k4oy01Lr_QmVyVM3UcD82O5U7M4mxTLhBpSUx7F5mwx3aIplfvw-ZkDUIFmisZMLj5jcVASfZeBJa5mbqpnl9ihF0m2N3GuGDJCqYGow5cs9MUOS0Dw
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFT9b4s8q1R_CcZQa4t7KHFp3_xAVlvOpnXFkCAhtVWSoaZUhCKmxWDCnS2tGcw_j3Mc2AZ88h6uv8a16iGdiQ1zxS7KzqcE7kXl1VY2qw1-qlPT0WBIeNnJiFzMu0Bbvo_Yi7xNwl4_6MNfgfVDWVjo42i1Tx3bHoFs7o=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGGDlm-PI4v5lnt_Lqzu14ojCqiCgV7awTwkLJ3puPo6f2cHgkK0HwGumG3-h1DAJpYLbEp9OEEVuROSeYDyXyptXLwuuWKDnktRUlIP8lF_HOpxZBl2qt1ZkAigE8CU_KWcxXpHkdVc3xWZIM7kwoyQFVEHFXKFv9zuah-Ki4ugwY75bUND2kj4jQUhefBwOaauZ2rzlZv68zA
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGSvXrkl8dmd7N5J5lLiPi0TgGe2dLYU5A7ggy_sXsvPC0TbDfGMIfg9jCZ7CUPNSs9T6TE6xl9alqzSC9Z3jpXdG7DsLwwPwpulTzBNn6oHLayU3RrIJ869rqDDnVvkC-uOs5j-J13cvY85AacYWNNxVvRMFIQ9UXP8_DVGlG3CP1_HoIewYlU-Wqa0A==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGhLGgeMXP5aSxqaI0_fse5-k3G_VPWLowkpJ9ZXL0RgLsc_F6KhjwRvbLBeOGH8Sx0HJXiMCNZyVyPv_RuuhQDyobdilYSqtwuos-mdpwgCRatKF9mxyCTcgb-lkQSRkitYVdyNMdErooFfDJpJV_xFl1x2EV33wTSRztPDb3rpG3WcCVmklx0xu_0CA==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHcCi8Io5jEM4hyz8WYM3xvX4CNyOIhaML1pMR3g7aFvzi2wfuPBMheniqDRYbztTVnk4VePa_rS9bOMT6XtBhgNEIDxaz1p3lVp52JleM6pM9nqGSWQSyjsIU-TDoOF6TYtshtQRNWtcVn9Fu_xTQkUHcg_S0yDeoUrm6ztP1kqOBwkzY=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHimKoD539Aezcub8ONKLc8Yi3RyuVZF5DwFKCs2pexE2-kX8_xF_Zdsm8lFRuNy4YG2edgxEsUFmpy9UoRINRC05TgvEvFq-ITcLaG3O0vtHRk3q8Do4E6vziLItP5th-IvLBcbykBM0JBSGZ9D0gp8JP6Pg8E4VN1O7aOZ9cyh3lX5jRrW0bNA5hgtg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHpzV7VUnhoZVjruPFAPtM5nuTmDs6KUmlV3i2JEOHHbB2rVvNiFu0u-Pj-3b2Vv1Ct36QuwC22hl_5GQhpYzMuHY1wR5OUBzx3CX4hSnZCMJsR3g0hAhjfgZL-mfdUwHNtuzEZ3W9FXnFWDLNwv8Pn7iiFKayLGSov4J0F0_iwmlcSMJGbtEtZEg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHrOTJs_jFUzG3ykSIx443imSTnAzFhqpt_HPkOQtMwAaTdhSSkMTveUnI-urTM-YkY6tNI45EM_iee9rXPgNjhdXAqVUkBlq2_ywumls3FH9F_0_GGPFlRQpS7Yommm1GNSyK4-cDY9jhc6ulXjJynI2E1FwGfXRS5cg1eDggakyDmxS99</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>BT-373</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>vintage toys</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Box lot of sports trading cards and collectibles, including 1992 Upper Deck All-Star FanFest set, Baseball's All-Time Greats set featuring Babe Ruth, PGA Tour Pro Set, laser-etched glass Joe Mauer card in case, Rockford IceHogs set, and various top-loaded and loose cards.: 1992 Upper Deck All-Star FanFest boxed set, Baseball's All-Time Greats set in green plastic case (Babe Ruth showing), PGA Tour Pro Set card pack/box, Laser-etched crystal card of Joe Mauer in black velvet display case, Rockford IceHogs 2019-2020 card pack, Stack of top-loaded individual sports cards (including Mickey Mantle), Loose and boxed trading cards</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>$20-$55</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>5</v>
+      </c>
+      <c r="F25" t="n">
+        <v>5</v>
+      </c>
+      <c r="G25" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="H25" t="n">
+        <v>1</v>
+      </c>
+      <c r="I25" t="n">
+        <v>5</v>
+      </c>
+      <c r="J25" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-SEND</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>grounded_search</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQE2hwRsPIW73ndeZPXwVRzs_a8CUYN9dsw15leIX5rqKhbAxO35mVpwlymNM-xuEgR5URsuPYqW2p4US1pmW4KAS4yLMkseWpR8FA-3baMflK4zwlQ1Jn6PyeYB8cM7qrWyj1ARkqp9T2UQD88-ZQGocAkrQKMTxH842pVI3cqgW1J8sa_PVhzE3ek4sVXyfae6BY0vOcvQXRDtYA9HyXuU9fiLFDDVtzXsRZ6XpAfD0Dm85RLdolw2lygWhKfjE3o0z6Dn-fVuFAcdfeV4UQkTUtoPIIeTR6IF_mMDjM926ebNWQPcqkywkjM9K3ULG9S9jeQ8ForZpDBSm5Ac3QpiZ5PnNRkIM9r5r0kO9XMMHsxkoKSJxtrVmcWFZ2sBhcuBIwkhXrY4PnSz4lMt51YrIKXJ6uFyqLk7w8XfD2B7TydoFCZvkfSinfihfv8nu7nCDLbF8-A7UGK8fr0Y8jYW8HboDwTI5XDZ3VOEwt_SeES5v_E4X56s1UUBNgUv8Y9vdLBJGVUCqRgLCiITGgSX6VzS0BmBSio4D2Mnhj_WgGiy7U_hPOWf-RAT2jMZf9ooOz3P_0mnmh_r2lSDdAC29nRi-hENFM8vQiIK6CHQ2XDLjdHmHR7yMEJm-N9v1ZeuWfAaemhmBdB7
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQE9YAICMTKrNT239glHVctESTbybUPuqHeQ3LxsPnvPYCdXiwUxKHtFdQyydzMOQBsBbhq-asBhrK4iFUVpzvY2CowA5MVvqE1pWkz9nEt_Sh32xBmEVlCi-DlhY8uCpKq78HFwif52xSVfIKhbVSEAA9kEg6VCx77CYBkUd6zqMzi5VWa8Twji64YBE__uiNdkEW3_da9h
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEFER7ox0XJzaKwaQA4ZP9PZE9H29uxcsyvdFS4SWQm1zo1k2i_V-Q3R2to7OUkVpVyelRsDLllj1pfXq_QZR3a7Sd0TdKLWGNz2DUgCEqj2AYXM9z22XTgxiWbbnxLXBiBznr5K9naW5aUtFVVcY0df0n681UCksIdLtIKqMN0YQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQESF-0AYcgBQKLpz2uRBIecknN86wtxaCEvricWlEG_dOzjonGL0WysEC9yeIkAgnYFHyuahuUPxO8RjCWghk9rcPDJd9NmFAMQVLwLAMR0sPnAjxF6fJUIActSFgeWU65um7WxaQ_LmBIo03QX5AH_kroYI_EUZmLtE3vwM5YOytNXH_-qv4EHvuTJtpBoqrhZlkNwtjjmVIDZvq48voYi
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEVy057XXSq8ATyzM919PggEd3yyocX-_vwfGsy51oYzo3owi6H1gvER0Ri7z23g5SpCaKTxxxkYLqQvtUW1Pakmueu4HjCS3gmgDHxLRj7lEAXb-dKA2798D1eDXO1HcV9TruD_VgYssvRCdSQOOBOnYwFhiJAxDiGChLs7CV366c=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEhxjjF0FwY6ce73iw5gK0D4ebGpNuUZ0kgS2NkGNIIADsUnYY3V7YLLzeBem1hn5k6cL4SAKN6H6n4AJQcxyy2RDipX57gw4AD4TByAFWxb3a8mbSHNNh-taM5FAfPo1lBGNGGdBVMg-ZnnqirlWRgQpU7TRDStxXap6F--CWs6TIgNZhhwo7JmA0BJ_f6NTuztRVTn9Jeb_iC6LkH
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEkmO1jGlNBTn0rRUxahx_DU9GUuJAGIFfT7npcyZACmGLiKTBBhMxZXuvR0ScEDd3YW4RuCeYIfa3dJEHbwzXlZKMtzk3qkB8PcQ0z-5DSlID0garUJ8gOEQGfHMx-Exr8DFPQdNiL2PwnjzPE6G1DRiZ-xzTp0xS2K-Ki6DrBTkPFikMbf3vyzmOeiavVnLo_cIZTzLHmf-OLJyoaJu-8rsLFwQX-ibcnZej6eAs0Jq_IwwA-TG9iEz6z4XhF4WapB5yuNxmIdf2Nmv-X1ySeUJ_h1W9T
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQF09Oezc1ysqXd6tIlpKfb6q58J2V0FN_SYqlfhmJGlDVgC3Hy9tgHtSVz6RmgIgm-CWbJ0XKVK6NzfMa4vxXhfMFj2RF7T8rnU5s8EcrtguZmAsEYLv3iOhYoAVYQV5iQ=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQF2XhfngqB_R4YnhdcLfaCYigatrrffkxVCA12WhDYLzRdOIeu90tcmpednaKdlczITg9FJ4rzbhlazGoCcFVs62BdNVYMA_IttBSm9qpI1GRWtPQGx7JbX_0Uiq5WxXXga2C-XMoMo1EzE91VNuT85xI2QoZX0QSSThQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFFU0w4cDSQiUMbiiOmFcmc6TLE7BY-2ryR4M5Crq0qGkkaFRD2koXJR5CTTbZHNfqhaPDB07siPtWu4K4gbp1p0aXSfdlGQVB8bBtYJ7mULzKacvnrMvdOBxyg3rTV8PTx1oEfs6_E6Qx7EafIG0gKn2D_FEbkcuX7lmqhcWqB
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFMkKhPPkvGtP7JcAEHSWg0F4k4vlHk0sUmvz_trMAUlwU2bOmhkbJBgtDxTHytsaDfZO3XvJNZJl9e1ycMW0oYYUGbpvq1cFL7GNis_VEq-I7NXSCWR62RFSCO9mwAJ8mkJ8KI9WMtP5wZjIJ_12h3m-K8JxUJTK6YeScuszaV7Nr9khugkQYsnl72JN_0-zH64PRMyyFZSO_mkAMXRNROCRrirMwF_I3Y
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFPJEwUXcpuYz8oNU3gapk9wqXhoRILkoI0Jj6ecfYb5fK5PwwVrQ3AppAUK4WKUuFHioDZNFtuzTpdXoqCUUeXzTRx0VmacGsI_BnyCf9TzToz_dxm9HJU7tgjH0YFHw==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFc-_6ovbz_gKEUyDnmcYcL2m6hiGn1XdQlUAXBIXlSQfzl-_8RG90PeYjMetkQKox92oT92ovhL0dA2IlLouvYnXvEu-kH1npKeV3g-wVZXihOtAziNsq-z8ZyKPx0oFCcS67USC9r8ZYf7ZhEajQB4t6XuXQqbrwi55gle7lFhdTLRA==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFh8o_MuW7yffGgKPW4YE1J4mnL06FevGfX62u_Vyo3Y5fXXyPjI0U48HhRaO7-NmwcqEg3DRh8eBDN-N3GXHV3dQzSWMiylD83IS7NkDaRdCGvPHpBot1SUvmGo9o0GCU631M1L1K-dreowKeCQygWkw41S_Iu5DLPZlssT17cVrmQf-I=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFvvSj1wSHtat0HYhSJvv-wUij-QUjNmrW1t5y2G-94PlC2W2FWq3IS6NqkcVMam1qukenmQM1ZKtOd0cjpo8D9A9g9n1jJyswnrl2quCbREWt3Jq0RaN_Fleu8ON7h_DE=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGKzQ6crJhcXzzwcBUI0EgTqAMDUwDtR7ai9FKaMPFUwcJTUg11pnI2GnnoedMOwLpf5G6RQTvI-5wrB48aCGBssLEuQZjklqdUhgFWy7WgK9VZjyLxG_kV-asfFaIsrDtvItB9PPYdGBoxIc6aHEbniSNnUpIqX081gfVBWSvnTwqEeMWw8gP5F8cykbwG8f90Aae3a34=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGP1xHtZqClWqbaHx_WPYS-6R4XRzwwJDD1F9jhFRKFBM5_aVh0y23bDw-_AeGDxaek_UHlBsYLTdltlwta-hhTZKwyuehVy_5PgO-vLu_-wHHM_I0tQBQ-hh6yH4ml8Ehfg1RAQPnWSnnorNwNCtpw7PKhkDpRIkRJYCYn2WNJ28UltN3olzSqat-s
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGYqpgshe7q8VBGrXEoBaOy_36G1w7wWyMRm7sxZIF32-o54pboGqH1iX4Ef090K-ZIv2psY2wzcK_kFDF5iX7rJ79CXi_uTFtH2mGq6Oiim8mz5bz26d0H_1PiMl278LEf9xGsNuO3hqqfSWg=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGi-CO7yxHDoR6SR_qt0i2y19125HUxhzEhBVWhQSIRd_FMGm9fZa3qag3LeqS1w5t9FJN6htHa-OQCEF4fZJzcV4XCcKOK7cztyhQCS-znqujrmQZmz-0dmPGFdXHGYBNd_HnaJgp-rs16Vznnx0dSZl1E-DdFegmTUCeACwWc9fi6TNfqKikW8ro=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGnCrQ4WGElV501AV6XH92ZWs0ZboCLjzUtK1-LWAZAHxoqrSctLjEnm4QsPzyjm7EngBwxLSXAOKNWwuUBw1o_w9tGYFwPTn_-T_QvOgZd-XkxC57rNFKt0TM2F5vM-xKIYKx_HpW3cAPAT8S0N_HD5TvXu-pKB8BrL231M8lDI56Chrv2UyLR9rC4LsL-k3Ya1Kp05A==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGxtYLuUCEqq4gwClNz0Wriz3S3aRxRu-kzxdQ2YWkoyG6MyQRkYAgibWBIdqC1KYUCJichfwfQoB74Y_txP-pclZ5ZBgmAWFq_5-pqqRYu_8V82IFnzKz4jvNRPjklsDPBeFc4VnZWt2bEi8c0QcnA7dkSjaPCgv21-qoUuiQQi9Bj6VZqnq15pKo9Lj7BoX6p2SZZcw6_IgxmyLxRlwU-KdRfUs50sp2e02WhwvOfyCc=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH1L0X3oIRyMqiDkQNeiDuA9tNXhCNICq4H6A1IiTmFamxJ8EifgEBTRjCmqafDGINE77FoZcYzKJatFizjCNW9kDdfYEkNqBk8ddU9haWvCOSxT8uxzgeZ8pA-HMOCfq-6S1iEIBDdlczfyBARP2WKECg3AQNfQD4lsuQsyQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH2OUTyFrSaFrn4KMjGWRvrR61kmvgzMYPjHDWL35WgC_kIAL0N5zHlfLWxBQnNvOG4-mgRqZl52llHdluTmSGeX9pnkJSJs5Bdzc0KrEnBMBDem4s4aCm1-3dnJdqJlF01jRMJ8Rfr6flPNqLuhrEKBCciBaK53QuuKr8sPVJ8sFT0IZSofQGN6-PGCcSWrcOxRetvLOEj
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH63EGejYetvK3Nici_6sZtJfiCwVm7mm27hRF2H4hKywk26Mzw6n7Wgkh9PIu4erohGzdFRbnNvQkvv6PqZHJ_EDW9jzIvd4dBL0itMhxVCD-Ph31XbP0Q6zSGrIRqwYA=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH7UXMXNrLexEgbPNkN4zUhVtkGkIxP6coogj1mYlkKqP5zoyo_dlu3hZb3uBrr5uE5c9PrcaH1B9w6ldntxrNXYuan3XcLn1nVyTVlryIImvGFtifYrQBH8Pn_h-wd2nw=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH8aRADfCt7T4zhOFmy4RNnUseIbML8isaNv4TRddpcrjrkP6ywWjVCTYmFNDQ059UCLmpTACnM--U3WRMNey2gRyWwSIXItAF_YH4C3X2fCVe3RjfUnmFMpnJKMsrnpmUh4t7QpmgmPdv6F5sVRW7qxKDRYTrDvDKhhsx04IVb7wE_HUU8YjKcmVHOqx_V9CguOw==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHRoo4fWmAwK9ha8cKYPK0zqiGMu5YDq63vvfSGT-N3yKFgSIhqguDpiAjiktQSYdw1GG1BUEaySW9oFj_NMx69TucIj-3CAqjKwjU8LHCTJbsBmBs4LHn87Uu8Nd38Ftw5J-zo2BRyEklIQKA1rROmGDPSVcbiROPL3C7PHpzZin4VjZ1DDXfW55HFyws1DVuo
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHUOF88n0K4JvRi9mU3hYQwI38ss4rmUH1R4_ri2XzObOo2Gj8EBFRnPpdWMd1pD0g1Ob5-DWdVrxES4_6Owf7ckK7rDxdGSO_rbTMHf8INhAjH51z5YldL74y1o9auhQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHdHU-e2F6_TBrKHy2w4dzDcVGQ5ygf6_plSetsBeV2k-WjRjRhK3jhTDCyd9jppK_xhbGppLdiZZd927GzauLV-vm6QAwwk4UUmIVZyPNi5XMr_JZceOfkPVVt0UCBNETLeZd831WXTdAZ_DtygjFCziEN3LAe
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHvHQQSXTxyGfATmbkCnhTwrVsBn6kqCllUNXYQsbyP-JpLBTJ3LQ0pw_dzePd5eAuBWQgc5OiBmqOp6pOJhiDVEymcGhNbLy63gB0EKJy50nOmGdpTNlga_DTm3-kYCkFg2cmn-XqW_j8WoIVGu3zobczbBzCv-BvhJRXVsiZmqmzS5AcSSO8FT2cwTl9bwHbRzJArlQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHvLSuJWUMpac4rBBQd9QstFUHc62xmCXJxRlzKfSZ7pzACzgTWDhoKeAadEJ71QEMGk5yy25OhyBD29mBVxDIMcJ3cbfa8CVUkS5XmFcFxuZkdWU7kRQIFhRjzTKvgPvSBteugOwx9orFPw7wLfJbiHUHP-QtCa2Nf0B-68j9p3e-UK5m0Ul8=</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>BT-384</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>advertising</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Assorted vintage advertising pinback buttons, commemorative medals (including 1962 Rock Island Arsenal Centennial), enameled lapel pins, tokens, and a pocket watch inside an El Producto cigar box, mid-20th century.: 1962 Rock Island Arsenal Centennial medal in 2x2 holder, Vintage pocket watch with aged dial, Advertising pinback buttons (Gold Miller, Safety First, Oakland), Enameled lapel pins and ribbon badges, Local Illinois tokens and tags</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>$15-$65</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>5</v>
+      </c>
+      <c r="F26" t="n">
+        <v>5</v>
+      </c>
+      <c r="G26" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="H26" t="n">
+        <v>1</v>
+      </c>
+      <c r="I26" t="n">
+        <v>5</v>
+      </c>
+      <c r="J26" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-SEND</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>grounded_search</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEHiSB3t7gsB9ezvS2cJqlB1Y2wY5SLNk0ujudJWjB7auP49Jx5ktw1Eg-GfjCq3Z5oi4Wz9vX37vgZuEtZS4GoCGkmuQ4XuSeDsoBdAvtSwODMQl4xBHV--sRTOGhUVd71ZJbwQs-NHwiorp4Y0y_KEV6UyexGsahp1bfN8UfHVzoGFJaq
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEfUr1QTkSzTCrtcyXVD-cqhyCTwmNpBUL0iPnkZok8KIhh-s5bcMaMH34rIZJkP9HuvSZxdOwqMn-X0_GtUaEioaOT1hHaD3io4CnkyJtP2Np6yj8iCpOge6Xv2fglH2dOHz8P2nYjvfoa81oljivHtQk9t0tjfUxt
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEnmh-XFoL6ilyeXhFRQ4dw0y7MhN-4VpthGIIu5eX8oxddAQsX7cEeSX0nCRCcoCcJxk1bKDX16_oVNs9TqREQMY4xk5O1C38LrcoNUD7vanV1sAgxsJfev-qifewy6aU=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEshLr0bOv1XSuh0chM8jgLo4NjGwFxf_NYlQrkGyDhJeZ3LQyKPZFyCVkazru3BycC6kzp7uuKej4V9ZMPI9PH5r9FE_6gU1fq_Ubgb4w9Ghh_l35OrKxBvFMT25Z55j8=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQF2zUpNAj8zZFWDqmSw2EkJJDe7Z8_xEmjR3exIl691bNZEV3_aXgp5VgGB9t7ld6GZczsZ1Zao6fc25g9s97DLHHVsTj126kH53SD9WQmT_ybe9YiTXkKC3nDMwUZV1kCQ9RHwmS0GEp6MhYESYDJG7XmU9opfSMBLt7DYg5m6vqWASeI3w6nR1Ltv5ZaCwLkv7s2PAyELnaK3OOeVli1F
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFQM70DPvYUeNVVlNZnxSS1UXLmR5-xOhtO41wHpdOGKUiy9r6ZwE5BgFH8D82EG2t2FV3AEp2ERjSGBHecTRM9WBN9AsxQP_tW6b6bZYUsUu8eRr4DnJ4-egs5F-u1LsD8nrcqBbQP0auPTzvsQsB-e_hNS6cGV9yjuqr_xYa7ZkaxVdGGLdrP8xjenQFnnn6hOixkAC873qk1IExweInc
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFbSyCgr67c4OHkj_Wu-UoNhXFxJdKWzoLKNkm7ALFcHtZh9Fx3HLHKIF2VeJyPylmCvfDgxWbx9ta4gtnM2J0nIIjRr-0GqC6tW1NeUaI0VlllTb_cTCMm-6T86YmvqCQw32ICghoe
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFs3fI-vxQ_Xg7pWl8D6Nf5WuMj5c9n063KC5owko6dzEqim_V9T5XFPOr5trm84H55XGEsmPuv5RSjtaGAW-6Wt_cgUFCI6rNOvW9s_Q6VpFSNy-y9BjOph1fFcDq2tEY=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQG-vDaTtBsqSHsIBpj9rYkg8t69KghdwaV8uU6fj-ffIvXlgYBldAvIHY1jAV3lv9iW0u_WIKQ05fzfJZQqcIzXJKpDGa5-a1alTNURL3gHaK-BSEf5lA_RyaCQcHasrSwb8gvYp4m5JvpFxuZamQWTIPxC-c8HPmfuEAFr1YVoSMpDhVOSdmmIHjGJMKWDCWe35rOvZq10APY1Dl01kLAv1lbUDtO9_-9cD_dYTPVXXlA=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGDsLY1GG5l4ILelXn_KGpCqT1rI-OoxPrq5M8_9CP7Sar_T6D8u9O2zUAG0dXH2Qsxt2lnLGql6bXfKBU_cfVdqhO2JhPL5rgX6n4VuF0kstQGywZtmW7R7uBilg57_dI=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQG_clKVFUftPJhid7UPEPqVkSG9Kss9mMVl2kk4Inq4HceozcarK0QFwG6jOf09TXewN_HwYRJU5xyFgepdsTn23sMdLuanHywuurABEv2stB5vKPVfo7hiPmZrTClGIWQVKGOXlmRrykd-65GBYSiCa7ZowC_6gAemP_4wp_xZnfB7vLei
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGsmbHTqPeLmMEWs9ozOf577pK8pYS2tk4DMWWVdvUqipS7b7mTEggDL81frmzPff7qSF4j5v5YWt9J0B5jI-oPAif5hFaAPFTYZp1Drjr4afCzAxXyZw5NZrsm1drkDrZZ4qyMrTQVwE_-ftMRMph9x7OUxNWN6aRixoCj1JtHzbiHGmZTH_z5s90NWccjWT9Nog_ovTBXHPfbiIkToPR7
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHghfUv1BByLZQmsXF25eLT5ylDPQs1yODMLDu-XgblU4JoxFENuVlcjykffkGeKkWGab6bCDlwLQeCfLMrCUUWXNMZ4VDDoat3052OU1H4hN6l24fVii6xCI2h1DHx5WB2xjMDXW7aZUeTmV4dZojsTJrV94oYe82tT2SbguO123lP</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>BT-388</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>advertising</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Cast iron oval relief plaque depicting a striding male figure in top hat and coat, likely an advertising sign or promotional plaque (possibly Johnnie Walker or similar motif), mid-20th century</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>$25-$95</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>5</v>
+      </c>
+      <c r="F27" t="n">
+        <v>5</v>
+      </c>
+      <c r="G27" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="H27" t="n">
+        <v>1</v>
+      </c>
+      <c r="I27" t="n">
+        <v>5</v>
+      </c>
+      <c r="J27" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-SEND</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>grounded_search</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQE32pYrj_NR-mwFZb3apWi_2drpQiGC0ZD5_ZMK4pzCSLvyBg7KjX993z_tT0E473axrR2rV4JT--RU9DuhfxW0NN_ahkKyNaCpbI-5BrWerjGt2QZTCabDrFnuYgoWMcjtOEb3hc3wFrkWc4ciktbVw4i5_o50xW3ZdBm1S5ev-7AKgPQLi9JRECD-FuiiP7Rd-j6gFTj60gcUoRCDzJ5hTXJVzOEfI0q_GuGdVOT3ldhveRw=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEEqMCvsB6CAMGedsCMU3OpDWIqLRr-NpAEMlpRs0x291ZugCotzROncqtxhmiyorVBq4ckSRx8n6SUPPEL_vBOXI9FcBC2qQ5rXdc4DXyxTFA6Uq_keZwLgSY9L3qQjVSSVQUzyiV0f1vQVpFb
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEJlnrbE9IpLX_hzk96i5l5dOKFv1tmZJXSy-O46B6JD1Zh6k-8E9GbgGkTR5sak-f2LMBi01T2k9xvx_3LRbrhesimlynuZfgXFFhjHFQWH9xpbOGODmFdmz5hfGfi9OsUsOxVX0AA
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEs9aF1GIGLOBzfCszGB-Jw_Uo-6kRkD-KxZ3lbZrCvmnv3wc_cmT_Op7v_BNj5rK_r1b26MRrGBufYtpZ7v_a6KFMgDIkVWKk9GaeQuXhMU-tgZRK84_8FinJuQNhB6ZP1ueAGCbITgUqZyDiWN7VYLgVccsrhj8dHLZBOU4RmlKoeXcZAj9zjZfMzdvLr5XDwQg4cY_1yHDU=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEynRQLQ_CP3k3kWMaztspymnWPtHdmUafXbSaTRnAESRXpQTw5vHFFsCzPiqPi8J7Q9IyhLkgGTI7C2ibVjP0Y2dm1PRCYHgksDzucF6x1MUX_76nrjafWdfVhvAcpOuvZeCkyT-iP-dqKls800bYz2iO_owDHUk7YDsQ=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQF8_kKXGKCfAFGmeaesO3oe_Gpx8F-o3eMZQX2kVKzr3tJynNw106qIVZq7zIMsOaaPUiPZQem6UY8_iS2WOPScCdyRu-TwRYwWjWNs1lAj7HZgWpVM3VKlS7Uv2V0m0MiAUpGQtccTBS41II8BH3HriA==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFj_wwBnYaxXbD9pnlyE6ceheqielxLOARVrh32ewZ4SA1wVjJEwrMd8UveMomOzbc2Kkci53bB0ic7y1PPZykxpjZMHVV3vkW6xya8XYQ48tebm0T4BmLN-AtffzsSgrlwKrfsT0jHNMlszFq3_5CYDDswQAefxvmQiw==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFwcfy7GUpH7yyybiEhCJuzXwibL0pLkBWJ5-tCPwjXLZTZXMJnBtCDRR02D-1gjJQI7XhE-MMmISDK6EeCgGYtDM5gDiUQ4vNG6mBI7iFzcV2c0mcQsx0SdNtt7OSHnvLN9P_34WAkJnkm199YLQEjJHl40tSU2pfXDXAlsLswGPMD0EHiSBmUmQbr3DFRCGp7A0CTg6Oe1C5_l7QKhykhjHBwhq6UxJoJOTQsM-AvOQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGa0Ru0UtRmNGzc2NLNwfb8pOsNVwR1vaGXX8Z6HZSRbmm52cyVNzp2HBUG90zy9nhbCLyw73kcs097ifoF9jyJ73WT6H30AOz1VEfMKEHVf8Hh-f_x4j86uuwyi1oRZBVe
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH2sOdDx-zz1dy56etz9m_oLDOgj5N365eCln1IgjwCjBpNeSl6neBRPhGDKi0L2fZ1bTtVamJCaF7sRtKmYHFkFDDobZIfbG4JMEXNxCCtLaYmOFAf79RIjE8AJHZxyPvTxTDuFd452LtD-A-Fj7rH8xyM3xXL0KR6Ps8qmmh7chJ5F2b3_i_YXj9hdtk1qJYqOwN4nXhYT7o=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHtGjkLC8caiMHBNmtcur0xOxk4rseXmStBRDb142_6dwKsK4ei5Fqa657Jp1N15klpTobpTLV0pJe_41Cs98zWMIoIUWRYnJa9Y-MpG0BnQOc4ysVTMBxU3T7ls770aN3nx6Ymtc3CrJ7VHrvtoHBb_C0q_yAClOTNYtQccJKtMAc=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHt_F48RNZxiRhE9SycEMLEuz39b2RGo4ymaJqdX03IZ2onGvH9wMnw7hy-2ALklxogISbX83rQpg0loXNVDIhtRrEu9atLBBPojufAmY8LbSCdTe_vocOgJDQFkaD5p7SLwl7gFUnIcZ3zcvwWwxSU_2HEyC2v8Kh896QBk3WBvIDabJjiPxqYX_077Xwmyyax_g==</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>BT-394</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>vintage toys</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Vintage novelty toy and ephemera box lot including packaged balsa wood plane kit, red plastic rocket/bomb toy, plastic figures, and vintage crayon box: Packaged balsa wood toy kit, Translucent red plastic bomb/rocket toy, Pink molded plastic novelty figure, Molded white plastic figures, Vintage box of wax crayons, Assorted small novelty items and paper novelties</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>$15-$45</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>5</v>
+      </c>
+      <c r="F28" t="n">
+        <v>5</v>
+      </c>
+      <c r="G28" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="H28" t="n">
+        <v>1</v>
+      </c>
+      <c r="I28" t="n">
+        <v>5</v>
+      </c>
+      <c r="J28" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-SEND</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>grounded_search</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEWSUA0oyTsunRwSsVhROdMbk8BfmLfJDh3L7dGT1IEgfKow_-3R6b1IGVzmMJKxzdW86wYfQ_D3quZHv33XwpFNlnM_zsy5EeHrwI3xfNC9z4tTgbeBrIhS-meP8x08XdtvHMhdqwtYg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEq8O6WRr95ssdi2hzaeWI5PISHHUHFM8F9lDMftXAP-btIIqiSJYD1wn7lZdZdzJWiCuS5tDBshxYgY-7muagul6ao3cWmC4jbbwa3BLwEgdmLDnwQ905pl4IY-gD5rOulTvx4amr2Owp_k5AqrSXaa0Nl5Adum40vOlKiOjnxknULEw==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFBji8nveUp8r5OSOtFcshvpbqBuLHKvYjb6ScSwfEeIUyhlhBuQBnL1_0oc01pzZIlugRpe5NJFv-9dlFU_0t2LNob5xBAa5UMVFmk7j6OpVVv0godKOD__XTv1lSCdWM--pihgd4gbSasmJfKH78UI0yI1LOzC3lyJIb_xUjRdAM3tBIXznMjDx_5o6PFsBqfJsmCUMYrxJ-pqM23kRpWlLeWhjX0S1UnRx1MEA9GnoTsVpi11x36oBzxqgJ5p_I=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFWEQGPUCpUWz372xM9rUJbGoGm-YOMlYlP2L6SfZw3fpyuVyvIPJcKFNDdWJYi3vpoJXQQwNjZgPn6xzyhfTDqf5UeXLYtBAPX0kB3AYK0kEcse17o-GTQMz9SahArNMCpWKL31ECwkBMy3g==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFXwhe4K5b-Whz_hJ1_Mr2jUDjE81S_OtKryKfDJrrOkoxPuw78iilIlShh_pssXxt1ycrkyQqdmNp5qoQFAQcOvTdxJFVuX7fqBwJg8G8t5gXCPizcbSu5XjH59pfFfyNfaoep9aosLwfI3oGjK4o119_V_havNkf4mt292EkevxA=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFZroNMdhfBNTttW18_IBA7RcRffkrx1czdjzjV3mrWzTyHww7vRmq8MDXaBdorcIXnrGaQUTMBKcsY9M_y7c52V8_Y0-qHDc4tbFYZl4cSifh5L2ioIkGLIHPhJldg7As6PxyxxdP8wPL1OMxz0BgOH-aM8vSq
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFeNwC2gFQ2hccFmpdppdyAULVpC797_c3oCRFdvn5_XiCj0C2eD9WAX4xna5ySiKYgAZvwdyMj_AMGv23gjjAp7SOcIckF0nKJGVv9PB876jSOn8VbbWMrR9v1lZfJDOrr1iTze41JOgk4CuAwzcpdVRa5ZshfValtsw9f_leRyBNdNw==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQG9adWcz_JdOrzb84FqZGXz5QYZ_Hf18Lc-9orpOzvJImcMcdecCpt8TvBmk5HthT9v37CBLv9P1K44tAOgXo4Qte7nje4VKrwxB_LenF5-eCBkQC2jhvyc5UD1Ejdp_UHfgdJjKdt2jkEcWh33Z7x9rAk6TdTBx20DK7I=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGBE7Ud7ChszK25c0g7hQjG8FA5ktw1m1uPFiJjjAsVTFJZFZdAwMu_a8DKZDzNM-u0BmCL1zn_qkyNQJRbEKT4eRT3CSLMEFF_varWEh5H7oPHuyQsoy-prEWRLoPPLncMeXXB9cWjBX035BxA5nw4lNDVjj0l-kiyOkRl3GtXRr8=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGDV5FF1QLF3kYwNCYDtK6Xf5P6DS4PiZUTyfJ_xpS65QrCK3hv5xImTL9rA9i74tyDdDSBckyweOd4f2NmIDgXyau0sTGnh88QiBrXpS0M4HKPjmj-ytNOmZ2KvY3JEarxQ9xEAPxNF-MLelkyzkF82ak50sM1M3Ox5Os4c_n-dRCdsuqdVwOR0c2313bc
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQG_1s_4-3mIrigw1_VcwKd5i10izhQufSGStvEKriPCQdoBPNXfQDQQ3yVl0OF-7mbLW4NnzOmHhcg1H9HEE_XIp_8ojqynmS83I0eWlFfNHEZEk81Rm0I7b-ttVuqDSc8TQSr07V7cpw==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGrVszuOnWvlUFt3WLgH11vsRbQstA1THr5IVdgFAs4jQgvSPpFiZJ19WblbL2qOOrJWhFCW5CZTrfXPVynBcDWuFR210IE71C_lRnOF00GwVBrRRRVODxo5Wv4BPymAPnT7e7YRvvt1DnLb-McRs_Jl8WxWnYVhPhVditdk46UVvLiZQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH264JODjm3TG4fThumkn55tQDfJyCktRddXsc2d6YfwZB0px8GdL8bFkX8vt_Za8u3TGcU_9OxGMt2xvscFOohZVAtNzk96yJydmhFk-SasZ-SzWDpJYSj_HcBMaCM-BqHkJZqrTyJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>BT-398</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>advertising</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Box lot of mid-20th century paper ephemera including 1950s Profitable Hobbies magazines, Sylvania Electric promotional game booklet, United States Athletic Company baseball scorebook, and vintage greeting cards.: United States Athletic Company Official Baseball Score Book, Sylvania Electric 'Beat the Clock' Party Game booklet, Profitable Hobbies magazines (1950), Vintage die-cut and novelty greeting cards</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>$15-$50</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>5</v>
+      </c>
+      <c r="F29" t="n">
+        <v>5</v>
+      </c>
+      <c r="G29" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="H29" t="n">
+        <v>1</v>
+      </c>
+      <c r="I29" t="n">
+        <v>5</v>
+      </c>
+      <c r="J29" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-SEND</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>grounded_search</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEbJy2cWVo4yreNbuKGa_52zCExpKBpanK1SPUNstLA8hPwTlyRWM3lm_cYULhFwsY1IcQA5IiRXtjUnl-yeBT7Eee_wE1BSgWw75XVns7Bo2erjI5f1lf5ivdU_3U6x7y5h89Fzt4qwioNEM3lVnlZWisRZdJsstaE2NbM-whjeQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEoR94dqQ8ZLxBw0K2YTjqBiHApkEt9OGC9gyDlPy-6OPOSfUtyaRErOLFcqViuTgn4fWJfw8cxGHprRNILiF8h5mdZZcKBi5t8k4-9tK2PBmxC0L30e3q-WuwVBqg1YAvheHeM518ALkKuZo48BzTNLtI7X3NmEAtEiVA=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEz6iAN-1gE5ebOhcYJwEfalG3Jo30ellhhgDj31_2Bf036kb9szxHGUCYCrA7DXxFXJbtEOwff7k7LsdrrCjz0rFFJnFhU61cwFm6R5jFpv6paO9iFs5_sb9Rb1Ks5Ggw=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQF3qhAIXSQlNMhom_0fmOyfSz9mGenxNk4QU4ELuLA9H7EwZ-cjdN5flkoZ5CswNfcstsh0-HbtpVhg9Nswi7vW-WrUIGOmBLw0g6Vg9k0RRP-ZL-Nu2y0oknBb4cNasCLEuDfCzeMszBEzEXp3L9FcC2NI2Q1YeMqZnrpJA__qlRX7DQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFCc_aCwNDY-jI5PN4jcRM0Y1JHFPtcqPQEVoNDsKgf8DZTiyI3fFI-K3uex_t18hCjHYpRfeiXjqsKFXOUGc6qgvWcd0PTrCcpcxPYCQ1-shkKKF0BWgSQngkXGzX0uxg=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFH77FoS0o1x4Iphne0wAIvskjjCDOOEJtw1C8ZCiPWhUBYSfgE5gbTHwao3NistOVrWd7gRq7izsNLUzaCznuMuuW5sORhaxLleIu2krS8MtxnhzZBxO8JU31WdXhj4zTC1gj5bHMfQg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFK_Z4J0ultM9e7YX0XzCHBfzSBOGUawdxOYihURy35blQ9xQzw5UXqvHjry8J7ig-n2g_1_0JwAg1FlUMKFy4oWevqYlFfFjBgvXXtQP0BeNPypSu9hNHOnr6x1NVANPt4KnQJjnw_hbutPg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFNDKzDkAR-JDMU665N5LNDW1akRS-MwXVIe0Hp4_WzNFN-4dLBTd9wHjp8NnpEBACZgTM7ALmQ5Rh78d0-X5BULZHuHYPaa7DwCxWhr6JTqKkZj_6hTWqRV06S1Ntbn1k=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFWmwHCnsuzpMhPw1vtdK5ItWsmuvIeiTzECNhytOxWkvg46Kj9DKcaFQhcacSi7uBcBlrlDdweSC0aufQNTucz_t4Qr4t7ZtdT0-tSeGqZpOtnOLVcOi8aZUiFHDA7VbtHHRKTUWKixTOoYN1wRq7BShcPb5WUyGwqirp1KGc62mMBhdB_4fKP
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFtwdpfTAjL5zJVbVNEDizd242r0_TpbNc3_8Jejg7D2EyjySesxf4xGS_iNMQjpkyfl9b7rnZThVzMtriXkCu-jaNcuJ4ZdWJhqwwDf7Zw2U5lAUYqaYyiYspYCAC2m7A43rvosq1UEuz1cgOpY2WGmsB6Hr8_SsmVaRUc1Lf6JXxbjeP2VqR4j18=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGM_crNWEaDlX8vz1GE3rkUFwIlLSfL_sJMJi-XCe8nLN58ybYV3CAgvZi97_sbgYHhPfSi6nFR0MroomoJ_ePiGMGiL7ksDwiGy72EC4LHEkXwJ0UE-149G8c4Wspqpe2T-iyupj3K7PHCKV2POsVX1dDDF2g=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGuIV9HjYqzmGtydilfTcFzqdFmjefVBSv1s50TjAD9oYVPC2cVpUS8fNGXp-mLi95b2qUCWnmtSvpaL_gtL8sqoYg2RwC45pSn8--EJD9ENsTz8_if1OWMQxnrI5UuMMmqhhELYje3TwA1xpeX5FvP3MCIgnjHrbY=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH6nw13vMFiwNSJ_r9IQlFDDkRRzQ1rQY1gK_oR3oq_-drwH1FcBYuYQ-T3FntqIZfQ2aVzxoSI4H03HZeQHhQrX-akLWsxS_G0zlWD0CuXElDug-Y1WPkw4qrlgaSIvaA=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHmyKSepwkr-miHQGYoVp1wJ3YbNoqZMW6lA1cx3vtT8wLW7SSlfBeHD7B4JPESmMMaqfqiEsXY4qgrDdIZEtUsUgienfaIOqMN0JnSmyx2Wzxskytqi1C7MUzb6zvEtz8L3cjdI6_D_24IV1sBKCGR9JIuFWeiZ5qLJqUwapiYSmlrrU5ob-B2yg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHxohuhPI5ZwYryBgGeRX_ZyVyebRceZtmWkH2ZnUqxqiUZiUuqhVfTdKIi_2wjXqSJLHDKbS8oIRNrVQ-HCnrxmmVYTIwpya9aCCGbUmJCuZTU19tVCUVnIBzXKim-K-PnKM6P7V3Fkqaa1JOFXvDXFB3gQPyFUw_6IGwouixoVufbC3NUgpBPqg==</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>BT-404</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>vintage toys</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Flat box of vintage sports memorabilia, ephemera, and trading cards, including a Rod Carew Popsicle cutout, Minnesota North Stars patch, and Miller High Life Braves booklet, c. 1970s-1990s.: Rod Carew Popsicle collection glove cutout, Minnesota North Stars patch, Miller High Life Root 'Em Braves booklet, Wilson Super Bowl booklet, Champion Spark Plugs emblem patch, Sleeved sports trading cards</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>$25-$65</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>5</v>
+      </c>
+      <c r="F30" t="n">
+        <v>5</v>
+      </c>
+      <c r="G30" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="H30" t="n">
+        <v>1</v>
+      </c>
+      <c r="I30" t="n">
+        <v>5</v>
+      </c>
+      <c r="J30" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-SEND</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>grounded_search</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEHcNBOra7GbtVRc1bT8iE2oZnIXKTcBkL1Klnz9IKDJ1W7bCXOjYrCoVRDr9763UuYairHQQTuaeVKE9dpu6-sM3UwrNpPSUGTOwBZxQfWqGExE2lXL2XcHcSwf9Bu4A==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEVs5ONHlXtq649RyI0EQuDSmZtfZrKHisxPKy_d36cAit_L90ArxrWXhgXAv55GJl19XXRrH59m6HCEGCRoAu0qTy_Q818cDCRDtSN4n-dG3_iUHW3s4Mty7CA5XUbvZojo3YRKL2LIuWLhASzj2lN3zbSoBHyBR4ifUXOuioAayZ8TCB9hSkT9e15t_1XsjqfpwEU_9cZ4LN7x3QZkg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEa3JnQDEhBY3EnjI2SQa1g8fI1NcDz6-TI0-684d9UjRoloFk8YmiEcNGArYe6r9MxUxxdyDtJchn_weszLLLDEEcsOrBHZFhYKWB-N62VhVI2zLmxfwtwpWZeBguk1FQ=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQF7KRrlUl_O4C-APIT4J0NvlY21hXEN5V-9rfekdWmxXGj-ISTKE4-PSM2vIZRGoJ824xDOP3NIW8XU8Y1IzHv-yTgtRXuXV7zxo5n0Rs8UJwZ4E7obtnUXFh_H4zI5fisnO0IluC84OlYRGOY_Xt0KAXIqQ4N3of3d1JaPFpRUE1SFAqE_ROK6owhCPzA8OfQorjewSgM=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQG4JlnRyHUvLbueGBm5dPcMEwpBaT3Z77ff6TFJobgRJzvMFEdR8JgiqKrOBr9m862IOccrQowCwAoAeGUAlZ5UuMwp49JEIe-vbcsrEvClG74zqN3nRZn6ryzL54P5Og==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGEup01wAAQUBG81iB41np2h1jc8i2urbY1WhVgaoumGfkUu2HN1TJa9flVhlJBLjr_ACQtsHt0wIAs6cSwG5nENX4m6377R92kbuhy_0EBVy5eZscKS-wQSYMcSaYxq7W0Qx4QTr4q8w==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGNf68tc4KGBCi_TZ_zHd8V1qWhgBDVOOsw7vAcYFR1lZEyLBdVo_4wIODYRn8R0-hzGKg4rXvEibZqdCAG58OBZ6Y8Bb4o2G9UUtB2fA4xwQyELBPTwuwolIpMhviqiNXlNAbo77l2d1CSyAFgpe-jITqlaSaX5ouLEB052fozaAbyAA==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGWo9eHqbhzA2kEDFD6Pw_rw5tWHw4I7ol98Nxl71kkVlkHqZCq8pNZKAae_aDYuJKUjHjGtanhgEwtEbFx7-UQNIK_qAY99Q8mGapFGU4by-rqpHKAzcCsc8OHRZn_ov_kjEHE8OsxLWMAU6U8EpJCK--rSM2_RapQFCZ5_ef0QoGl4tuzXVz-Zyw=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQG__hSB6xxLvKZ9nhdFOkn5EOD6Kus-v-Smi9mYiQCtshPPGgPydLuFCoY9BCgxMs58Vkzgcn3SRDdTgmVJl-ICkgPnn5tA8_MAOPECEZGhWG9HHVwxBVpnj8AoyT-h1EE=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGaK0HLAl9Csoq7ZzStcUz0sy4mhkAu5Q-BO30IaqW6ajGySsak18-46Q_dITyQ9pZzYJhhxahumIqZ_xMJOgTw5bhE8-pe-4GDgIjTewSMSEB9uKo_gOuhlIxx_kAQ5Mrp4L-5Sv_cLOJsWCcq2PvugfjeV-nh3DvlIu4iVSvS9TyPcA==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGy8KHwUmoHZvwYsP9meDUMjaZg1X1bvGYNv3hiuWmLHv7Lb5hfdD3b5ENbsvjHyNONIbCwKXVv4FZwpS83DKhFIq3SfF6PUUlIx6cV-Yt4uhs2YVJVXRaMC0RlGcHV5uADBx6dI6Vo1XN14fBB1v7AE_Eu31H1kbAL8Q==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHIe9zc3FnQ3KbtpHF1Zd7wCHbRqPq2v9lbhe9oyRvM2K3Xs_1YUz-_s0G0rA8j_a9eQgBp1sgI5lFYTbMALyzdvlzjb3O2LhUmi8adrQZYDGH7LwCx1nEtSxjNiDOcu0epIxgbAUbtOIFSdRMgJmWOEq-vIjbCr7U=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHMBMZLz4QqfhlJXBZhV2-Vfov7C-dCBxSEUgq9HtJWXTfnhT1cZT4TQ3koKDADBoss4_RSpi6tNUOrx7bIPHXXv1DxnjhT66tDCQ_MaMGoFBW_9yeOOZGvVdiC1DtEIww=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHRhSlk5VlsqKKnmkEImQRvX_8EjSzzph1DOQpCXYO_fHDTxbEek_-ZxYzw4vHVHPJcZdC9q7uw12r0VNwQwC9Pbcy_IF6BgUNPisdvrz6Ssf_aeoghv2fBkJvo_H3gGsexzEcoizMP5Vjt
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHWkcYwgat4e52efa_CHpPpJdFsnrhzWXv-AV394wBtfLdNiZ6yR70AA9zC9IbyK-9SRjlf5fhgksXWZ4L7ZLQq60e3UGsfI7uSgGqvfaOSCoSu-dZX_p1x9cGDBviRFQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHxcWZk81u0md5K3RAHW7B1YKk2Aj4m4RbxyqUWvCOJsR37fzyylq-mJx-41qFNqcdReeDcWpNGMtmhWYTJOQMuZSg3kFMCjorMZ4VS_I-ax79fqFp62I8gLs0oaK047jg5IQDqRX29hOSgicLPli3HmNtG3tCrCMboIp9CiXuCBpKcLY2iw-2M</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>BT-441</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>vintage toys</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Barbie doll in winter ensemble (patterned coat with black faux fur trim, red pants, black boots, hat) accompanied by Hallmark Barbie ephemera and a 2001 Hallmark Keepsake Ornaments Dream Book, c. 1990s-2001: Barbie fashion doll in winter outfit, Hallmark Keepsake Ornaments 2001 Dream Book, Hallmark Barbie printed ephemera</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>$15-$35</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>5</v>
+      </c>
+      <c r="F31" t="n">
+        <v>5</v>
+      </c>
+      <c r="G31" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="H31" t="n">
+        <v>1</v>
+      </c>
+      <c r="I31" t="n">
+        <v>5</v>
+      </c>
+      <c r="J31" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-SEND</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>grounded_search</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEZHc-Z59HuEH9ea273BYgPy0cG8-gvWo0AqXUrkaYFD_rysN-GwUmeWyoq-Q4hyzk1s9fJqYpgdUFbZrsTs_OIn6hGs4xFqSiXzRFTKmxFVr7COqGP-Gqz7Lys8pfn-82PJ7Ee6vMMSw==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEbHQetiGlAVvR6rdK4tz21eXqMv-rAVmPdUJlYf47P-_LDx-_yLVT4HaTC8s8gunORzZhyu6PTIHNPNJ1-3cHZI8IXQASwhtUu039xI3XoYhQQDBFcYbsU-rhrjYDyGbxjjkFslLLjfn21OML4fdUKPpMq-delWw==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEwioSu2t5xK5lntNEQNtt_LPxatYy846tiJobRhZ4kZJ8Vm26xrY3IuKGsu13j44qIosd7aNFyD6AXiyW-0eciIvSmEYDp3noezfXDVZPI7exbmYGLC1MQYrTqsphj4Zk=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFKTQGorVryiBkZy23SvtyVWuzSLAiminRScM5wAoAnAVOK42BxnjodbwEmUsgBecQ53ju8djTFWVW9RtXfh90iHZFNXsBIrREff4-ctdI9iaQQL-46Kgz-E4WmypbMa9LJBRi1vgDYVQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQG9BKfHnQjczBreIdVMXTPkpl7dMOj2hAVY_lX39PEMofhmmgQ2aUmQbIc2MHIoiHoj52CdX0ygxlixxxtlic2IElLw3zzLyUFb0ezVJ1VtkCWy5az6zvzkBk-CFPnao6w40qaupUsNRvQ=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGU_aiQEG9pOExRakK5q86cn-g9-L7tUQihtViVV10KOS2D42wkRSxOMxwU1kRPNRpIKr1Fn2nhAbv9ebI4_5OS_-6f-tKIQRC5OumgU0QMCxtj0qLttjPthhpwB-Dj2TMLR3InGo7R
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGVbGpMatJMe1aePeqGX7j4VxATxVVt3ww9yk46luGJnwoniOuELy0385FDO6fmU4ZO2ZuqC0dtNvJcjS85LgoFElO9PAoxkhinfRWe_qYfUie8dEO30v7VaiEeXlnl0g==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGpprghtWlnfKqchERsgDDiOFMxjmbqWUHoa_Rn1uBIzfChthh2MvM0GdOVYMyrekLXUeBKRMuUyZO6GuNm-oB8nNZFsQXQMCqEPX79ePAa4EJFu0iG8giDPYa1jW9DPPjWAQjAi0oQJlNnOt9E8pwQ7JyfP8JPx_by9ms=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGxC9X9r3l-KuH3ljYx8Zln8kKayUuckE8u5Xlh3BTnLAJTmG-ZtNG_SiSWGybLWk3C-5jLd6nbJW3oharIfG6zRvS9bnRJawjkIIcmSCVTs1uR1OJLHQ9Rr-2H7Q==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH20luUcPSkEdr1UFs7tihRuBs0wrPtPSb_8frZ8P8E-k3QUeCGxk7xsLEjAXFfcr87hTqRg_UAZaLJ6zPpVHBqVUHdtEjwXPvh4fQegBYasW56QZpxYQDTAY2C-ypkSQQ=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH6lFYKZnv7eV5Fwy5AlCkwRocYD0sNqDoSOiYuQZVwAedLpVWNLsMAX5D76I0ZV09gx8w9Nq_OnzVPc010E2k_d0DJd1VY0cTHaOEBIyScZJSMTWoeoPDH4f7T-bumFxdbXmQGinCy
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH6xBaQA7UYAqEIT1l1IHtl5irPlJnCU03kGZ4CNCNevBczujpKfDFxuoCDLpETm3SW_69rxTYFmTdak4p2g_TUa8JDPb0R6x8ZAE0KTeeLHUJrrYqG-vecp_rLcQ1M8yDqW1w4dWDk0VmwVQFIAypFnmxfubc9gFFZNKobKXIi_iig7VenZ5OSWYVQ
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHNzmJQcE4UUgAdvi1nwFoH4beHTCeXz07RK7iDMwBLxzXhts4NJvOPOiBFU9RvbFkmTiKBrto1oSQ2tWgIdf3zMQQF2-mvd9f1SBS4GlVMtj8xvazczeih9gycj6mYP7cRWNVUV1eEryzk13WnOvCLvvkP
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHZ99eNfsbCeW_AOF6ho0pOwelM1y6DS2xF6pptsEVDhlDDW3GLgQNqt0J9wLmsjNCPX9RzxLfAmxlus8mcqH34_j7rZsAVxNPq6v3dWqOQyKdzylKOdX5CjuQOgdI2TQA=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHq96lyPiKsR83UASy5r31K5_JALAHV-W2xb_QKYE5PwLnSBYMBRrvNQHZF7FJMKjh3jFBULLh_tlJ7rnGJmsK3msMGcr9hb-REO22IxVBMSr__bVGHj4nht2lBpFLNLaNA1-1I6N-VDA==</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>BT-447</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>cameras</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Argus C3 'The Brick' 35mm rangefinder camera in brown leather ever-ready case, c. 1940s-1950s</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>$10-$100</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>5</v>
+      </c>
+      <c r="F32" t="n">
+        <v>5</v>
+      </c>
+      <c r="G32" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="H32" t="n">
+        <v>1</v>
+      </c>
+      <c r="I32" t="n">
+        <v>5</v>
+      </c>
+      <c r="J32" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-SEND</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>grounded_search</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEDHuBp8WvgfiEB3dXm7lpvRxoR0kCUp4PLf8sbPWZkEE7ZJawHV5HkjCCX1rdzHkmHSfXQXi0rgUb9jckTwzxjrrv2TW-qu41hqFo-mysF7VUamLdqtYFSzYMplCJjSsFCMqYrSCGtA7RuM1E6TLnJ1f4qsOWPAAPWDElPlR0Ohz2WGJ4L9iz82a7OuGooDOlfu2bmk21DUrDRS5NhGkiHqgXPkmBx0JLxl4lIBfNp8O0=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEMQmzjLSUoPwjWN48k41MEfmxxwqCjG1qCwHu6bQL-ZouTjJeqzBkRVUOP9Jml1RjvjCX7jkQM3SGgVHfZ_xyzJ6cr2Qo01XlZd0d0AW1nTTVWdq3FZOXko7Yu-dQd3iGSdbYZ8G6OSROBmpnyb_QE_1Oznzg49VF6RAIzbiuVwGRLlJ5fbF0jETqtZy2uBXWSgSc4OQQZ
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEPFPXb2rbv45MFu83iorkohYLMqAY1T89S4n6WqLOsjPMpQKvOEy_N-Hd5GP9YGcaCaDH4PF5ruw5hc-Qu9iA-Pq2jbRBrJvdSTwhH0ReWlDyqy7dAksoqNSI4Ti4SD9UmdQ74vUHHSS0bfUwCv3579VflFrYoPfrTdJhe1qdkN6Rfj6jG0VuIc-I7o9cM5HvwUcyw8dLH
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQERpQ3A_tm7cixv5LE_9tw-DaTE-U5LvSHWNXcc9uvNV8NjvH4j6-y7CD8XdLtbXAUZFpB7lN_ok1yHdlNUcW2hyQ3kdHh9isINyp0I1e9jLD5t7FkF74ESRpKSbX3gLkYTLfG4-xgEVMDdMOKqwmSq9JBmWRiSD121B4c=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEVSGFK8FeGkDpxSoBb_KJcqh9Sepr_hwpwqOoDBZ1bA1-Rj8FMOsFjBkj_Zr-AA0uQEXA7F9v4RR6GAAtPZrX3x60HaCo5u-crK6KQxr6s4gmBWKNe35yhrh_VFgYRSfFOoXRytdz292fgJfbjD9bmb2yaumXJSJt7Foc0eOy0DjW4c0f_2ahv2LbV2w-GA5vd5esCwr7R-B26SdPQPgAjaGs1
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEcLuBhms4u4luY5Aa5XJIemTO5HDFgNOFfq1nNgH_KVqDPoCLWUgFdxs6P-kR7vtzdawTnxfCAS6XY95y4LkWljOGyHwdXU6vGpTibmOoFiRH2fDXXNZZfMs7tZe86BmIBme7wRzfBWVBVJ_T8MuI6-JAV0w==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQElWgJQwRU3gSRFPMuFDolPGfj6EaeLDtbcAlkNtrG0mlcFeiTiXchWaLMMQ0O6NiaYHyudY3evSySFOSsdwnC1LafFzUGj7CLFfISFTYi2AXWunoKzj_VTWvraKnmRKrZ3ek67j8daX-IXruvtsOumo-P2zaJlm7U34UkCQ7noJxUHIU_hMxHvl1f3I1zWhB7HKgRsRurcVA==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQF2GhSJ_ZX_fY2Jpqkl05LZSwfZk4g3fG1spcwTDNSgS1pbS4MHZdjeyXqoopzMMP_pEydNUFQRJp-Myr3QtDXbfBem0PUL3jDG4gKIyLtBL2YRK6ZfCzb3GZyM5Q41wLfVPJlC_HJqrErt
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQF9dCAz5rExVxwZCLgNIUpkb9smnw9iTyr5n8B0ug7lZ8YwqbyBKnsqj2n1UQ2Ier9_aQGtqAzXdIPArC7oYUgBJ9vbMk_y6uinotLCQfM5VbFjqBRnbjat7RoxFyqfIQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFgZCFHVQ-KmUrnBgG835gWkaO-YbDZlX7Na7m1SaWzHiyQZujdT0pw8ezR_fjxWpSoLTqnWOY9pPLDn51LzCLesRjt_tXPH5CTxsh8nVpTgnF1FNy5vr8xNDGydQ6sb62IIgEO90KOFYYQpjvUUyMO02ZxejdiinbOnw==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGjrT6MSYRk-Ejc2BbRTZNZqRmreLtXgYOxu7_b_yQ2IetDiQWYtLGaTPGhxWKiPA3yFfnvBbuHBAlx1ezbSFiy6r9FHVYt-9qfbvUfrNwPpJUHAJ_YnTVn26KwOlBTWC0hs8idh2U0euH2LoqZ6dZUcqc7UuwO5PQhiA==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGk1jyGuZmWiRwbdRhmzLqrZJAyBxMoc5E2v8prRLYeAWCgv0Am6da38O9Z2jcK5wmKNdHxcyBSVdRwK09wdHpW0e85fEdEsVg7uoDe_DN-iP0bFEVw-fcMpCm5OyoPOkJjPOBZM5nsth-GeD5aqhzJ59HrkGDLIOFRSiWxU5q0rFAl-gJlCw-tAvfHRSthjja6FOtJKA8e5M9iNQjkhKQBW7xTFbMz6gtgXKA4gA==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGlCDvfkfp4mjlTI1ak2p2qZBgdsA0RmYDByqthXu6PcL94ANYgstdJHscflO10j1_oKPsDeq3du6-Dk2OyEtix034ypk8f3VOm6SZR3odCWXI2e0G32Za869cYgtF6uMqbV_1sLYT7VxTpH1rhjuU9q7tu4yt3X4wy05brHh4=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGr7132iE9medzprW9FyXX3Bvia7AIYe0XJj1wD6TIxx-cRI-JVmW8xkkv7Qtfps6AuyPR1TwsOmrDzftFcQMMr6S1ODk_sdFjl4I-J20W-_TqAyz4j0KRRJC9fd3uqRSe1zJClkZFc69zQZg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH9PATbClareGmY8wS1jcSKziRXoVlpIfEmDS_7Pv-hiIv2NG19poEMel_Yq9z5i1eGc_GKlsd-E4hJw_GoiOhnUsZurygsNVX6BURQpIJEovDSxIxouFVU9qTNBjKcKsszpS7GlTSsmsrxQQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHe-oevQIYrBJXccfKC-LwF67Cm3VqVq8hX1pFeLYdUXU7m8GTbJi-HUs5yyt4zfNt_w9hU14n6jMHL7X9EmjTXnoRJ9JL3Rnzt1IaE9TPvJmBTg9OExBvhjfI9fZT42Cjx7zbCGkKnbAnelWM=</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>BT-450</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>vintage toys</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Assorted mid-20th-century boxed games, plastic building bricks, dominoes, and miniature iron in cardboard tray: Flinch card game in original worn box, Canasta card game set in green box, Boxed vintage black domino set, Bagged plastic building bricks (Lego/Elgo style), Bagged plastic dominoes with colored dots, Miniature green enamel/painted iron with fabric-wrapped cord</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>$15-$40</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>5</v>
+      </c>
+      <c r="F33" t="n">
+        <v>5</v>
+      </c>
+      <c r="G33" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="H33" t="n">
+        <v>1</v>
+      </c>
+      <c r="I33" t="n">
+        <v>5</v>
+      </c>
+      <c r="J33" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-SEND</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>grounded_search</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQE8QdVPqFtvboZOaSHwHmV_6FuJyV57MxDrCqPQT4kZUDToc8Zt2XGYWp0qJwzfStq1PQepCSslDMHldmREXActGckTlplfUnyNMLrAejVBVWhlgyPvzGK7CrRNG12097G9gL4w70jAeWnZDBBCdlSdHQw-CWiQCbqSGD7PVkNi3fY=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEG9HM_kgIp8BHmQEirZ1zzgC_S5jcwuoRIseT6ENvi619rbkswVxxk-A4BoN5FZccbjU4cmVAX7RS--QJM44EuY-2t2IX71ggj9SwhTV7IRWRVK0VHiVhiAkVrD4DQkhiqCmWxfb0ySFXWxOLGw-tBuWoEBlu5p1sQuGgeYaTapd7pQ4s=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEI0djEOLYNCdORVEONjb_SCK_QNlXtTJ4gnIt26ZmVRSV6m8pBYNj9bpP0Dssa8BXIRVmtUB1UXlE_VrsOxyB8B7AaKaAToOjzCeoFDrF2jh-kiVIwKkePAM5-Pf0sHZRnsxAaHZbI0g==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEOhery18QhONXohK9CyFXRADtfKkGQAzK7ZU4jDiV3i_8eF9vQxWVhYjxvqdGo8wEg54DdFC-RhgTR6pXz7ECpQIHwGF5bNCwsHcxc_XyBuFAjmgOQ4aFqoPcS7vNj7OkDazXhBgvbv0XHv_WkpO8LFLt0ZVsZCDA3YoEnjmW1JvBi
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEX14qXnPhDemBurZnJ5557XlJR3RU6ivZEZLKq0AOCpuiBi2palvjfE74vZnvoZCnsT_X993oL7U490SpEpPNdOPeem4DAn3GvdFtJucZFFnvG8BZ-8xsIHp5gZGapnSRnw6TuAgsm_acAcYaTzH3YLbFUGVLuLTEaNuNYoK-d0kUk5NJ6lpFzTZc=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEeQFackErBhr6WsPMTflERA5uVkLuOSoB99pCcjzSv2CsMBuFAu2ZgNPFu-aUuWDJ-BaWgN7OBiHejTd_udhR3d_Sdr0gU9qCW6NQvf_4_CE5GfNfZTiAwntToD5NHG8J6R0CELO-TIRu8C0dm2HBe9bqBzKAW_xTfP-xKISPmByl7JauPLNp5pCkx44eI
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQErZ9Obq8-1B8yDA1_NWDxtROgf4gU3yBJDzMMX3CeTP0V4qZQbPdDH2Z3S2cimK_Kx9qc-Gvr3JUX5jHLvqdgNJgtUQlpZQrPBvRMVaHubQ0EoxT4VXyrlXR3LbElG1RXiXT9ggHAm9X0KeeZ6jy6dTXm1SjelNBNdoiv7N6BXaKofxO91CPiicNPJQ0gxOVGX
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQExSm_3qrVXFhV_SLFplY0MeKdULl1vdBznXhviGhSrF9HxHbzzeBTpSdzTIkhnEuZx0WZ4ENpDcO-aGqUhTFbKcGPvnnxkB6g23XIGiWgjUz1RjvBEI_WtC3uuDM2uSg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQF0C7zGhYTyaxjCvtGWxv5mXhPO3YksE8K2QQTMcLgVTrV-U55EuX-Tlk55LIreE7N1quIlGEV65FOf6VqxncWtbQ_VA40ThD19KqwHsc90_rUxyAnSPsK9cynGD9GAMeyt-h3JLvWYJCfzlXBmX57UQOM_tmbF65j-yblHUadIAA==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQF3j0fjeUIaYd9VDt4umh96F6xkHMW3qSTOHPVtzmCV8m9NDixa3y0gnLPp9WGONHnXw4UvWZKNfKwq5WD0_NTHY7J_STptBWPJQh1r-t3kkQkSN6GJ5K-5P_QmDMAmerIfVFJeALZCMh4lWQflFVnM_rKGcSNUAnI9vUtBQkBFWyA=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQF7Hdq_zVLFYoK75xjRyICuSwQH3AJ6BoFxRTgQGx0gIGRuOsoQR-JG5iIWLXQs9bASA0VK1iThjqypTJIaoJrFHTgUJ80kUYqJBDXJMI9WPG7m8xnBOLShNhb5KDkw53Ve6aAQQzvZhQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFEmw016SG0rzFKsVVot2t6oGLeauOmFw41Zm1Tzwq6KJNWVpBnJYBfSBcTJCjFM_dPEQXpjwfT4gvMhM4i8tRRjnz_EyA7yZcEshLsicSn8FmnOxQU2gMaulCVOHPJXQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFKTsxv7crEwaRlvbJ5qPKk7LMgGzBRsUxdz4f48y8O76yyRck8qduwQBDWYPMnQxzJTmue2dtwuUbyCprQPuVUkjUVeeZfM5BYluH4Yy1bNMe8rksb-D40AXdQ_BhP0JXaOStU5Y5avVa8ggLP3IwZn0dcnKE-ijmXs9U6Krnp5Mo8QACBgKS05vR7adOCiQUaU8I=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFddYhBQp0lgwCG4mZnerbdxhB13eiUS-ylYM03VPaVRY-UwrZFmDSU97DYDUoQbKsVYi7ZXbfFO3EBYxCDCiQ1F1rYBeZAFMCIgjjCOCALoGHYLoTTpb49eXQ0L65Kk2yBFviA7ZZ_g9q-sRQ7xR7TmQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGMCjvozNOkxJ4dJM53MtN1uRwUb7zIpmxxJCqQ9dN4ugPqPNhFQhrVDM7eFsyClnpENzW_DbH5jRlvFK51dVkrxoURzeGYwbddNy644R-T4P00U6W-t5pQ0QemMHcIbfccbQ4ZEmf0NimX9hIzT0SQR1JzwTZPeENLz55Cal9LhNnJH9zE2aPVeOmHhcNpaiPSUr04hjHkkX7pVEtUOtEBwSlkhhLp3FMX8uzgH3nsp8TOFnmeYsiSqYfHLPFCzAIK4dEqyR1Zg0o_6S4=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGVYCI0Jd1JUqdUGXfkwRgFWLMeuT5eFIEiIEAk4EkfW6gwcPCFP68moPSx4GQT3ks28WMqGqarfuhu9UVMKKD3qRZ_lZ-t2T1uF60gdLk_awYIU_nz1OI_rxdyMXo40CBv8Xwf
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGc7DUrP_61Vpc4cJwagbKozYaXgwAgkTqKbR_lwtvSan_wCcqfjzGQQN7Wp4Ik5z1DyKhbijCbi2SDn2qgnAcDWavb8evxBFDgRi6k7-2JlF0RRySZgxQ0wkOx2VWfkBmHK_4VlLSoEOZA4VLQQJ4vjpxCFPp7CKfjrF-AjgIk-LwhjqcW8x5vNC-7PgREjpLNCwSST-BIIUhe9r_kqmQp7TPgLU6WD4V2aA6kkUwNFhGFHsP50nm99qw5l6-9eJDKocoanhfVHLpMel4kc66IcaFma9ffzPtsb7QTuC2O7sq6ezEaVJLI
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGcWGAwSDHS5h9cZUdhbIY-AUspNiKlXHQmNx8bQZX_ZCR6UKnHYFFU4he3LvQu3xjEUx3PLjimgahzM-G1ES5Ih9qHY6JO7SgHdzZUCTG319RvVVp2r0YzxCDp4gQBoxxKaI3PNePxKQE43k_gpQ_ZsfkC3bk_KLwU0q9ENWyd
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGdffkoV8_gryQPYCAAdoBDFIwBD74JiMgARXFSgrlTPcOHVgix_iUA-of01QQAz9ULbGINGYiDj5BzwNbD6-LnMj4u3C5FsYSH7OxOHavzBfeH5wDMppX8eOtuq1lmgRpI5vm5xIY2ZVZota2t
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH-GDrOlH_ix8lJK6PpNYV5FE3AWRnnbb43B-dVcvpSXRaPizOK8rmtw5OAnAsvccebGCl4hoAji8dNTml0H5aXZXsqHlppxrOgePBBZ_m4H9aQqE1RtZ6rltT_qXL73ezfZGpScZgVNdkOfJyCn7mDvi3z0zPaZsS6zOQO0QwpAHM=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHD46jRDT7PrqlbPDBWq7XEvwJOTc1gEWYLNTqfBwDWnNGc8oZGLlsQubCRs4CE8yHdF1OvF7xCCz6DBN0aTL9GGOVIIymjf_brIMMB4tp8YV1R7UFh1MmhQGwFDGFWrAeREuJ3a43GKTGGvFMtsmnZ2kuERksoPonmZh7PVAN0GEMaYgteHljvOznaQhUScnr80f4VGD7JZT9BNCZ1BwK6ZiHLbpUgecbrLQyqKRQ12JYmIJuTca6_0yhQCa1OJgDfb5wqgGD7liCTUSPCcg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHFBVh1wPEOoTMf8A9Z3Xg_zbzVyz0l5dnWG1wUx6P3_UGr83EdcOVCqFrjBRizRuJHan2HwUDoXpQstf2j0huHiudr_ERA9XpW9qjjGjVQjrbnlPic8IVNnF-Opk4WLdQkrUnVR-VNX4rqmA==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHMpZXsjjrkABDKldzRW44xhzrW_H7G7rtb4Yc5JdVEjzWwRWdjVgv_oAsnhKtbViXFeVPIgc3rxF3xH_x6uOxmjMRgH59GKvZTWXkHggi89TXQp_tyejoK5TzOjs7CiatS09u1eVN8Bivsrq9_uVgKqcDrrUd6nzwX</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>BT-457</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>cameras</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Group of vintage cameras in a leather outfit bag, including a Kodak instant camera with built-in electronic flash and a 35mm SLR camera body missing its lens, c. late 1970s-1980s.: Kodak instant camera with electronic flash, 35mm SLR camera body (lacks lens), Brown leather outfit case</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>$24-$65</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>5</v>
+      </c>
+      <c r="F34" t="n">
+        <v>5</v>
+      </c>
+      <c r="G34" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="H34" t="n">
+        <v>1</v>
+      </c>
+      <c r="I34" t="n">
+        <v>5</v>
+      </c>
+      <c r="J34" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-SEND</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>grounded_search</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQETp2F_ZpjgOCKL0L56uLJ2ELWOjYJQhiiEpd7Jl0w4YtD6SmzH6c5SQktVyzaL9GjYU9JbfzQPAKeaa7Vqw8sNvXqWCFoD-UYoyUA8xveMIG9xIKUHXkXEoPgfNA2oAjs19VpjxtVdnGefV2_-X-w6lURs1KQ3bbfRSekuYXY7CeeJ4tYDHF6LJGg=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEZt7GjCHZzucFbLlYBWgEbn74BY6_DNuM1pwV_nANxEkp_LPG5MUC2_znPbS6m-YnOnPX9AOgLfg7yLHhxqpd2VCrjfW9h6ell0kE1Oz1Gzj4n_8Ew0tXa
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEgk3_bbVlTIcL_3MnGiKi71Td158teyOyYtC7bbYp1CD7bcX3jtIHtcceUDyOyC6LWOXJMG1xITOdlgPTyDC7l3hpcpuz9YE8rKVeYFP_Q_I_VOP2NoqN26H2L4ZrnSblGBW7lcPUi11FwX6SBdNK3qMaA5cRTgyiCDmS2GWfjGiJp4U1x
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEh09bTn3mgCcdS61e4v4hkoJnPKD8B0pG8MAOkwQIsrajBROMal5DkI5j-0LPyuDQLvReK5i16siYxSE-AHO-v6lmh7hHyXbGAm1eJJ2DgecWMXXd1OVF4wtCmWoX3UYIbTi3WfLiVh5cJegFJl67BJXUOmk5HWeB0aNUQ5W2ENYv0
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFKXEfLTLYgUfoDr4n0B9mzYk3rAOjNe5kTfas2l-r32j_FmDsEVOkVxIIwREk91WxZDcBrWnRL0ap50gmGOZL8Qdn0KYP2JDQTaq5fiT5BCa-Mm1hZ9Xv3UnJAcpaS1pA=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFM1Sz-JI9QttT1zqBZmD3BY9aEoHdpjWipznEORDXOraT5DNDKGl21pYenhFENqCMr0XYKhwBRyNUDnSdfFwh7q0yiGoyx4d6wvaQAElAMhlkmRg3Fc_vrxVE86SmXOas=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFamdIQWEp_3wBaRTfsvJqn84t_t6tKIjboYa2iHbWCDh5gykAMYpktKScpKDzOPl6qE_pfll_FCjBpKOfzHOgdFDlMEjb3IWTvMpV0T0mOTq8pp6jUUQ-Iu_80ycT7OajV2c-iOAFu4xhHUHph
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFtYnhO_Ff1B-8moK9EKfK1cnkzOrEO3oR1MwTSGvtaEPCepCl93Wm39K2n_8pp5uB5LUNaIV_a4u0s21oC1CjB-_-364FduOR7VAYqBU769vA77PPHobhyiklF1nWZmvjNSu0=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQG3hcWdJBoaTrDwDkdYBugX9H5GnT2buMwFQaSap_X5ReLmpQHAaDg_aQl1BeUZHMi_OdA7cHhvmJKmukAaKUIMYe_rX7V0GHOzeyJsHNKPW3z9Rmm630OVRC599PVOpeQIfGuiHRQkLG4tHZ1qLR4nKipbXfMATCXbw1RHoTtSuiiEHrMqPhAKBdBLxG5H3sqE
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQG8PG1aQ7hzjpZSwGMG2kOegaoZjruiyr3JQnVc2hpa3Mta4gGaBoBRbMDQNxjw67To9X2BP4y5M4bsYf5Tjciin8XttA838TSX-031V9M1tEV4QkzyoU3Orcr1eiX0cf0lO-79mugT3AFWju9a97H8Y9FpoeYy-3qOzHvZeX5hLTRuNN3ampNh6KndCJ5dqyBXMABNPSFUmynzh40GoHkBJlXffPVEvKT0CRunkWZaIo3KU5jkxL8tusgF4T66lQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGNkMPZLSsr6CYAJ4ZmFUg-aG-YytZxRAVjN28TvyAs4u0Zk5oTKFD97sWhDai2ZWBdJ5GwfXtWhgwsDn36X456dYAUkUfVmEAaOhr31rGexbHJNA5jXmEhQYyz1IcV9SLd1bJdt_XdamXaAzqsWAhLys5Y4hYrYp3wTQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGpE7jaB8Xy3idbjg-lPKUME9insPtfB7xwCb30c6iK9GKfJo-7U1H4OVhg9blEvELBbgKITMRFYNB0fT5yEcRMIHndwAweXdF_rR6AIDKsPN8u-fwLws5flbhywuAa-jxVPvkguCc3O6kmM83lVv90r4OZzMmqQGO9OLo=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGqI2ddNa8a0McDEok1Gc5NIILmyTuejcf4qUuepHnux2KiMLUNoFEOF190OpRXDmEtMq0VX9ZwYq6EuIRBmHgpbQOFkfU_KE3mWNIbzUqnX-iRYA7e2TwWGlBY10sDxYZZRQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGwZvvK7jKezH60YVXaV1Vww1YCNzOA_IC563RoP0JiOPdAuWnvSFkVi_4mvjgOiKI8mbHQeAfMCDyHBjWM9n98FXLKLpe41cuVAaA7iGoM1x_n6bzFT242UuiIRpV3AOtKSpYRxlsfcNVYmjHxUsIDuba2XBJnpjZzWwwic5Z13g==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH7hf2lchkJRYsTUohi2VoTGQaD1QgJwBKz7HmyJetgj9LKwAYOjaDDSA9bw9ypTK6-036WVnm6ZjfutBKMLq1Nk0o1bbiIK6Jgod4AWHY7HanlIpeCtXcLMUlAw0-N-ChnlAUhz47EJ5mcPLohDCxdX1MgLKXhbbBDjglJWpKIux5bvfHxlOx0jCPL5N9qlw==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH8ws5q9rqWhx0YkQ-BfAnexI5ClaRbAYsNJik6fBNwQm55iTtwE5lFN3xHG_7TmSARNxOFp2dRQeJJDA_a3TgweI6cfDcANX8tNfKSatmZZMIc80IKNTKnoqQIRTu6pfi3J8bS3LY8RQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHNO7AwH2FS9jgdx4s6km2qUMMlKCtQ4lG4kpI0lwD-2s0PicfJIIHjW8krTNlWBM6aWyDiRNm4QJqk1NsDVna2s3r06CahSr8gh8yIBGvWUUGB5ID03VD0nn_R1ite8Olz2GfuOUctDTyBJ6hlswVydjIQU5-w0x0oU5NIyBsw8W-rL6cksS9W
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHcjdsVqkqGhzymyc5A0czDE1FP7l7Wl6cg2fQzex_wqto0n8fyboyW0eto_hV5RAqYRjeZU52M37crYKOZTw0vmJjOp4U_jz2iMVlexkSObskL_gXdHivfjMTahfN7OkemrpP4zsVh5YeERxSrPHUWDfbY7RHG2Q58AR7wR2eSpG1T</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>BT-113</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>vintage toys</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Tray lot of vintage Topps sports trading cards in protective holders, including 1968 Topps Willie McCovey, 1970 Topps Rod Carew All-Star, 1970 Topps Johnny Bench All-Star, and others, c. 1968-1980s.: 1968 Topps Willie McCovey #240, 1970 Topps Rod Carew All-Star #453, 1970 Topps Johnny Bench All-Star #464, Wayne Gretzky card in holder, Dan Marino card in holder, Assorted top-loaded vintage baseball and sports cards</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>$35-$125</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>5</v>
+      </c>
+      <c r="F35" t="n">
+        <v>10</v>
+      </c>
+      <c r="G35" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H35" t="n">
+        <v>1</v>
+      </c>
+      <c r="I35" t="n">
+        <v>10</v>
+      </c>
+      <c r="J35" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-SEND</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>grounded_search</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQE-eI8keyaFQIzRn9egCffr7zQcgCf8Mzno8V3ongZQfoG7GRPK2aA92s0mXam8cYRbzmJLRnkmNeGkIvQfTfBnWc-BeOzt3v8NztzpjMDa3KPygeaVUdgK94DpKZnTGyG5pFVfbGyQ8TVN2XDWw_EFxeVBBIiY70lcmXovvqAzj47LXnChNBi0I9R25r8AxL9G2OMLuLkZSLhxEIBWbIttAxutKw==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQE3O3_RajRT06R70x3mFLNC4fzI1J2B7qUM-jeK4ppqCwzj4Z31k3S1IXmb92K8rx9q1pFYEg2BnKTJKiDVUMTMfmZ-e8AHBwQIDjq16Mbm45ghq0P_w1EpwzeuSoZCoH2tb5D-1PNQNHQDoifLIrhdnd7CCUNsXdOQ-x5jBmbFK_sZmIyOyST0sTt8
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQE42vGQWiXRa7BpKjU-548CMb5o5RHSab68ceoulyKnODGQ-ln8krdmkjL3uomo0P3XBGhLoYnB_27PZSq1WOHNBOsSoTuDupF9Yhvg3waDdFM23rbl7iNNsTe2h7Nv0JAyapN7w-tDWtvWLBdE3BtJ7m62mBsdCqiU27WTkjs=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEkX_KkhagF8z_jnB91xcwJIxIoIXlEzJCScn8sy0ejqHYNlRA9uPE89NXdxpt8HR8rusJaMUSFNjUg8zclg7nF4xslPqkNsGSyPLUai803yWxTxKvIcnJUGwTAM3RpSgj_Zb9wwW0Z1qpFaWf-XEwbtrL-RLNEbeTo6o4FTTnjuj9dDPza0aCZ2vswwW5qrgHL9NQIoaBRS9gyD6365teuJavs-GO0FFLx-vvYcV0=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEuA98dt5Am-rdC_3wFVAhLVp2MmzTxgzEwAnWEeVc2yoICuj6HgCwRJ_FsXZzA-RKn4HJBmM64mFGw7ipRt96OBdTEt8_4JimantPpGGWSCOdvv0y1gDPgEwXJ5Kk4Mg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFEUOC-bdDu_K7xtyJgTfE9lngJuJVNnIbPzU2hLt_Q80TmuzzEHQgHvAS684q8WHj9yGvuX7NTDztzCbOh6PqGfukHxN3xHwxEICNrRyk15wwZ9PjnVNAq5PQo05IL6zU5-KSpGZ5LsDKbEUpxpCQ94MfvMFCx3rk_1sr6fUCByQY9MlASA1tXAsg=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFEYH3Gkt6BwdtzW0fQfSZcxUT-m-YilYyfniA9MJbbhNPexdB9YMfY6t2x1B_AvpD1xeI--RkNIva-EB0BmiW90FrnjH4ZEzLWb4ePh4SKnmL8uKBkBchjUdkrYW2dAgI=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFIvzQJ8FjTwq21VXO-jJvys2x6YpTEtxXQLljXYTK5qJ8YE9vA9v6jYgxYSjsBI8UlCQgWpv2y8GzSg8AxXUSWrMzvvTH0BS04r8tcpXuHae6QmAlnWxpQ6wfIAGh-GVXrPzUM0buMgdCkxyreFnPR5jHGW5u6n8xKKhNPqQ7tM9azwzTaRchL_xvF
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFU9xqnVy3iGmXO6MCXRhQAz-hp30xJKs0ddLbHKICr3ZN7UsRgh89pYpl8SkuE2aUVP0d96MdcfRevkkaHLBnoMrhKKOTkJ7i9JrwB-e1jDBGCiiXtHfhL5zDSeZw1ZVA=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFVzFRm5xWB4VYAJQmL41AxC6RngVV9OcLEds3haUZVD3-01VSU1t3vDu3bKGgMTwdPmPMhhrjdH77PBwzsXi_ZAUfJG_H_6fT47AcRseUssH5bh9p-Fkc9-rAEadgX1w==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFXvQPXcPsAXOCSgPsWPR8FbC1cLKPywBaZcW4O1W6dT4dgq1fJAfpa6UXfm8wyCEVmmq8QAHc-cVxp4lco52FUw42MIPozMn1MrAHSW0dqGmhLgPP2aW3sepHmyKNbFA-xYArA2WOHA-lN_w==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFbbw7spgnbXwGiGZyPTzsNPGOKiydZRR9DQ0ONAQI8knf6r_odmjrCkAm4k-MskeCaRw2tx3R5Xt5Uyo25-UwzB7T9TZI5gZWO0pWrr8_4iOQxChr5sErkdQupmlp8HuVpcI7njTjwB2JNiqw4lK1HtrO-nV9XG84e3vdjTE6o8Wo=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFrRXE03Ou5vd7FT9rFuESOBPY4GhlRDd1oWp9TiLtTNuyzOEdp22xWc9lQl5F1npvCFVfcsKgjtKbtLBYlQMGzH4MHIeGyuATx0PRgM3rbh8gFap_l1Ym25u89eDygX4dV73O1c7gxvF--Fao9UdBbmM3qEjl_x7xPcwFKi7AeD6d4b2PCzWcUZznpbw==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFuizTXsM50x3f674283Hp7w0H-PaAlOsgqO2_TgRhKQOIgusG9BGUz6nJxBTHdNFYsTJK7xOJSCGh56MSlz84djGJe3ElpP0MyUi73d8SpjGbEnW01pwokFHHU6DvZqcI=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFxuacLyLytGjAC_xcMCpG5bmMeWxyWz7AP-r18XOHrm4Bj9mDrpnSlPnJENFHdAD1fgBm2VYJaymZG8mb_s2eARAf1JxNU0uE4gOUHcYMfcVCiSIO1fiCPuYe9r6p9hm-_BC3agDZV2XgG3QFHZmppIiyu2-xjT5z_2WhL86Lps5LFNviAosaCU-xJ9HW-3MfxKovslS5IdoRm0mA3ZJevnxYFIGI=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQG6tduMkTz_o7igA-MhnzCKvEsyVUVolJMkWPGBppq1ypoPgvgVThIJeWLR6brXmcNamqJxa76l3Hzb8-wZllJTWJZGtbiz8t3-IBvro57yb9E35tdVZerKUgoIDOHuK3I8UFyor2YQEnnPu4CBoI3BFONv4BUhIHWY_6Bv9pMK
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGB1xZA5-XLizHXTer_jhYHSULp4uRQfBOOmQ0v_cCE1X7c7AQsnbVq92-w_SAke08rZTVMcwBgRGGbgLqqwj_N9wTayKJA4zatdAh9wcB8p-ADzkQfx1AS_s-CzhpZsmQdjgiNjKaH0gDAvz2oOhoL9-RQwqjcjISk4-HnOXWQqJvCjRfH77CcW6ZoaLGqnY5x2OCMI3hNzPEThj8QM4Rjv1Cs6Y4=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGMP0rA40em-puqgw4dxbDs5zzaT36UPf7enhUEEL8mC-jnSOM8quXZqXGfRwfyAZy_GwgWRxlaYJbW_V7GVroTRvYdTGWBXc3RNdabExRdQfi0-WF0BPukqzK_f85J-80H8PwMkAJg9_2OOqMflBhzWwJcPXOccNwUCWKo8_jEPXpZLxSKf6l2eg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGkKl6rRy0S3avh2dc_AfcSk8SuBYK28nptBei3pGqjNRRUZX_W1luaS7zEos5Hc1N9Rji7NjrO-77n5-NXj8gH2T_igHxL6WqbyeGZscKNXXogv19ThpWXpXMGNLAL3U_M5_TRoQlqIr74bdDP4Krl1QUjZ4KTW8A5hDRb29aMci_DbOL1W1dVpAqgHuGSsL9Uj-G3eqFHK40cpmp7Wo0J78brcD4-29I=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH1CP6hT_xlKIjsoRvcVaAO9C1JOr8AE5B1Dc4JtWO61KA1gTxoi93deHtApysTE6SOfk6HkUOfQloOR4MWoaAQdueNfTmX9pXGflQ4vXQV7KfOhLJsY4SKoS8i7MELQ5XAJpIA328IYqYsltAkTwJUiQ6I7Pv2IUMTEb4-NVxn-MroMbjKf6N47WTIaW_GBqXLo51hWXUVeFMzqLU19_NJM1oy-UBw35m1lf3XOXQ=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHQ-bPTE9UbjmblzBcKxFlNzF8IWjssqaFS7BYoWAitEJxmsdAOrNzcL4mZUcA8KgtGvabZcH94v_cnYx-I_aAFh-c5WZ3hpaRr4ISxkw8CbRwTFnXaCFphh2zVULSxjjZ3s6jNLE_JlHBuU3quhWJ4fdtNk329scOaLjPZIPkX5xLMjR1b7A==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHTo45EvXuMNoOpHwLLkalyCw2i7mtB_aVDgBPp_2lYUNiqEHOIV0v-6nrPKex7GHvMMwdGDSXHulkjfz7orNGjrpFTE-zoY0QXYcHQSStWS0v5-p6XfXVaumwTzMyv-pJB4gzK2PFzcuiFYrFigBSXXrKNJMoegys49n0es3FbhnE=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHm7MPc4r8LlULeN5ieCPp-J9pggCxbwVJ_IerxNG2hCl7L0hyoqqw5aedj6_Hhnj_hJ5O8wrfnGUxOGJ5rtdaitBLMn3VeyFMpRZsZbSg8C_WWBHRieiurE0VKKgR81wtokx1yS7H0QWipZEACYxUwivWMkBe6GeiQZxLc6C2vZ0CoFkvhr2w=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHxKQDMBmuhjIkXxfJgLk87Gs9TMixWBT4-2mKWM-C_8zc4fA9te2se8m9qXGa7Ota8MAasq_vZaASK2Zk4kG2VKsvAPfQQyDiYcZ0drteZiaZYQZfhBntan0OPO-Qq4fie4Kj-UpanIn_R</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>BT-165</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>vintage toys</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Collection of modern pop culture, sports, and advertising bobbleheads including Walking Dead Daryl Dixon, Star Wars Stormtrooper Wacky Wobbler, Beetlejuice, Miller Lite, and sports mascots, c. 2000s–2020s.</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>$20-$100</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>5</v>
+      </c>
+      <c r="F36" t="n">
+        <v>10</v>
+      </c>
+      <c r="G36" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H36" t="n">
+        <v>1</v>
+      </c>
+      <c r="I36" t="n">
+        <v>10</v>
+      </c>
+      <c r="J36" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-SEND</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>grounded_search</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQECEYGqu7ZEBsrkti-j8niEzqS1gDBdyvX7FrpDT6LxgoqayEDJ4VZheiXb0fjtvhwPFuQCBMcm3sB64DO4o_QNBJudi7pFLRsDAXpayhHQVgDBezrDN-OahQFhQGKRMnXQrELuzvR1UEdETicEHZftnTeUogJM51L2Ca3YEd9HNWbgXRBqB7S_wqcnSRhFhcCWl0BK_jLdfSFyNnVVTGrW3JcpuYcLeOgC9TykVYumkuxvCOTJQvhC2Bi1fCUI_mCWbzALqawnHbxwoogcSO1V8FNyAM_OREEr
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQELtbjgCXMivwy50zDR0SVUt0aCHp4t3ekVgt8Plk-aeCXAnJj7GXvaFCGLH4qHYNPZxAhAFgLwyjyQI7RZIg2lyd1LTLsiUkm49MmB7fR_vIJBAfsOUX6iP4nGStVW481CORG2-kD488Ci599_-l6QYxVlwpubCN9mV-Q_a1QTEybEGicudNxbRPkstu3v6ON0Ri5Gu15efQDbdDHEllEFB45j
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEQNc46CNb81tdmYjzXtBM09ntNgu9qBiUDrxLoJqpIt0q1ZAi7ajU2MfMxnUy3VZzoiYXDBZzMNlrACiGZhlwySLfUDW1kSRyjD6gDeJUyEd9EZhRE9lAW3QMFFlB9EETMWIOrufxQD2p3xwIrYVIbtLg70w==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEgtsFYtyqaHy8WpxwDksOgnHF3rZ0pbqSqmEEokP5Ae-2bTaCNPcQix4tpG95ggDVFQGzDAjuR78fvFi-U4eClOaAVJqdax2FgtsWA7LWvA4nekU7k3kNMpYnHRCgcnpaEr_HqallVQ8ST-ligiITYzEhv9GSW1e0og7ixkH6B74ofT1eElIigXbUlySDQNnJbBOv2wk7-9NszFipeQsQ=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQErcrWUqJh1i1ZwMgz2hlBVrXFfuaKnUayDx5LccyqMjVcUhk-Apzy0uoIlY2vYH58LkPg_4xFKzspgycFywE6fCkMc2XJWeVr7DUd4mzYNFNq8yZhwUXcd_7PITIlTGH2SErlW7AXjJVBwaFR8z-PlxMI8VI2QVSE3YKtztKeAeJKow9T56uIV91q28YkIIdYGiJ3W7DV93By5tzcMnedRAONP
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQF6oWBqrVb1RT7Rp8E_puLqeZqEZB99smbGN2xx4Kf0qWLaJVde9IYZQYXjBjzXhv5aMjJQWGnc7xErhe72B_j3EKD456NIOG1PSwUdWA5ObGZ7jg96Navn3wHKpkV93Jd1-2X26RX9
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQF8hcnpFEqh661sxpVlnPPxs5oEbgBszLH89wUjJqPB4Vaur09qizNE4LpzgiPTK3vkSA8wxIW5VhQMu6xlYUE3NH-uv678lCCdJO53smxWzXzxYchJaz11bVzzUsfYqxapKyq-l42Ac9iG-Wezv_spgXDaxcq_2mbkFwgeuBW6vcbpDQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQF8qVBDqvQfu2KBOINlzk1r3hlceJA8xGok0xHUulMsrIHZ7D70V5CjUyYw6XVItPtBwuqthq5Kd4_Xy_PrnpEAU6wkFa7vXwbmHwXjKiH7LMwwRinohvR18xxj_URoyya0xDyyhhI_sZrurItReHSnzN2RRmjkR6I5K73rHVp3w-GJH_bj_w==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFCkQGFQF_xEJaNSWG6bjrrNYbiyYoLSuaaJE8Cp6sbriFK5UsVyKKJUis0bdJ1P_WeDwY0JXfCkS2bDkSs2nRsZOWB7zQcAhWjZYlIOwM6ARybuSaOuWU47yaJMsjMJwvsG-t2rpj9fmJ9N-qPRCTtNHNGjsKC
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFaQFMNoSVmNrwgw9WAbpxYziKSv6WLr4UXqMlC3YtImlOGSjC_VyKSjMJvskstyCewaAxuq4GJ4ANsZTH_RGl1BQuZJ5rYZq5aOjmIhORC64oMthcQVASjQmYPU6js1Q00
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQG5bTQvTuUkaFMfLguUr_t5RcoK-kc8GaLWq2ai9PJIer-Di8FlADU9oYGIUGp-TWAWH5ezQBIb0B1i-tV-xAkTJwfN1SEXVpDOhGIrKooSd1V4VYMdDqicpvxuTnoWajoJ_9UYqt69yZyflLaA1QIRBcM7XWJFC4oTAcQr0Pm27WlvD74ln7Pde8x8FlqSStiKU6WDTodcIHoSAdRduh2oZGiSIvapNS_wDXdkIPX8JnSD2oKQVwbdKBE8S58DJMZZrS5g-NpW45mLzymTK362w7rwTPXKSYhrEuo=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQG9Tc26O1LDiCKWCZz2D6SiuFm2sMggIJ50rQ390QrVoym1Gxhu3VAQyjFkB8-p0ncPyc3wjCO-P3_UiJQCS3cRK2jWDoZ3xy3ktPOENqrPzMFR3X4WQ08A-oU9U00ASfRuTP5ZO3PlumXXHwLuD3msWfVOEsQUC_i4FG9DmF7f2lsfwYcrb05GMwURw2GO3IQ5x8CqKvAzuRCBC6C4cGA_SvuW7g==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGFEMdHwgY8KphvRD5fkj5DFWIdXuD0_pF0ozY8qjebFbJ6TDzQhauk-imr0cRVmgfvBvcv6n_QaD1cjq6Jww25hTcH4NEB4ciDULCBYgU5u07pBy8M7ROdJo5tRTeVrGvy1DhPoUQs7uPvkNqYYdfCvccr6nBYz7jZ
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGGWK0_pr_5hUpsqKHQS1bQwDssaDTOx4WtdQBpr9T8ascqqj2tJLpwgxqERn_DXZx_4O9ozilGmTtbJiH1TqwILmcjP3zP5_UQn1IY4uWh4lrYrL1jsEpI24f7VdPHkU0=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGQKL-HYF4jP57NnTxrqFV5VS4Afn2o_PBaPKoilwQg1UNIQjVpOIbCCs2YE4SHBpfa8ea1gXSEeus94ytv0Tz2DsHed8iHtZn6GZOfLE3ltH5n49f8BI6uWcU9zAl4JsK1w3bvB709HCejSxUu1esAg0E-comwgvrj4rYIcwBOhA==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGScdCS_C6sy1Tk3qgR61lVo2pR7Vgul3T7r2f_CMw9Ll0vH_SAYFcTbsmeo8WhiAH6rZbliTvUZI7c0I1-v5-RLf_RvNszIhMD--0NGXCgETdMCm26KO-4jc_CNEzVUN3fxa2kNLH_UtW1j29EsSLaqNJi03_bTh3F
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGZ8QPllu9Eeqh_Ir0mM9x2uvZPRKXA2a8yqpvlSDfiTwTcaB1sWqQkePze4VETVD9bBl6gULWiZavCsSCRdenAzY1-abTNo5zlLiEf82UKoQcFPsN-ZqeV98nYJoNfO7uDHu3sSZ5s
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGaQovEoOnzvTSteaIh47MX4kRHUnsQnorwVj9lStdG-qCNf2ODjaxqJ9q8hYgPAQRvpBiFE9saep4Ci-1QHoopY9Kqe62bmcJqNUH4aHXJSZZ3GhrWX3Xj6tr8CMry0LgAIZPQrpTaTvq2EMI0CDdSVgE-XR5wEeSlKQMOb69F-20=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGbZ5o3cmvRHmjrP6g85pEJ9iePhGe2-ztKhKFGPmBcogl8Y-DNnAvOpdf7KzDD6avlY8ZnPaqNyE3mc3pJYsqsVZ3g-5wVITqMKe8UdVeymKrpTbtc2nX7mgDYNPRZdZXERy68bDhvJueAiVXWjaJqjayjuZtsektO
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGc3c4DdBUuNu5BV_S04yC3lmCEi15HD33N4u9DFdSvhRJR6cL0UpkOyY25TrY5YBW3olhp5mITpEAgJWBqgbt0JxPQxMKJ-9a9pNJV1cw_zR7jr08RScmEJ_CZjFWGAr425lL9L7oT7nJJQw-h1fd9W8rNSnXyHT3WPUg5Cujjzb4h_9TVa2AGJ8y4N1SCBYBUjdi_
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGkLwopwDetTQrsegifWh9UuV_yswZWwA3k08-dix9ihwtwEYvSs0sv9FDcGTxufBMS5OiJos7IqmV_D7_WutK5SPmipi05T4F0pIYFjKrVvztptH80tjD-1t-PAsvwHQO9yTNi7oZmRm8Wmh-eZ5opX5_UefsRX-P0
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGn27gmMamH2FZaRjtEGLPF_M5yQbncsukAS4PfFc4ntLSpb1PVb1xwkMJBNbKeHPK0GNgpJHfznEnLG-VlWZ8za2wFFDZBgH2LPhlhyqUYvLI1ULYZWcc8GvZvpRL6Sje_8HF2rnwtEW6DRdYs7Hm18lNIaeQe2vT3zZ_IZpDs7MwpLTWG-XmTzCrrcM81sjTpNA==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGxzsoA4F7gX6qkGcuZI_EplzseqgzPYEe3s7HyTJsfkC1K--MLZ5Ackis3zyLk8Gky1KW5bJbba9TEtR1rYFOI1EHhkroCoaQUPcUAkeVeI_-OpyyABHai4mGW-BToM4EuaSL7FnAqGHuAv-tA5g75P43LgM5MXOgqZnKqlBIri-kN9MC7xbXd_86NUiz5cRRACG3URu9KZEPVtn94-MQ=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH5CSXklT_EA3iI2NLCxQoHQsB77NAy-UnRj5_uhzeDmQChVRcSXKwbv9SaX4BWcVQgShNbCDH-ZGUgHVF9_UCTd8_a-A03Q13sMlLLggP15eInFz7bV7mAM_ZtQArFiGwYM0xzOg0SsKNpN68jRFr6yzpgGVM=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHJT-Yh-f8K6jinJtNq0CwMPWimgqb8W0yczGkNN21HNttK7FSUTbwN1MbNRTVLpxgbR1bnsddvtkouaFveMqfgCl4hUulmFcLYPmvYfXvGqXueS7GFWGL6Y5Nn-rzPCDdJhijnfqPVBnkJisgc2gmvkOcd8jdIvpdaiN67szBVvkv12kRnclkWrFdmE83rSZL4jXFfIvSKyAip0Cc=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHZN2P8-APWVKJ5BhgcJttT055BI6C0Rv5EN3HL0S_-7w5tUCHl6kXuJ4P7yQZXhQtY1T7qy1vgTHqVyXRSarzYO8ppZnrh-CaD3x6mL20OQRwwuz4aqVfAMxBGtHEIgAu75WZAKGIJ5tPft_CvP08pPb3Pq3pyib4aZmshTdbMCJT_SOtc
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHb_FUfWszeuk6TJVDBnTqVx_PrLb6Dp79-mp3cmOy91f56Ia1YrTvtYnJ4xTe46w0fJFZlYyKr3zbe3NoGxnryyuv0kjdRiNfTwe0Z-pzN-WjxRFd1McSZx0CU1f5rEJSP4cPHZvGiyZOcQtgDh8M-Dfu_VnoetY2ueb3PPTTPopVrKwgl7XOnwobc4jN--ij2RhhMfjDHSWLYqzIC6kZnM40iB_kCCQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHgHZHSe2KSKZo_cvkIsv9JBI2mqi4q_AozATKtaraFc8sPaqAwcwiQSGq3dYCS0xHI2BbgobKxWa_xpgc70710QkbSIcgnoM8xGWnC_arhDpIOFhQDfn2n9wEmuDHAAbQg1XwvWnv8kpvwX4waMLkLeIkY9PP4nCtX7MbT4-YodQEbkIHrATZD6JxmfQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHgeIK7OLpzcKRydh5eZoRWlUAVUlXyUteFo5zwhrFO2yhaxENvB9v6FCSAj3_7EQgXI3RbfCUhzAMif8GhaEyYvLftZJsyRWv88YoGG9FD8fqjjdlRazI8lOX1uEaVeuyIGlGOaxDttk2Ej8XYm1bfm7NmeCoRW1j_PJ10EOFXaY4fpaVW9cyFwaoCDJHgzCYRihx-9cevYsAIvwA=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHhhOiiu8gwkDQ7XrHViGCHIYo857FkItWOoKC7G7VZMZMaODpe4Z77ykixzadeU8RjQFQo6c8Z71KVDlUIYicMp8Hws0c5WHneC1xDV0b9pONH0LfALhyEVT7atWMx0qwtKDHwdy1fPjUF6Xq6xWoCaQV7C2UMSw==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHi_Rd2pzmYsbVpaPfcWY5T3CJkLqbx8Oo_ZrvHIZ569V1EthSM1y5AztjxIpDYzBKH6-gOAAZxSh53nGs4K9hhFeUFd69yuWnsE57UMMI6iflKnEMACSodZ7OCdlZAmoiY-iMCP5UYz8VO8InCTpjU1zytpuRySObggWcQDAjTqJhisw2qkwY=</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>BT-203</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>advertising</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Planters Peanuts commercial advertising display sign or rack header featuring Mr. Peanut, late 20th century.</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>$25-$99</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>5</v>
+      </c>
+      <c r="F37" t="n">
+        <v>10</v>
+      </c>
+      <c r="G37" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H37" t="n">
+        <v>1</v>
+      </c>
+      <c r="I37" t="n">
+        <v>10</v>
+      </c>
+      <c r="J37" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-SEND</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>grounded_search</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEXnHCqNepRpBu6GFxO05HHzc8ZWSyoDGMa85E5o5K9CsveNEIFhR5BBE-svELLPl54b_78Yo-Ng5Rji5ptusqgk7wfFRcB0xlvhPfCb7Oo-j-YzFLHhbI7LQV-r3CkUmaFpS3ftk3Rmq0E-XD6WBedA8rLU-Nsyl9xjfc1g4_9u-cW0g==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEimKgUw4MC5IZWSAJuYgRPbeTQ2Zu0WUPgHAJo7XQa8am2nkGTWfGr2Qshun7fac815FqPAIZwE9-oZ1XsL3P3MLjVUYIq2xr6YRxtm9otqQk0SHaayFOlLqtHhb2j_8g=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEm6w1vxeg5vd31hF5cFYw6wg0go2Mq3IPZRt-AB5k9FGHqcDHZLpGlyVv3gIKzqRC4f4qVyYEe5H-cr-SkMB9UNN3OfqNlkta5A73il083PdS7-cscsugu4U3zaZ2FjDUUIHtwAFJWTalrHP2WTRjSsosFLFK8DtS6d7jHSz0M3COhvQitEMglE3CoZXDQgdgXjw==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFR5ml7cYCYQtSs3wjMiwgDoSbCiTV7rX-afINZcrc3e5Vdkm7tv35ItRsiIp7mJAYIIyhBNyPIr_XvcwkVXephMMiu_ByHzNMWqoZXmzOYaqy3F7JGxwuPO8LaQAiTGic=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQF_KEyblnfmnW_YuDXuZrnGboyAxVaqb3zypuSThq0l6Zy5mT6AJ8nI0N5LPZakJV2Utvm8WoLoGvnnMP9qfQQcBhG4jWYfvrrvlWimo919MZBrwhoUgZtZH61abWREx4mRe_PnriXVRB_syegqPHESVcxaH4dg
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFj8hVThOrLT4TJUQW-VIzehlHTXPgeO0FjkJsVGY6nBGu_SFesthMtY0CPO5Dogo4L4u3tsDblj9ymeC6Ge2oaWNurMnC9ZS8kwKwNUDW4a40EVRrhoZlUOMFX5DCv-IsNHh5-eDPK-5PCoNbz0ohNSlxU6REqAMeicu3wOD0scm7wtfwxhso65FrEmzz26Q==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGfR2ksgdO6TEp4ZuJPMTn4hyeDWL02RbwPawhnXVZ8pxwhXhcDfd0JzmwYUKELjKnCk893IJeY083wXy7gWfBOqWClaqLAMdX_Adh9i-uWgTR4w4eap0NIJHDsuojsayx2aOg6hcsimXR2bhDcGTW3Qu_sRsPrkA==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH-fU2Q1qMzb2HDL_rejYR7iy2p9J4QsxowIDhDbE6xYogasv2ZMXg7KDg8oZgzFPdgkesjqmTxM7Of-F__UrYi5wS0FC_J1oER321zfjNNF0wjwWVtAV8T9g9iRG3kmR8=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHEW2qQODSrsvo4jF8DRQheUsmuiMShcYJv2RRF1rX85tYQMSMJUK1cEFEhvu5RfhPT3DAnXNabBIV9FvcoXtJkRsvdoqoRervSyumKCPAEIHK_9ZtOCR6rAoFMl5GoUg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHO52P3hwPDawgwPAm088RpK5h9qBjX15FKi4EGtrD3lIn_uMsVd9L49cw2IHYS2IWjhHr6JbvCRIxxJs7ZRr18T9lBUMRLdVEoZ75yqUYXIam8BNVUBIE9s56tsfTSH3AnqPT50Q3Jl1n3sF1lmYzMm0hIXAP1n3nLjybJ49m6AYfX
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH_ra1zQUfANkzp8mMMk82ZoKZ_MvE4Wncte3-lYket36BenS0C6v9OuLD1I_awHrai8IhwKODcD0nsWqjxWlJmegqaXZkQZkih-xs1OTDqlUqlprFStyAWskuJhGjq8cUUG9oN3gUQfZTmTGB5q6RIGUi8anrrAqnwNFaIfz_NKpM8tcKRQUdkCoPIn6FS6lgEBQqUNqLSLsikupeg
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHej79QcbiGUiOPWnvTNEcWtG51YvFcCW6TFZ8hIFdvrUjshwjzmhrMxX2mwaqS29RCm_DWmXcGQYDyLr4D5ZXtPy3l4l8xW_yuSmS1r8GsOt-OmmWFPPg2n9k4w5g0bojzvjei-FU__kxHjFsl5f3GgFR0yPTKrg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHm772TbgLig1EqP83xPx79cqe9FpH3e9qTi0SKgQhY5RaQUN-wvfg7mwIuyJW0ahM_92sNxQ_oxlqB5M_QRF3X23rU2y8te-e5weTAbbuxJPfLbhW2yX-6yDYMvUWztk_rCd_o-_0h_yFe5efWStAXAJEEdd-D9b5H5i2ROAsxSSP_Qg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHpGN7kSSjBcHZj50UaSmhgwscGhUnn8vpIZVZWbBb52NIxnBtiA2WvVVyNOsnIwssZOHVboGc3Xu2b10MQjoY0wGXmsv-8Pd5-31V1H1vIhDxq8c12E8eT8B4Y7-p978l3K8HzHTFBWrF1Jj3IhaPoFryuJVyp5BK092qnKOMECduN</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>BT-242</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>vintage toys</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Lot of vintage glass Christmas tree ornaments, including Shiny Brite boxed sets, a Silvestri box, and clip-on feathered birds, mid-20th century.: Shiny Brite boxed glass ornament sets, Silvestri boxed ornament, Clip-on feathered bird ornaments, Loose mercury glass baubles and indented ornaments</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>$25-$85</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>5</v>
+      </c>
+      <c r="F38" t="n">
+        <v>10</v>
+      </c>
+      <c r="G38" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H38" t="n">
+        <v>1</v>
+      </c>
+      <c r="I38" t="n">
+        <v>10</v>
+      </c>
+      <c r="J38" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-SEND</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>grounded_search</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEE7FQ1vk5rcvOKyY73GV-_U0efwIp6P9jVJ5BTJDWGvM_Xj6xB6981w4zqFzf-xTcp8b3lWdPa73nGJbzu1NmGNygYQBWXOqWxwFX15LTcWM6CFRLyrCp8yvS8Ki07C8AqjyniPopQ8F2aXeHkpL1IDg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEKBQI9thiEDG8dOg2YhSPn-3VnecN1zy1YYuEz7byutpoH7OOJ8FRpnUbzW1nF97ztqqcelH_RrlON9IduWJw5HVq8rWpQ3han-egJ1FeV8VOdWXNvEAAoWemVqamlxxtl3v24UR7S-s9b
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEVnlH_v5CNNRggTH6rNOEaQUiSyoMD-FBI9uh9vcKlaiDZdJwFur0BTLrBGzY6A_4i9SfBPXXuOjEGa06mgJK1P5nHrrxLPFBOsmDPY2D2LKDKj7mr3PjUR_4Hh9CMPtDNPCsec3tZ1pxJof8Or5Wr2_MgEtUlpHzP89E76R5geZVplyrhbWcql5KkcqrpnBrGm0A1yjdoFJ6XCFvemynNwpYXUzdHIQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQElxLWENRdiYdBrmvcib9ox6iCuH5AtnpNglc8O0pqJ1sxLnwkdp9cr48mDUtEFy9slFlR-pcmg32GwRJzEvmGznMO6oxAjUwPk-FXzT8CdYM66yPb3ELYEQaakkCD398ALoFKtk2ZejsalMvCVsqZ3IwCgrVKmQnmkWaH-QgcZmZ5zYm0IOyaGU9f4-zU9wrACZTGVANm0wBOwTAg=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEwMUYAjt-XesS5qKomCFRNDUuLFS__7buJiKU3eFsTmLOzsAVCEkCUt-VgZbrqCOm75M2bpKoS2caywQPDsES43XZCXuo5Aji_J8lJ93FaOe7ud7JQ3vQA2XoPdjvhYNqLAvXi-PnZZ3uPKP6VsY3o3y73uPnReHlN6ghQ3QosnsUDw3BI94i5TkSJug==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQF3rsBpfVLdtPSlW71KsdTZUjHf-JtZgHa5A6oQ3IOGaHVGnBRBNtaXcg3XmZzDoRGJduNVR9LSxXi3UaFmenomaGHttUQLGXXq_9H4_rmhy1vvi7d5YT8bvLOblHdqkLojyAFlTrT1HwdoWbPqY4Q16Kp59hhADn2WIui0yL1XfFI8LA3Uus3OSHdxNw==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQF4uPer5bREiaEZwbI5w8OZI3a2--vsigchEOeN7XC4L7J7HswF-Qxt1YYSMA_rzn3vjBUV2cvCvwE-T5WACaZrKZxGTVBX_oaqbJz5ZF1IiNtwnkLhIPJAhgBHcaSr9g==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFS0-4AGfsDpfzQsg0IRdq4tX3Zk4GTWg6TFns_GHMpe5PJtJe_Zu7ssPvc_YCNmqn0QvefBw2nQ9-F3FxNMDheYlYdRNK7jPzG__oodm46-5ePI32MTxlzA8S4ybE5dTQwSh_2RUc3
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFVklm1_v_IZHIfj_YNC_of9YVVlBi8qZgopwls_zJ116A68rXUV2Xmp6fvL-QCkOy-xU2nZqKfRwrzew6KUAgsW6NNhum2jgTEk7SgXh9CTgCwoGTs9--7MALWpD1C0yNqmq0csfarNedSboANknBZy-ftIbqv9jgsMr_iDfsRCikPY1A6dp_buUf-3geiBcQzSuJGIr8fL5Jk2aucdImqLHDmuRODm5NeFrRVBcOmF9lMj1-Vmv4I99pAMDm2_A==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFsiFDG9tzShNZo3pmNxcLit7iqYFr-q4JkgflGFWqXSZJggRVHQi9VcEn1S5yt30DTkeL7gL6stTafYziUGzDy2YnmRD8ziRSdKwyY2WRUk2WZoMGFVQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQG35o23WFCJ--8Jqa1jPyTQUxGG7QlEgRpHL8hy8kzVowBvAERc2AR3wXsMvwJIfDxqas4R70-SJtUsL5SFq4NSVqE17KXKVH5ufcNWIguxoxkaLzfAhDZdJ8vshSK1HimyBusp3Wrq8bF4ksu8nn9RyoMPhA9LSthkEvRks7I8TRoO4NV8m373IJKcS-1n0sG86b68qXfoSFNAuEjM3HNaopIn9sNfqdOq
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGHYoqZJk4N3HAFNwtWL6famubek-SjuChvoToNKoY4F9-Fdig_v0ppt3NO7eNu_HD4t-qLEir5ANWrVmZ2d1ymmk3NqyhLsc38luWXTshjTM8mDxJnl5AxLy4U_DepAd6W7PQOgQS39HmX7VGwqnZZ36IwCX6tyuf-4WYJq7OS6X8IaeA8DLB-RmKnWv4DEH131KJd1GQ=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGQ-Rgm2czT9SpRI_aQN3Dl3x4nowWDz-lOMe5w4UyuLmWm7mZXl054BlsO9_dkOSI5M6Acr58yEC6JcOfxyMLquLTnGSOlYC0yp5gvZR2s78RZpZXCmEt5Wiy97j-FMbCTdvU0xU_LHwZGrCpnktFLQwSS
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGRYgDdlARexQRlJfB8Y_Crpli52dwHDgnF0oKU-yLnuIg90KvYAZmHMOwVCEyt9jCrZXDAw5SJWAEKOSeb_vE02GTSvFcNCRRJ9pedR1KwNhP3g6D08dY_3Y6vh-a75utiRX3zlw70U2q10Dxqlyf_wC5eMRJaZGlD
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGyHE03znlZbCMgiSKZ5qnLj6qYN12k0pbeBBkoy9KvMnUcydO6ZJuyHpoHb6ztV_lVb2WJfS7vlphxn86Ob4anYuZD9m0QEISZYwN_flIFBR7CqcE_WcuKrhUGX53Dd0CIYYn4bOQXsaJ-pZASwwIlXeLif-UlLrs_yAy8BQ6t8ke3MIMi
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGzK4js5yXkoakjlRtx6UsmupcW-_dRla0ubm-lOJYB4E6JSgbzmMnSX6Y6i41ZREB7TBhRf-OmY2rAC5LVVt9Baa90JfASYmtK6gWY7SZ7J1MXa7pQtpXJqnAvXofB6rOwl4jhLpdVNRX0K4pUUFpdtc_rUbA9fz-bqpEoY2f-W3b21_a7x7TlAYwWbEJTHjxVFusp3ryovJaselU=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH79R4oo0O9BJe0mQhC1bfRhEJMsxNsSQ5OCHMweRlPJQhwd5mcmKqDAkMYy9s6WwXKvP1iARFotUkdREMjA0PNS9LzmxahpcGMXIUbNwhUpFxtiJn6ZmS1DbFYCcaxK_0ymC0nwh7VrX4k9lYfSVpxuMtTqvm9z9u1NB2GiwdiH8UjjGdJgA==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHhwCFCrMh7KIOVfZnMMPP4Mg3oNeL6QwXfr7ciRO60xhSU12W5PYl9-62mbBA9_E78dNCGiMBw0IO05AYsiDWCAWxgUNnpL9cYgyn8IY1pYnoSTHtD-3L3i24Wv-gSiQ70Cinoqd_LBMENNJwTGLds2oDlLsAYEo4UqveuIc6OumWn6g==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHlbmug4KDbtlnERI9XoUeHwBCT3WomKsmQkVpBrr6IN37hi9cNjAVBP9ceaSLWJYKGi9_m4U2Ofqz108hTjotLYpOKADoIrK4EQvsZOutyJDZBmFImApLZermPoasp_PkkZIm9wxUuks09J8LaZXoyZk_1DmI5m4PFoek_RwAP0bg=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHs36-sODVVdbss5BOjrq2YRZomMA46F-ek7KxEa3Tq-3XLlYIyKo8TQKMgTgQewaXyJnRl5gJ5i1OTHqZ3Eiv5kpn1DXAXKwvjFcWjDWsx1NV5Nv254ge9ma4luSeKWUJkiSV1x7i_WNSNZDKt3RfVqWiiAD87VJlR
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHvu7BPnBo-dSgcRMvnwAr-Iz0NzzwhnBGOvbvrFnXN9Il1wzczrm8OLJ9MaK2HvdCzJ2tTPRrDo2fSC_uUXVH63kIabZIW0kSctR_xTMmelfQW03wS4JVaQSpQlYv_nCiyKsOP1XvRHEjmDm55fWlO9YTkMk5XWSVGtaoY8Gu9Y9agyN_4</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>BT-329</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>vintage toys</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>The Tiny Golden Library 12-book miniature set in original cardboard display box, authored by Dorothy Kunhardt and illustrated by Garth Williams, Golden Press, c. 1950s-1960s.</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>$35-$77</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>5</v>
+      </c>
+      <c r="F39" t="n">
+        <v>10</v>
+      </c>
+      <c r="G39" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H39" t="n">
+        <v>1</v>
+      </c>
+      <c r="I39" t="n">
+        <v>10</v>
+      </c>
+      <c r="J39" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-SEND</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>grounded_search</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEKxu1pAzPucc4Eg2oAhHfNCUSJAI-U9ej9S4LmKs9k_QcL0ZAFTQWetL7-sPgSJBj4Txtc37toCV5jkkrb-W7w3OVnvh3BBIxB5XCS83cP07YgyTkSw0ExJeG8Vo1WoquiUdaV0UNPdpRqu0Hv7_CEFe4DUucgBfJk20CiaB8q1E510sMNsMM4GNyQDfjL2ENMMZmrlrq08WRmOu4A8tCIUD-VLDzE1oC7GxnE
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEWqOwFXGQr9XmMe9t6bsr2lbjhpvXMPd7aC-bhGl2L5QBgPLIpG5WUFHabKcf0kpvOZcFqgfHUNj3onXgX9aIyT7Q323xQIAH-x8qGKsSOAcm5e0TIvH8O7e2niDYJdNyEnoSCkVx2zFWD7Cnr6RLkza3A3vtVA1TLMUctq6uZVt-8YyVSMSiznp1XPvDtGUUttCTbffpqfC1Tvh4U_Q==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFMtiktM1QTSvIw2dDDOhw04aecQb9_G_sLOgiv1QYxLipExbbiPJgdHWWgd6o6MMmEO2Ywht8-40WS7YBea3ZiJy8qlMMg2NsI1QBmHKECeqyeL2U7rjgfw_6BoQVffk4_IC_lH9dhKG1GBYcTECwXVstdsS9khC-lxZkDTVgtijPTmoCI6AUYwOM0oI6cL-6_sEPzIvxiXXP5KU28zpOd2_7jXY8_yioXwogJ
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFXT5d-EHGxafXn2hgRCFfQbN6-v-4r1wysK7nucctX5o1assbKgCTNCtpV92EFu-tjmHuykKq9ObviF1y-rAdIq2KcnXJEAUhQEAq_IzQaORhzLa2I250MdYxUijdsKCOMDL33tT8WzfKJ9c_pCKhO8pF1kMy2VP4I8yU=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQG9TR40SVEre1oD40-90PrUT2if-QkrMKtzKRqCWm4xag_zmfk8VpjFAdyJJsPLTdIKshc2AudZ9d4HcQkJ__cLhIl8LM9uaCiszLsQNwFOvDInuqY-ranJOr_ngKneTW7OcBtTp_gkjSZnKCG3Z0mC5lWleUlFSbbSfHYNUtChOib29eOKMvuenEmDV2-zPjACJYGCtoMZ-p-HCq7mSg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGDDxUgSqtHvhQmje1Kkj--e45t7P12yiXL1cSpG8YUMEy2MQYwDMRpdSCzmFA_q7yF12NnV-cGVhgeBtutr69NQPEzWuL5sMlxWJkwBOjOxox2opttSKAN74Cl_aq4ysk_vZJGdHpiyvEYikh4QJpLsO8=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGFP6Cb9rw520FU2LIMbI_RinsQEK4R0qvEWzid8yD3ILc8I5VO4e3WQdjgYm3xt_jvIHR32fBEgnNq6FPzF19yprW7yyXhDPxv3FiabkPuHI0OVtyxCJ94WKPzNByofj95uJhqyoHicFutqHVpT3p7-3-1ov22riqlAS07H_rzANWl4dDbwto_RFljh6F958u6ajqNvKfoDvdOocXIdX_EYUU0CMtIaU75f9yr
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGyCd2HfH5IJh0Wb6efkRCeWl9rqwgfvuPJ75g_zc2D9mWCHUiPk7WlU6gWr4Bgk1L4tvsPIni1JBbxHXmShlo7YVZVvNcIYQLMt1Xhc4KaIVl87Cd_tgBF09LAYUVw3ZxIOUBINRLb74ASZJ8NUAg=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH8V3cyFAAtp2p4OM2FZwmZNNaBhLCJTH-ng_YCzjJLog4aF_gK-necZTqAohiDk2b4drAmv5X1taQaSop0RpzgARv_vK6NimG354k5khrtrG-MZsLtsEpU664QGTurJAQ_6g0G-5juwZWzEeH9PwZq3aT5pIRnQEMKTUdEm_CSuzIqibwOqseJeuB4jQTviZRRKQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHOncsoqGq-zOSSlFWJpDHV6HgevNnSyXUskcjE7zZkip3HkPLof4FTjeaSPT-7X0iW5hB9Qn2FCWlArgQKBD1u_8cLqGk6evqOk0mFBy40Y2icoSoqX_ilFNpN4JheuMLk4IzSVJn4aw==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHnASK0OeCLJI-2rSdfOWfrsFCsddPjt1KjLwMivYA6DyHH1YeSiVzYqwCLBmyzLx2xKQqmNG9Vx-dcGAvLe7o82Lt9cXKjGyqyHsrv64pkjRaM2coAXrVReCe2SH0rZkI=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHnJNDZxvc0VchwtU-YvPWpXd3Z8bnNx8KcFSpwT8Gtsn2hHNzjhqAAmEvrwEMjsBafCxoU5ocbKDUy4YGPUX8W_EtceYxtWVOwdsYmVo2gigLgFQn9oIGIK2Afyh5fouTi7ug31pgtWrL_k1c97uyRjKvIMaqmBUuJCLBxU_MLngQGTptn8KZpjteA1aqZiA==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHvlNw7NNlD39BTrLH6yRGBk_vS57SK5rjpcN6qUErDB74b8Ka_En24VfrAfWrKIJ9vU_xBSciwC9T0n-0BKdJhbYC-Wmz5kC-hlKW509tuyVHG6ZlBP-jNBSNIR2ADU2M=</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>BT-332</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>railroad</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Dietz railroad or utility lantern with wire globe guard and clear glass globe, early to mid-20th century</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>$25-$78</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>5</v>
+      </c>
+      <c r="F40" t="n">
+        <v>10</v>
+      </c>
+      <c r="G40" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H40" t="n">
+        <v>1</v>
+      </c>
+      <c r="I40" t="n">
+        <v>10</v>
+      </c>
+      <c r="J40" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-SEND</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>grounded_search</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEkiKr0emnB5EFZ5lGLdXy8M3bFyVmXwOaI53ufHj8-PYaHfyzZXwSRZIvkihSj37QnOd6t5XhIiED8fNYoNNQ4YhD_Uu45-g880ACsPc9-vYdfuzu-L00hhmNBdbUUkvalLxV6fDAr3IP3F4TxcnrzbfQnCOYV5ONMy_5uAlrlLMvUe34aRg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEltAoNkKDukEkPMW-W88Vyib4iW5AOEu_CovO0ExACQLDSTuM9QOicH7d4R7KyM5xYETuDuzSBgIctFlDdNbAsy_EvboP3k9lHUahFLrOON4-Bgijbjotc6mOUnM9LEc8wPbjcxMxvGtEHudV4v0fyz8hSLThDdMp96S4wVgagVVes7_lJ
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEuDrq2d5UHbLNYXstU9RhvJrU6UMDZVTIPh0RRk_pZYgkRkYV-M8yy9-YZptc7XPRVWf5tu_vUPFiATmpNQRk4-Ez32Lpj6sMC7DU8t647g2M11mmmxJz2tkcf0UzYy8qZ-3vBDyl3cWPvA5NiklWYYQNC
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEyFpqtJYyGpJ4OeQgCF_HMsXnIAY3e1ab6m42b_Go0fMAGdd8DixtzHDeu2cBlJYIVFm98Qpmf-aNPne6yACAzPbfdketFzjq_HoDsjdx9xDdQtP5pFvQzAC9jSg1XcOv2I16vWB_Drqqv_bnFJUcQry5BrQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFv9HsPy7UEq0H4992R58WiqT4mZvdxnvbSBFBVRV2JPWh2uL-p5JeXILsTDw1IEY10XVKQy0h1a5nCnoiwzklzC6stfd5ALhOQ655kY5QeIUSfGD7RenYB6m3Dwvly2FGSn1-rvOXszzLd1JNuR10X7TPxsbWPzJ-ncPsmikMcLkIMww==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGHQzxT2JLMi6tx_r_Ae0c52f_jQsjtncf_NPUJi0_F9QC-Ug7EWuyKqX8BPOxDsy5ZvdPyEyFm6ldAtDIN-9pE-aRdkkDvpDciIPBMw_hMnEmw8HGPY80U3RFytWdAZ8DNUHOvSnJpBxOF3E_RZKfR56P4L0ueQAn-ViO3r1T_r8Ht9o8iy3ahJMmc5socm8Q=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGlM1jaeQLEvUFnS5-jjKM7BpAmTlc-eEgRMvw7nNfW1yz0O7fR5xlOmkNrWzfX1QxdfSxl10Qd7NVKxE3c2SyQ_hm1hTtlokTjQxPauoToaWRGd1mxbbTPBx8WxhDqXtGYujq9a9Sfvs8EvJSwXgtmClgZXE2U1SZMoIuXye1S8eZI89tery7W2cOvSg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGzlnlHwZg24jTEzDnVo-pyfRatk_BdT8KM6ddNuHrXELDpK3XgmXdo1GHSfd_ihZ6ps7x774iij1J-J3FY2NTnaNfG-1W1dY0FZYPJt0GumJ_HfmbMBkdoga7_WiOxKXcXx_aQ48RcS1FYQo_O3GCJtExtS40KLLZLMWf77olTiO4ke8c-QOc=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH8b9ObljspZvGgraet1thW-d0UJ-wZse1staOMfcCXgdTwyN2u1WCj3zIt9js65yHuGQkalPQNRRGz05rNk-FycuYVqsCxKn-NhnzGV4C3PMMvdrSPo2vx8i_TkYG0kZQ0P1soNyYTMiZvNZVQXCsROEO_g-I_4qV7Xu9alaJddzfaSyugHPZd28PrXATm0N4Bc1rf_fDtDNx8FCTHwj3-taS4GQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHMRj56LSc5lpc5IyaHhe_5G13yi6Inut9k3597YQrKu0siCCclKQlghrGIsCs8iALLtlGQFf77Y8etbQhYqmVl7fxg8d9JmVRyNYUNUm_bAQG9_oV-NpusndxXJsqzAWf7bXQFvYGD2RPSoRVhk5y609L7kbHLYeFyL3Px
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHQeLdcT-SZmZnecE-Jj4rFhUjd7T8968z1AXIrP3RnEf6js4XV47C2esS0nO0WRW9FuuCIWJkepiI5aKbiVW2fv1POknO-yMJznuGE6h2ZnnMianR1ZEPtJVlSnoKu3BVyDke9SfRYUQJWAHpJWkZWswilSyOZ4d2ex8bbmt9bt6c=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHaqVZEEtVJwCHme0qFhx12_By9SDhmtwozYzIAOjGDYJpW1EgYvxN2YA7TP_NBhITyPIM_MbpBGlotfRcYZgbkq8r_aj2OBq9KrFjCgpBywe_rCEDdZ2l3yCXWRPQQxkgbbeNUvOz-jZioEQuMXMcI2mp9du_FKyRHcY10
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHrC1c_gNkNu5rLw8ltMzpKCRvD7XC6T990A4MkwAUl6VxmWml9j-VT6sqvXqSGeOh51rgc60yoh2rIxvvL4ExcigN23D2RN8vqel34ZFUPJAwN6fhr8kD1qys0Gdg-8nUTIW4OBt8YMEcUqD-SETn33r7IGeULEyhhj-r9uPIaBfgyYkiPRTNZ9PeA0OOxHm1j</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>BT-348</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>advertising</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Assorted advertising novelties and collectibles including miniature gas pump pocket knives (Sunoco), Budweiser Clydesdale 8-horse hitch wagon figurine, gargoyle orb figurine, and boxed belt buckles, late 20th century.</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>$30-$85</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>5</v>
+      </c>
+      <c r="F41" t="n">
+        <v>10</v>
+      </c>
+      <c r="G41" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H41" t="n">
+        <v>1</v>
+      </c>
+      <c r="I41" t="n">
+        <v>10</v>
+      </c>
+      <c r="J41" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-SEND</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>grounded_search</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEH7uPR6jLoU1HyRQdbq3ChOH5qAXlCDJo6giKy12RrSJjXLytzHTBeEUxH-_WvCdN6IhHvy7-XRCKwOQmJxidyCdjLxGVuw-ID3s04mmBVi_0WllpatZUt5-qi2s2h19Iwyg8WVqZQTzTM4rwVbO6lVM_DprcoRPm-X0gWJYeVS3LDMFMQlPks8c2Cw5DjeqKE9GQn7JbdbnBETg8spzwlywH_ZO8XvxFt0eHeY4RQuswc6w==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEeGodGT44khWyPiYbdtWUlpYwSgzYuB6oCrdpY6SAFqpZWzmmd7oyAC7XguZXb3YBkj9F1l1id5uIRwdXCjfcRvboVFvLSgBLasXYQGZFvNkwMVnrCYFnUAOpOWJf5A-GHJmSZYiyeKIVcJrib3Z2avE6Lwh9O-vQnsWJ8wm2KVjXkoquXxv4ZWaFz
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEhHNu-1YfVgjIsyMjfKLxuUKWoYrqZjD0KN2ZZWS43jGyWfiXUStz2CH5CVRP3UdUyMSqwxvu1p2m7xL9LlKUI2jRDwH35_uwP-Mn9qCzYMf32UbQk1k9y6AyctmO80lnDBiz_-k0VLywOKAP-m02We7MeB4kN8-YQjfXOwAp9uizlBmthwZFZXB6GWyzcVXfMGEPlSZlJzY_nlAWOl1oZWy3HHZ3q7A1Xithpc4YHHOmrswJBjAs7EA8e8ZOyjA==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEq8b-UEKlepklvvRbdDNlMXAcW7sMML3cSm3LZuauRMDUogcb2Cf91sC6x3IadXXfdzCosUBUqK44hFwBUb_lkyo9BqFOZ71WovfDyDfLZ-_Za-5NLSkg5cQ5G53yJc01ouGkk2JGuYtQVHR5hxcr9TutABurfdYgCObPOmk0txij5Qcs=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEqDF0nBlPVPD5x3-mlz5mGglGc37bN8AO0oJa7BW_h9t5P4ASYVv9y-7WjOkOP5K5ms6b__sZs1js2V6pW_5oQp16Spfc7Pb5qKS61OrXrHtcvIAGLGzkpIx6PbaENEJLVDsibol94rQEjbOuGsmv1M7MDCfk-w2x7rrwL8_StzYUhNMvc8u56oKzBNcud6Kys_uBfQH1MHLhlefeo5IzTiX3a6omDhd7sQo5dg-lACFNgpQxoO4Umdi5ZM7R9AvVr6lKH
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEuFMV_Wl0ankFJhtgpPFKBx542Pfm1qojMQXzUfE0rLb8iSHhL7fwE96_kh2VlxnS-JHyvNr9OciskwgrwoObzRSvJNWemwI9JTdhflHD06ITyQKfxtILSxe6b8yawXWG6AS5Gm_NYN1qfnzl7_tf6uvMSQii-1t0oHq45_DbxG67VRN5mvEMqxOx-z1tPhHFSmaYRB2Ybow==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQF5PE5Lx4qDAHwHL7mIRSkbM0y-d31mGfNA-A0QDU_a2qKoleqkR_e5Ks1oP9-ptDcEFihdtvFXRU4fZbMaRo2ysdCAQq9CVZYiO4fIfe3UsbNsBJzEAtLNxCPNrij1fXFq-hs6YIdxCFOuUzN4bv-lmhQr3v1tBeQc9Lid7n0suIlWGtx2h5jzKeVL1CvOYLYmt6kcx01s2CMkyzRarOU-
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFSM_qXvqO7g2VKUPo4vbofHEnK5JGB27QInciRlBHZnGpugSHDd5qjVexui3b-jIm_TzRR7LaA7gF0AqLK_sgQwuqcqoX_FCzK_qwk0Y94OLgGlir9FA4fYH0DuSwJ4AIWJ_GsbviIbkeR0BX5y0ocCFIQiobUcUpdyxAtExSo
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFTt-X73QylJDjQXTaSHNSsXkkBjglFiTbG-Ok2IrdoMUZKzj2EFZKCIWUbF9Yah7NK80HQChomS2Zt7TXXTh91ANHmft5HLS2rvWPOB8H9CiH7nE9fx7emdaPm14_vDVz0sk-p_S74Uol6tW9ty3evIhRi0-BkLrwPhmT7HJVifykzxN-b1ZmamkcC
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFWPpLw179Fq46SM7QGZVEFBEG9VuXgplhuLX4DtWqi_x5e8CBbEZcSS1XNoTZTS-RU_Q-y4SYqcmcT-S66K0RXqpsZxFoJzCOrS9qx3yK3dFWV-MxphHmU6MM3jCGr45hN0BeUm_Tc917bPEAMfcXcyrcMB0pRShuw6g-z5V_d1jbEA9vCNSn73wtoEZZqxmOnwLxO2bzK
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFojnZ_aG4zkiKcM_THumRMPgNzGqWs-eG_0aNhCPXV4otDEjAnt9mUQWT3VGL1OaMFGp5YqEBfBCDaUmha5I5ERNKirXgH7SKbQhKB00jI8YZIZgrQ1J70ldjBov-zcDbPqK8zG0uRJhyA2lv6jYwvoROL02unjxLbDbomtCmH-j3MVBzy2NO3WDIJY-mn2HyiCYcd2PP-8bWKsqm5mFQWS00HGaaZpgQM9LO89GJROzls7QtTA_xIpnBh0XVNpIjSbmF4
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFv5ezciVkfhHRpglEtVJ6YHrBrHocwMzZ7ViyxXwQDw4-MflGsoL_R370CfhqLcU4jPe3kDEolEs37PRsXBCjLMITk39BB-ALnBQAgs9mYjMYLLC4TDZhA7e5FZtS_HZ5gH_RXBAAQ6zKSRFXZSB8DE851E0XaTIoxJWmCf4Oz6nwxfmA_NzwS569dgIjWc35WICXL
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQG9se6aBjCmHdUfaBoDxyKyGmT8Seo0lmrGtqCTKRciCOCWX6wSToVYaZU5xdeLuj3VM25BuUr32T1vUlMOLpo51iFwh4oaoAdDSmRN9cf5G-jGUAIEUyBwoW9kSTpbx9PbQAQThhTE
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGF5CJfQ3CwmbrCD2GCNb6wW1qjYL4AClu5WgNlNsEBSx03p1w_qCvZLsgGLjOOb4ru77Rw7FhtR_j2q0gCaIM3Yc6SbZZXTlQTZTLW7E2zWMP4v_To83TNWxcy2ofcR3ICVQz5hyalQnGjcF1gAhV-u_7ntvhpSx_lXIK0aEtjVlFRm9BCI19fwbq26-c4GRwgZZ1370Ltz3qos3MZFkl9c9YoodX2bN2pAfEARO4EV4ITw6fWU4HgyMYXEEsYnQMcBR9XjGVarg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGmy6AU_BT7yEr9oGj7caaDlM5BoJjECGvIuRHv4CQezJ9F7OGRVEd2x__qM0XxBe_e4XpGA3kSgt6bsM_Rvy2Kx3369V3D7unjjVl5PNrFzIXAMBE3nUXavhae6s8Wnjcz3NKRTegaeyH4sgMkMXN3uWfcQebAmovN3C1I8Q2-WhrgPr83W3ZZfdYlSbIWVnxIQYeOdZYPjvoBUvsy1g==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGxKX78PzSH2SU_qOxGkvEonPq4aO3zcrtN2kuzrTC5AAvS9wrbdRAhP7u9WfltKsP_xhY6cOvozaYs5uyeCpE_6ybpKFIQN2VFFmb8W_QOXhFuqdLQeen21_7PJRwExaJFgIQtim9J1B5DeH7AEQ8z_gIZmohw_pOEjXq_3IerV9EjiIle_m9Bkx2wTh8d5lJKLhI=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHHV-k_GkrbY7jtB5K1ClXqILr8OoK8mXwcpRruRGM4vAarur6DmZZ9Zc6LXE5t-1Z_li__hrhATk-5sn9qHOls7eHSTW1rtLx1u5VI3PhYCrOBIqZ5P-h_yQ7laMwIFnc5J6RGMl8duEEH3M57z910qr7Z6Q==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHZUEujmt-BcP3DYK9SJySfXBu0naUcIp5X40LeGi3fwEB_qWKHTENPMfJsHtBfMDgNhQAn3Jc75_4nw3jNdcL2Rt9CXoyN34FEMfulpt185523b7oieTDmDtCJ5PbMcD25PTxVExo0cuDNYfAoJWM9PRqC27ckDPNwesFu0XqwldUDzzOB7kth7Wbg
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHeHIY-6lUhQXZNRcZYoiUJnaKGOZ3NtdfISkYSqzwkEzC--iAZrQ0z8r73NdQl7bC7WVYFg7seaRmKqU9acinqmoxrMMulcp6vfbF38ZKuGH2CdddEgKnzJ2Vgq0kyZl0aUvvKFK71WWbRk9D_jch9xA9wVH9I_0Xdz_FrWqvYiGm9cc7KxLulHcq6tJ4OjMniMLYY540b4A==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHxW9zeROBRSDWtwkp04MFfdmgwSqeRbQ0R0AgpO6ldaXR1CJ_6uYE7bkMkDXdUfSiV7NJduJyIZ3mTWvXcdhkMFmoEsS3RoUbaM6YFKUFgr9QwMknLBPYzyjy1w8GVbUhUYJxgDL80qJN3xQ==</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>BT-372</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>vintage toys</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Cardboard two-row card storage box filled with trading cards, featuring 1990s Ty Beanie Babies Official Club collector cards in protective sleeves, alongside a tray of 1/6 scale military action figure gear and accessories (G.I. Joe style), circa late 1990s.: 1990s Ty Beanie Babies Official Club collector trading cards in top loaders, Bulk double-row cardboard storage box of assorted trading cards, Assorted 1/6 scale military action figure uniforms, helmets, and gear accessories</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>$30-$70</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>5</v>
+      </c>
+      <c r="F42" t="n">
+        <v>10</v>
+      </c>
+      <c r="G42" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H42" t="n">
+        <v>1</v>
+      </c>
+      <c r="I42" t="n">
+        <v>10</v>
+      </c>
+      <c r="J42" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-SEND</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>grounded_search</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEfK5jCCCJIguEQOn-h-lZMwFdpwDxFno5e6uiqiRrFV1KOIe7H3RoY7hRqoqcmXKRmtJuklq3XA78AIVsxXx4MJwiXsPmkjVKNU9syIQCYuAH9EyNlf3DfonXPZJ8Dew==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEw16646sy0_Ad3nxxY8ReCBjgUpsynf0OLG0K2T0HbwFHx21kZPOXHA0LCHCoNq7YVOxJ9B0ayLdNyDzXdTuK8mCiOWBdcnTNZlc9SqO2EJ_6kOubbnJ2nEA8k9TGKuxg=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFDPupw8ifuSFljlSUkZloPXigNFa9zM5pyNNtlzWyzK0D91-0kcosLmrUtPevP9P8ZSI3_eDtqpPnRXTMFfrTR6T0Col-4ZBIO0sOaL95SgESX4t4x5xm2K4BHhpWhAf6SiK4PGNbgiAaLzrIhg9I337LbV2D6KBe9PEW5NBE=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFIAhnBg3oc2JIgIUJqmx3AgH7DjJxZF6VR4_iPSOOBkf_2s2ax_9Lm-Gb6rId-FWpgXclIcAFOIVf0DHn1k3ZTeEiY0si-NZVMPLxOBGq1yW0f2YYIrJgnb9ofD5VevFX8ljwi9Lgqo-Mi7vXYH7fMQsTU8keoFsXofv3FgyO2sUiXIdEJ0bmw8jDGZ1eKYT0JTbLN
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFMlFalS318IvOtdI5nkds5D-zjPN7GtLWMWP628sLqvwVnnqbdSMr9q0l2yAN4Q-tlAFgwdxWC40qmgFGRIF3uMasobsS5c8fzbf2qyV-rLRQQfmNaP-GBHWrBtJbgcfdPbB1AhHxMfFfgrjro8HZa7Iq7FDqVYxL0
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFQ1PnCHw-gwVlNgLB1m2Uome3wMsgc6pOM7yEa7leaVwMX_fQtjs9DDkZhfdbcvIvFhrOf2UFC_Eg8com35eM8CjPskjnk6VI618GApPOLr64Qu9wwd4NXfMhNbt1L3w==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFTxfEQQTgiqlAql9GKiUtsFc60LStybqZZoIx6jWSBzCHpb1xjfg-iTHlrMtjIPKP1oVHS7B4YkWViIbAxV7fP-C0Jpm2B5B82h1h3rwHEZPQVXPiziIB4fV5-XFq7mDo1cxUHpHVcOysohLBubWM8N6RekKDeOQhiL7tK9P0rcpyOJKQukg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFujoA_zNUQrk0n1XKJLIgC2b8IRPegl3-WdKWbGeeitqH64CAaHT9SQMJ-9YUdwhnn-0zX13hwfd0I0kpiHZxWGNIfwsZvMEMVxw5vZlLpKSte1sDBE2vooaZvBHwCDwMGUOUEJoI2jKBS9nLPVPP6Xw==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFwo8m9FpJnzrzrKG0Xq_buCweB7a_8e4MxFJ3Zqqoyi3EvXkmpW7FeoQUlTIClGvTd_Ko_pKUAc6oX--4esECAAv-aCNULrNrzv5TQK-mByHsNHwYLuy2ERv19ZuzwdKM=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQG8eoiVhfywfw9PWQZ5SABL4GmXEattmpZB9KRAGVBWW3BRfv0kLDsHw61tlwrbAOdk8z63ArzUM8DDdsfsf9kluU2HWRBtTlgdL-8vDcHr-iYVhqJBHV0-Zq92Zbp8qVLJRTr0qH0xlychG3wQpgsiI8A1tiIvoMqhp6I3VepKC_YkF1xZ9jGSqR0SaS_P
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQG9dPkr4z8P-7-NIpTSy01dyFbn013w-um03CiPuplXeCZ-ZLBt7hFsTwXL_Cg43BN-i6uRcEMpfxM2KGimlvI-7becanbs-fe4J29mzeBcDowRVO56MUphLixGNiUnM5MCsZVM-WtI07wRou8sSugHG2nfFZUjjsmWl7E=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGMzO8HP6S-01kb8GL3IhGXFC7dzj7l-npNscGqCbksBGwN6-XpyrPK30yx3bVotKMiRSn_SgH6sn6hXx0G7l-sPMRDz6M-_UWie2eClqbeiAH3-VN1nDlA-zFXtFvM8wwwgw445X7hzPwIqRO0crtjmjNf98Pd_QWZByJX0nn27uK3DkMFZKF-mZVCYBdMTYfinuNQ
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGaHZj2uRKde901g4YeXftTctWgU4JlXyZxUS116Er29oOgjrkiySiA9FRIYAIamuvpP1BzaRX9x8BDn24UkRkuXXaVc-ziVjTuZMm_COLNxJxkDsfbSJIa9HK_-08lh-v-yPNG1LIo6cv0-yJ4gB1IWtpN5CWhAAoTnie5Imf3nbw=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGeVnG48BjVFhoQK7I_KIPW8amz_KfReTGgwYLVKB6nJePYZfqEJ3czpEDx7JMlzkxg6AV3lmqMQS8C7ujj81CqWnbjuul2QqZiquVmYtvY3JnuI12tA8E-rmqNA7Yu6dTaK8fesYTuK4vM5aZzUyRNzH1R35TZqpw=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGySaWMPHwcDZvWBWhNN4CpzoS_VYnPuT4-NhSbGzWJOykDRa15Cjom3nmo3QvzhxsdWqhNsp909ewQXS15UpY__oKUjWXS1m6zlJMDxn-lBNgvOErZydQHTiI6-TOKrIganYivDm51UVxP02mN7CU=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHUMZ_Qpj9IpnVScaqe3Do6TA9qDIzyXqn_p38ziZ6ZYCLmZVSDb1p5MIdUVUYQdxHpOfC1pQbn7TxTTqdKnTp8MKf-FiNKnVop-DYZYgVP12who8LwwiDdY48-PEO4RWSAVXrkVeNVkKAJZ8KFlu2Ki9ySfSx40A-9p_J-BVuer9Y=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHVtT3iulN2BfrwQqOR1H9lIAhdteWIUfSWkFWfKd5N0x5ibyql2leOv6lzG06WVDwgOd0WT8Y4UCBlJFcioJSvFaChIQw9F5xhhDJtg25jeJUmlVj6kluDH2zF5V9YT28jIHNy_8GBgKkmvbGeS7m2Q3Q=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHXNQv79b16a9IUXxzxu4LGN9t1AAf7eKgWS8ARGB8uy28kBazmdzHkCFk5QM9nB_3QgySqgB6d7V7UyyBvuO0qvqInIuG8_KMQrrkA4ttHv8V6uuO7-FUC5iMWoSK_Kw0mXYnzlsUtKQ3n-zRyi84OuRTc9wc_OZsSBKIpB1-oNIWsg-FGV5T8
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHklRsCDik2vCKQXjCkh5RfCCQbocaQgZeM4KeWzxsYzqWgfl5SB2a_12Yi6P5rM2PvsiuVDEg9laZAltaGoJF_nAPklHdEiOV1oRQ7vxiULoNJ734W3VeTsE0eZYCCMQEjQOnSE2z-IsCkfWA=</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>BT-385</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>vintage toys</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Vintage Mattel Hot Wheels vinyl carrying case / Gear Box, circa 1968-1970.</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>$22-$110</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>5</v>
+      </c>
+      <c r="F43" t="n">
+        <v>10</v>
+      </c>
+      <c r="G43" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H43" t="n">
+        <v>1</v>
+      </c>
+      <c r="I43" t="n">
+        <v>10</v>
+      </c>
+      <c r="J43" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-SEND</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>grounded_search</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEBC28GiFuIjBhEqMtdbOAY13KF1hOAW8vYGgE_uP1hgOEzyOJc3WKoVrJaEcXib9a0roHZgK7aJfKh7F27tF8HsTnkPHg-8iOUvBXCs7kXaDjyMS2u3uf02BAzfxXf_G9LKoL6phB6l3onUQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEQI629CsvNkqVn4MxEDlZQ2xM1qgReHsH-FJv7XyzHoGG7g2BPeoXDG2brHo_j4U4wsPVum_ba0njRsVumcuZSjPOlWgvAOi4PqnA1vfSpCI7raAkLJSd-8-v_gFMqygbuPIfXu9qxgnXiurZOJj0hrio6f0YcqJxLbR1p8CgbYFWowpvvuA==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEUPFPapoZVvTjiWUeifB6sYmqdqW_We3fzOhaQxdp9T8iv3m9p6F9jiORjahUD3YANbmUd2wZ6wQJ4_I6-m44H58spZnW8rJik2wc-WX_ZE0PnkngCXsMl-ueegnEWFWrJHUrZhmaX6jwV6qL1gD0K61F2cS4bSzZqbeAvgye0Qjzgv1ZNGL6-ByLV11OGozYNdKy_e01RseI=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEv4u1O5XEZPPwaG1c2F8qXChlt0MemN-ESSpTFwinzGhKA46yXWpwzGRH-FEbab2Wx7tLFHSaj9DbjRhCO-sIixTsu8aNWjmxd-iQtmp5V7jGtcnmB77dXRzFHoKR93FKIVzK5BiFWnojsvHoeVrwyOcWgQIdrJdWXTYVtj5ql9nZaSdK5HT76i1G78RBI_EOxXWdg3TQT3i50
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFDj8hQ9FM8mtYnejjaRlYVTV5U20tA9-MGF8KL6D6N6I7IYz0gQc6O9EvlgLvN4inEZdvUpCFqknSh_wcj_O0fOp1Raiz0XjlAX5-V6JXFraWi0ZVICd-rzw7kHc6Hv8uxNMin7Et_2ZfRiCO8PXUKbdMwYddcl3jIWiHYVwtl6P2XSAc2VhODco7MSDugdsS51ZT7LeRmZXLONYUtSDrqRVrOwns9ZXUirES1cWHqSmm5IXmnBcNYDXaWiTF_
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFhDc79bLlL1Pk0n8tbzlq1olyfrCFnjmCvG-Ltikuh4YPMznI7FKOxH7yRuOpPmWhcnUqQsiS0KKkX1E22Z2setNkG6gpim_O2tKtuyu7WB2SxwtTuvdywPZOlRX9-sG9KMHCLea124Ea819TE7UkV_6Eiq-6HqmIOmP6J
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFuNxCKNHiomRNU7GBBRd2OMv4wjHPag6J78UBXS1oJv6s8GMUFdljNLO8UcEMTlLngrkc_Qrw4F3VMexwnzar9VzhliCCCtngnZUX_aJIc_0pfDuw1GB0cf2lfSm8wxsXV6C_ZBf6YPz8f8-SQno-C5DkbyG6NkzWvWoimn9r-fOKOH1Nbzp8aZeFSqjXk0D9gaa9fLh66Ef9Cm5j4KnP-uRHzJPI=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFvPS-sMdOdHhaqdfewWUelnAj-Fas3NeYDM30WsdRsVqWZXr1XlaSs3Pf54dtq63PXJTl0l3l_PQ9Rzdud2eNdXAFiYsLwvnxZ_4JZ6-pVGfmYMXi26ZeI6NqFiffOal9Gdaaezzyc7T9VXpQN
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQG8AzFS0Du_su7pt-SNpud1s01BxRdoipBkEl3qSdSMhkTVfjp7yfJLr6U_y_AeOfelKPBOUG4oLKf2Ms-1ODDYIWLN9lVVq5AMqbQw5IkJ8tnyFesOGAACOj1-NAwMPHPHfSir65wMlWx0KeVsLTKO2l2xsTTjip3zL5I5FzHHo0X0o8mPCvQR449xi-6fw3p8FmobZgFBJw==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGLywuanXVzW5RKzhp2PUV9Irpd53t1CYIfd_jHmVU30WDhFs0NtIzhFe-uaSxxzbGOqy46AR3NNuE6c7BYCCmu4hEFtJsvoMgUeA_VbxTkoNPIhcAQ55WhZEinHMjjVqsv6ENBwDnuEB-ucNf_WlGOzi4KsBHnk4i2m1e4PdC8M3k0
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH04Vu3ok_hf2O4w0MxLUyjLAMZ67lq16i9eJZhkaZNn3J2avdvFlGr_nMYWUYwOexQ73cJgEBAny8oHbvUbMihKIgDcVaZldPWNM2Gd6t0CofaGebQF5Z6G5vYJ48jm-evogAi1EOy6sTLrB_dFeRp26tE9hkliqlbRJY=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH0ZxjYGOR5GY4xmwpyuHrO5vrGX-OlzrGOYyOTcTiN59UoA7Pf4SyShr_WlFooppbwDB226WX0ZtZIsr4pOEzL9smIIUHzAfD5qDS1eDUvXYfDSR3_zMCtugqpFTdR2vd7amYFe7rRZg3wdEzS7Dv1yInbntYzTVM_wVlFJRP3gUgpuHpkRxpQ
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHShgLg7mBg0GBWpZvcdAw-iWFHxU-nTREk22D5_qAY8arOXscixl9kGV56Uxh5SN01sTaXJwgOGReMSF5WZJaxqoxK9SIsil77Y3_NxIgjgUptJaLB4EiMTtXHBq4OfAb7tb4lR7784P84UZzTJWdRzncRyRgJWSw7zhatlZ5C9kVdcypwgXYdiQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHWgv7kumoMP73ft8t6unWR0ITedBkFOftviZpdmG3bUFl9pIBR2FwfhqP5QnHxV4UlWwyppMfLzyIR12m907PvAu4M9Pg_BGfqG_5d0rNWiyS6Epte0yHM_E97S2Z2ms06d43UOpZ8Ss_Xb_dbBABcfv9s5To=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHcZqQDAmo6sPBXMG4Na0vC4cpzY0NapmQ40eiI1upiyIrdUswP39USR8KE5cUogzavNxOsECKjhTmiIOUCX1lMAaKf5eme5SC8Rp2LOhtdHRTKoZglgBnTYcmTGSMvOqu86WGcp1028mrIL7KB3YMLChG7o1_tAvdYBFXU</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>BT-432</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>vintage toys</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Assorted vintage Pokémon plastic collectibles and electronics, including Pikachu figures/banks and a pair of Tiger Electronics Pokémon Walkie Talkies (Meowth and Pikachu), c. 1998–2000.: Tiger Electronics Pokémon Walkie Talkies pair (Meowth and Pikachu), Large waving Pikachu molded plastic figure/bank, Large sitting Pikachu molded plastic figure/bank, Small Pokéball toy, Small Pikachu figure</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>$35-$75</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>5</v>
+      </c>
+      <c r="F44" t="n">
+        <v>10</v>
+      </c>
+      <c r="G44" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H44" t="n">
+        <v>1</v>
+      </c>
+      <c r="I44" t="n">
+        <v>10</v>
+      </c>
+      <c r="J44" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-SEND</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>grounded_search</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEM3LlU-ITCjjuuvZFz1Y4FL9Bqu7AOg7IgwNwWefPddCIHGCrYb8TfFL1dsAlz2jXtRiu0ZPV5NxYuSdEAy4zLuN6uwAyzohnKZTnKaYoxmgBpcvGkorcgAds4EU4c-S8=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEYiP44r87-AYHD6AxrkNlcdZfzJJ0vcixEh15xLPyhwhT0aPKf02um9VoJN2pOluufQMQenNjCQnlmM22UY2g7i9fgosKS0ZiDnDxJcBxXvsW3LfD5u7toGm_-8n6qwtU=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQE_Zv7KlrGPNMA1aK8vw8uR98BoftelliJoUc4ITZ06L841qehasZRl4aeg-CIWSQTe4aOkqeB6Io2UXXGLvJ0pDHPYmpffDkDIys0TMuwv7ECxJ7zXZnEYeGpYuXIozWuapT9nPNoG8sz_14Ye1ghZsFjRWMYtMN4cXkQlw0-KqHT9nAfNeHbjZc98Nt5Y_4bdWgJKB3hZzO40RKwO
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEl1L7DZxGWioelGbiGQrC9yWUgTUXNbGPvV53yJXCR-ZmyOQG3kkmZThXX2rzFgZoslqhcUn_qvtwlVmdo6maeGI9SgLYrHgtEcDZDyXhaHuuzYE6d_oe7VTChSDWLET4srls0hxXy
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEod-IZDj54M4omEFxKXZTXEvbh9DZVZolTmFRhEv6wOpBqvqcq9wCRpiv2Jv7XqdHuVBk-jrfBbL2Bo4tWdkiYEweO4u7HunEbYmwmJYx5Z9g9w4sgNR50CA8tdViv2BiJpIO2aTKOQUfmbX0iS5thQ2euME64brX9ehTGQ9YSs_lOn1zFKginMpTmv-ri8pisvgeDfrKP3ZwUZw==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEyqI6YxwRe9-BHVatxr39_3UIhYLXEpoUo-telDVIhO-YZ49vxLfw7DWdtmM4lHtttWOJcp82NUGCOMcyw0WhsNkpxSs6qSwsb3aCkeSFOUAfhL-1AHCUeyQroSApZNgg=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFC9LmH4qDuxB47J7dMUNTeAKkzhU6oI3Pt4-mrIDabxaj36-VFfv_QAsJWCa6t00E9oBemhABHC5LJw1y7CPC0Pbsve7KYqdZRkGIqsGBeGo5k14qQ76nkSVGtHZSGm5mTlOIPPEfgRn_8eF-wSkuCEkfvEcFhz_lHr3xALWfWYTicjweF0JUY-7mF4EX6GqnTO04HNTVJLYAbPg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFEhJAwnkJDQ-TBPVk9s-ThDENs-mVcvAwlGECDkXHLglOY9aiuB67WSpYgyCgB3rS889-xIbwze7Myeh7K_ll86cH1CCDq_veQ4e3bvFTkNy1lYmYnvj10hB7KqJl_0tA=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFFMOmcp4GquMET2xXkWNNRlQFAot8qZ-Kp9AUmQYqFKXU-REp2gTiMismBNABjSXpxz9aMJO1Ybx5EBUcZGg1FkIlShyhoFFMpSKtiID8EZZaFYbd_lnuBzuTC6avHWMs=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFGM0ViGnAFZBCPmlvnXI8GeY0UJRn72h06QOJ7bKuxv8Ovvq-N9Pw75ucyR_c72AERUz8i9DV1XpKpCyijGITKskDu9eqtOTqPjZWS1CJYS4RZ23D4n4WMv9mC9fmIZb1zgzRxSYBKU1KHRz9wUj0AxRAVZFPRfifj5XeXPA==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFI26Z3LkR3EVkI3qKdF7MwQjB-p-8r463ly2k9V0R1dXcKKCuRD3zh4p9XxgPCj8ZWluK2osyprvTM2q_aWQDkFWGZxNKtUFRdBNLwqO8EgvfU5BTnnGKPoQ28T8WIzHoHVx-2Lh4q_81ojE9ZNAZ6nGXDN5XL79UzqCHSie2V_eGz3cOZgftmggcl_TcQwTOKoQGY
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFUHqxvfki-Y3f-ocZjyLM2oZihdZS6x4bF1MjP_i6oP73Q80InpXYKhZq5-Ex7M2bLLJfyJLJRUSM011kjxTVEkHt2rcqrP0ZTTMqztPHncHiludSN6naRjibV-T4zkY-8RfCMPtWmeL5gnhQTWsXOuxVp3_hiqWyhaJg=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFoUPltToVzQUae_sAgjlYy2Ln0C590t9JeOSI-7pfY_BWCduZCfNozwxNRqKl1KrfOrImNXHu40wKi-xlIMGYYP-p3uij4KGtXF2KXj5bGaeeErbsjwdmv5HRofObAUhk=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFuoMaIIcvuDL3BefgZvuE2wcFJMygdAuztAY_ZLwuQcQShsPZ7-LVEoLNiP69G70D2UJEW26cnGqFXNbiErFJ00-C12VpEDIlQVE2mHgZE-qeskSFHxOkW5mqizLTYjjYObfMs-qaryp1mBfJ9rHlLalzV9tcF_x7Pa629-qVWOJQmWRXbmShzuhDGpGEvkC5VdVm92aPd6fXg
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGNQOs5yoFqtkggnUK9u5_1oKKrgpZKmctbnkdJYTNP2q67xl-94Vm1eYHiNXvaxceo3uS8PkezgJCgVMxxpIc7JwsM_T3rPmXXpre78jLvfOv1VDYhtmjMJwyGd1Rm3O8=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGRU8FpWSWlf7vyw2G3V4EAAaPDEkvHReDf73cEyaNCEitpf5-b_NQIO7DaK8BXnpkV8g8vswmCw4CSuVB2y1KtzGpROdQU4FW7AIlIDPN4g6Vb1-JEqsazwX6KRE10XX4=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGTHn6G7r3dJO8SbfNvttvEiZyfd-WrmWY5SQs3eVqsArgl9m0uKbBX-Dx0MC_C-slDOkuk2jgd6bKuibLy3KpwB_ApIB4nPzKC5g47Eq42MzyDRjsOFLxSMolc7GEPF-O9WqJFh09cxZ8diw5H0hFgehrPaEWwfNSc2mEKtmvSww-vGVsbbaUP6COU
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGWZUfgUZv72QAXwKB9zF--T1UfJ7pyILJO3_7hMfVdy_00-oOD5w0_DvIubVvicLrBQyWTzvQdamlz3oWl_R8M7H-WAANx90BG4kOtHRI5fVUdlt5qy6iewnsY1PHEcpSNgaC3dpn_civCjPZYQmjj242FhJYMZMgUKmvb3_hREuFoLXRpeuWQ
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGaqpFI7i2i2H65uCknyPCRR2gdN-PXGJ2t1S8C-tW8bJjj2tAn2_y3Zn293gXAuIjJ7B50Dmg_oFzzUEfP3-AfrpHvbkaXSKSH9XxZ4YXPClyr4PgUk89D0hosZLDtD7PS36u4K1a5cjkhBEKE8YRS1Vu8ebo17GcnEvShZiiVXQlI4CFxmeUA2R9FRZydb0WN2G7j
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH8PFz8t43e-mEXqxBsUF7Fp5QCzbCE3URwG2KU0HlxxsxBZ79BiE3S-otAXwGKpRwLQyAAPNEGDRVIV95VQD3_QSCh37n1b-GFkzcrGSlcFg6a4G27dYpeLI75Kg11HPyg7zDywSEQBjbVYC1QdHB4oI1FBRAIwbohpURFfM-5
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHBTFQZQHdmqxG6A66MwwRpxQV7oyYgL9MCNcf9h-GMGaSOHNbSVCXFYBmVC8BsZCMVWGz0xcPxgGhxkt7aEdFIcGTWvfQQ9wNRgQ85FrIaHjpNUeS8CyG6BqlI8uzvybbOUouEnE3z4nRxLWehJpOm4z1PEkLAGYtl9v0hPFnpNByk9LGVNDMn1CTReQYc7F097EU=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHC0RDrYAqNTHNKMP1uNJwVbrKje_Iv4CPWegkF80cTG38jyDaGuo-hW2WoPbQkyAnlh1hqj040CCbZhzzvst0OAK2ScXcDA6BGwBSYqqe29Ije6QIlAuGYKhk07_mk-RGB69JWEGVCungJM0W3uyZQDHM6wz2VHnh3U351ZHK_-8fg4iG0NeR3rA==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH_kXH5XsGtRkBTLZM24_iEkpL_GoM2U-gicE4cPVape5JaZmDhiOjKxBR1nkjqlDHa1aAEuX4bcb2VVpXTEo4FswKL3vUFmjSpvZTD2AdYxvOdn_YERCAFUEjd0FowVKoER4gOSiUqdPBhknnH7pF47l2OscoXYbvBA4bJw9W9MFf8lIaHK6oTV6Ff
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHhouKUN4hhZbspqlzr8t8H8jnh9QQysYSo5XTa6g5sfjFRchMNVe0HnjtDAwcMqFtytlmLKZIGLT1bCqz1cbDAB0tMrNYbd9FganH643IOsmHiP_febqcgnPleF6IJ7s9ZGzvqQ3IkE7TcxrUFWugbzkdL4GUC2YL-hPQLc6-KUpgV
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHn4NP8W9uMJgqKbmzecsBkV-9w6MaNdsg1iMrpo-RQvUYKcW1hesyyzcPUv0d3PmRv4SbrEE6vmipSUm41SjhC5L_d1CmcpYLo-3NqGxXCJ8axvH6dNVuWR26kywp-5deY8-Yqi6W7IM1ga_kGmA7Wx2Jezf2i8YW96nsyE4Gsow30M6ceVnrIs3RNebyY09hVcQT4dBO4Wq5oSg==</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>BT-434</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>vintage toys</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Vintage Lincoln Logs canister set (Playskool No. 891, 125 pcs) and Original Tinkertoy canister set (No. 116), c. 1970s</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>$33-$73</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>5</v>
+      </c>
+      <c r="F45" t="n">
+        <v>10</v>
+      </c>
+      <c r="G45" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H45" t="n">
+        <v>1</v>
+      </c>
+      <c r="I45" t="n">
+        <v>10</v>
+      </c>
+      <c r="J45" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-SEND</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>grounded_search</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQE6YUHM4T3pE704OHI-p4Q8a-GMbmhtQpu-3nvrSUJG4sD_JwUx2NXW4EQAjFf9PjqTDgIP9OLZswe57OBhhF1AoieBNRV7MG7bwmtxpLEguspIGleJ-LkELK_l3Lq3-BI-8hJLMXgdSJ12QTQuQY8M4ToigwUyqsCgk2xf01uR37XZpuH2BwFr5zuQ4C3vP-k=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEfkXaL0UlcCej1_QcOMc_ALOTjkfos6yUlGR_6gZVoF8IEC9Ruwy3XZrqQq7F0I1odsdPN5Ynh0Vx2iBcXmv4ZNPv_eWzZbEDEMv7n5N_eef8Hyf5snSe8pmPeTqak5Q==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEixny4OENhReZxk6L-7-_oETo-pp0mvi90ackfoZvJiTIU5QysBO1Kuq7kVqX8E50WMsMfw4DZ0ry7YVKFcZM1fmq0HUw1M71ncNQv-CTpAIxEQAv44uWKRTtHwdW_CA==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEytgcCLYYWKpHYYg0FCQS3TBwpcEZBW9qlywt7vejH7iS0GVJ4Gqgy806s9McovFy602NJdETGWRqdYYMj6RFpuysMiMWsVnFLoE3KvaCKneaZWtLTwg2fKHmzq6ILdJC3goN64MvBi7y2hincCOTKQ_w44dJxwH5ZVY4NBEvge1IbyGV148Q=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQF3Sk6P4QeeDOGS5pycCl7ngNdDaiG9sV36RjYfERy3NpOJhNwKwxsE3ucYob89u2CIZTMPA8JtaPn8KwqYtGt2xIF6OxkX60DaY_D3RfImDJUYPPh676Pok8EqjPNNOM3G-dcgHwBVw3G1M7dPHwpQb-9_nK6rtQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQF7uYQhT2ebyXRNJTbnp8LYC4Z4s6mS6hNIVUDJN1U2U04GCWNNw_RwY03kObjPxdemVWzKmIdgrSZuUtzYpR9gHtfiqD7gTugp1P1v-92kanudxR_ocpsy8Mo3lfQh6B30tyLSOrFIJVGF42RsVHwxn7ECYjcZ
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFBMYAy325gv0KqE2-Ff_9k4feGwhIRERfnIVJ6Q7aKNj4XR28yaxsHZtvCM5eVcnfQ5GJGdXPKXFmt8a7bDFUz31ZbNqSYb3Nibj8vSXzJYTLh3AqdeZBa5mkfxZpXOyaKT3mpXc4Pv9Zrnjvrfvq2l5GJllpeKQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFCd-Cm099QKg7LUoHY9nCnN0YG1iukmPkP_xHT5qUfP67V25UB4wgIjLjShozY98lPf7eL5bV3O_4kR1ngt0V7F97PLBrKeE2NjtNdw2CT2q2EWSIBM_OLZKkcZJdLUA==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFFJMVdmfUykmpHIkCgjciwX0pOrH8pz9TRcWK7nwwmFDJupOuzCB5xqUBBrYkmEyM2fggHnus8oWeAYbEDvZzYl_rUWZNzoaduRY7H6uLJ28BmkExuOjCw9Aw4o-8R5ElWkhrGjmVU1M7AQwfkMCN-QuN6v-B-b16ORgVOYHUlsAreIh885jjD
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFFNnYcH8OFe-QfGDje8Fd9Qhy7qBNrVRiTBpoWYG1aQP5voVw0ibER3FN5vHKCPJZKisnG4jqj5vSOhn0YYehxGNS5P41XMnt4th5eSN8FSTSTJb0W2JsroEbOCc0PIFi8viFudNUjHf2wwB5YMfg0uxQ9u3eiUg1dYiXkDTpIcb2PwztyynGNTekHX9fLdACL2fcrV3zncDdB1u844w==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFKmZx6XCnLxuwWTuEV_2VHy2PgMUzXmDGixtVBPNMNwjG44b4Qt4mPHV06iTsLFSbEWwcpqZa5kia1cQ_P0g41lQP3jFaaA8DyH5LEL5w1EoKBJTA3yiUK_EM-05CPa8E=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFN_SFowWeg1yzblmbxAObwh-LQSDle3WP6u5i3G5OVo7XIAa9k_2i2Jq_J8BE1OJlV3rdn5SjC6jrSaX0RI7agqUzKzL2LV2Zx0PhcnciApEySuR_az86KfFpDnU-Q
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFTxNHKbHhlwAwkDBIsP28O5m-wE5VY8RKVa-6InR_-sruYgOVkqogg8ug_S7ztHetGygNs68hUax-8ddtSXU_VUji5GRPIBfCiFntNOGLAfOkOJEwrLD_LAydtUZfZOyAFD1YVd3rnZGljRr9HQbQr9_TPlL3J7uRzXg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFXxqSgClQWLHG6oBeH8FOCDbTXqSEvwkqOtrAEoFRl_R1P_a92VRGa7LsG-b8R616U2Xy2OQMflSVdZ5YVfrvBZsJiYX-BWE8dNnhm0ACwqT6iNoY2DWFPPAWgOS_lG1kZjJZE78cJuOlOG8mh2TJnLm0uJOHU9-Xgqog577Pi1hCNpQGPUeYGSgTAOE9uYxS6Tf9hRg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQG2dXrJVrTaQg8zRbtifw5I15E2BGCSZUeCoueR33uOj39apwVFkRak8q5l7uAbgRWm9ZOmD9W3IbO1LPWvslKqzcnfpHrPxV-2ZUhUx1H-mFOw02FG6bkpwWuP6Ed8QGqUqBdLxxXatAylsZ_Fw6-KM7wpc1UPBKeOi_B7mH4Pyv11wMg0fL_TAxM_Qnog
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQG9EYd9C-oUTBaHwAkXedsKkGH4X-V_UhRot3IdlQtMLICzhcL3uBtlI3Hp92hRn6iVibXQm7wALdrTfSaevKuEOgey8coXnoS9B3YefOmrlKpOZ49oaCpubv_aP0EFAGSbGQwrZmEq8yvFP5GhKTS8PK-Ec_3Po_Rk312Dimypi4Cn
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGL-FsM8SVOhF0zQQ8vvd0Vjlq_PsSYicpl_Ga0cfdNuHmL7cCnCx3ZEVl3ffHR_4lvGrOeSkeYms_W-juExSifYq033UEEFwBX--QQHmk2dSrl-4qzF8zeaq0Y1vaGoTE=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGQ8kZqqBPfNeHPWOlTS_HnVNOErsnllZpjmRW7oLplrdIpYlIC6Mt4ZvgcYLNnaCnYIkmI7uc2vVuyybWzFoDRz71W6iq6ctBcckNuJX8YMS2iyldavAJpmsPJPZAR13WXMDyiP8UmGJK_wwgqCIN4j05vMpmBbp1Dzg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGWplZMJgkzOxuE7Vtpsqfgswz3SU55AkUGRNWcFBu9-zK3MwaZJIJkd27bYZBJJVxnBGlmyDQLx0RVJr6ZyFckqMJwRU80Ddh0m3d91hCVkYbBefFDZKQ0L2cTOdZJay1IIpxMPPqmMPb0yMaypHHpuv7Umj_2spFc2BBPLcs7CTRYHwnUzvTuzAfaFntHlXdVngAIz93hfce_4qs8cWPVbto=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGjdJAjqatp4oUe9_lASRidIYgjjXE3tKAF3yF3HYcqr6NBWXjECoMh2GThFgJgLfou1eR2SJglJpGyfD62SJq1hfs8YE5N9M6f2IT5ockGPFiEAzfoeXIdMpbk_JIc_gcSfB73d3Gca9FIFvqJjOVgHjEhrAPeqbSjppcSc4egz2dXsWfIEvk=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGzuE8yxjRanmuA8Ikv97hQXCMK2LCBtygWYH7kAgja3mXdxf_g66G8ZepEe9ETZErRSKR9beA5zfRoDvtm2tKghmveGV9MhPyp4lHGRkE4ZGCezHUuAUF-baRWCMvqfSXojDso-3sJTgCMQlyJ0pJCmRD_V9yDlm8wYWTA3-DPJfTCrc9jA01M91Gcu2KWkk8q7BRpdEwOgbyRDXE-WaonFhzhoQ42C6Rfcg_y
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHKsRgzxYhvlcVG1YtXHkkXJnifgJkZXb5BLAUAhln6kv75IhsbPwE0MdM8bz8atg0BpnzJT5bIx6KQP96vr9yaiJ5Rq_z7Kg3dqFChV8jNTangJbSQ0Dz6LfxHqebd1dh2iYo6SE01VLp0ERwNDqlbgOJC9E_paAOkc4bK4YE6-j_D2XbZjV59Py8rYJ6V
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHZvTSNWLL9Dg7Owbz_MTsAgxigYEkV71cFktqMJUR08TcfmEykLjL_pK2ra-bp_3HsiW2Aj2icC6Z1CpsEs7h_5HFn1Z6Wuk8gQvaFL9kNV5yMq7JqnKdHCu22qE8dPAteg6Pem_awwZ_ZPq0nCwVYXAXEea2GnYBKLEDRs2ptaUeEH9aUgz40ITSBte0l9w==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHamaRRK3TarFM2N4_AYwRxsLSPRWEgafFQnMxSuJpVTe5-dHE0PJXSTuQy2KiOC5t7UHIDuuO5bve8BWvP_jSJYHmvpVgSmQlhOXhyYvFKeCjKPgOweglI-Z1dGmujNg==</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>BT-436</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>breweriana</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Vintage Hamm's Beer 'Tapper' aluminum draft mini keg dispenser, manufactured by Reynolds Metals Co. for Theodore Hamm Brewing Co., c. 1960s</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>$20-$82</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>5</v>
+      </c>
+      <c r="F46" t="n">
+        <v>10</v>
+      </c>
+      <c r="G46" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H46" t="n">
+        <v>1</v>
+      </c>
+      <c r="I46" t="n">
+        <v>10</v>
+      </c>
+      <c r="J46" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-SEND</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>grounded_search</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFfyS_AjMdJ7apj_qaM_MCW6CRJ2mwcr-8HD4oU5wNlEoYIdOEjorw7NBTzGibQswWSwXfaoXk8XsOA-Fl1Y6FUgPfarK6Us5jC0BRi7Z9QXB1tB3fK-U0c7NoEPSBiadp5jsaiqket31ATuZw-CnqkAjwY_-QHh0s1BSnJSQSAzVoh4jz4TsFS_T7KYL0UrUBtcg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQG1CRtbhmjEgqPhm2GWUyKb_u_vlAU2BqxHbgaRRBAVahaHKZ2oY-2HfApY1u-djHrnTnxeg5txQCW4WuH5c2E-p7lFitpbeB_vyRPU5G7S1eyTZi5oCzQmoAA4AUEEJVXz56gTRnpUQuaY0QU2xGQLdlhQdA==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQG5t0akY4E8yKLBR7uETc28lcfBpW7P_Vn2o0GJqYBz-3uji_VyppLpjVgG7fP8WHC_vevgA68AsplYsxRufbgS0j3KibJ-T4IEVVf762DpcdIfYHNcGzaGBp6r3_RE3QYEa_xfOePwdntxVkFN_4JKIP4w3G7K
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGODNX1j-vO2FXNDTpQV5UXgvmw9xZRV5jSv_QoSoW4laerUKYzfuAhdsNczABJx6ZasQijQsE5sFhp1OAn-ofvNBN_npjhdfh8kyNFXGjKsUtu5z5lrKIkDBr7dHfeapRCBYU5XrHNwPRhNFkyKY8qr0Vprh-ieY8_Eu6lOgnkYQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGYcYSq5WDuZqyzIqcg_uvYiF_VoVABRwcCF-Lgk8r4_jAHCNB_B9cD8trIYUyGcoVlMV3ZH9of5Lw8B_xcfAIxhX4FFn5arTGszP1UdsApunvcf6Lu0jNtIXlAZ6WO--AzBJXGvNF6Y6vX5aY5Paeva8N9RsO0mQ==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGiWvp0mmWjqzV7JXXiqevb5fJJoGUvkmZ0UDY_JImJ6LN_2HNEgUCdmUk1tkg-ApUVBH9_FKZ26ClbueQrZ-kAPl-Ln1TOke9O45-2vTAiRqPlfcXIASd3tay_1f73KYQtyhquu_cHrd-qpf8fDdKD9hvWTM2K0paUnbp2h0VIlDot4yQgJVawwnfyZwNQPhVNUg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH1mEVkG4okTFoe3RmZtvwBE964DwfJNLkwJ5OsdoSRqME8thwnRXhcmA9MMqMy79l1LZk7eP5FSFInuW8wqO2PY2n32a-Otaeqjt5EY1J36VJu-A50tdNcPVRbTYf9CV6usqlVvw==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHpCaZhp3ls8M5Bv-IOkXyTPLfYrUP0JhOzLi7rjKGr4Ikh3OcpCw7im1yzVC6GClcYIwsSpVN7b2MSWr5fgNYEUFd_mjRcVA_ih8Ud3XpuBPOakJrbxqMWC2ETPlXcgNv3o71BdDxW
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHr1PdQaW_MFHkn9Vn9WYZn6AdoCZkzkVBxgHsSsqkNHWi_4bEg2752Hcttmh1j3z5xOJDKkKhZ25kYdpNwjCLHpuuthwl8Q6oOolP2p3TwWkZ__azOHTpwGNR-r61kRElXDe5oK9TFe8onXt_nC6nimg0cglXVMQvAJ_MS14kKch8_N9f3_KNWIFLR6bQw-cXa-g==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHxC4Ng0wFeMVcEPXl3Zyk3ZSd4_g3IC-WnYLaYaFRlA6rkyqh8hkEoteffKsljPlPRI1rOeN5g0QAb6waf0Gg4jt1PFTN7ANMELDh1UWG1PE3Ae77_e3ddZxwvP9XgwB8qEtEQeT64pgx8QRaK6h8H0z5Livka8Pwktu3MULez_C3qhg17GNZgl7GVv9nTKQ==</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>BT-213</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>vintage toys</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Star Wars commercial art posters featuring X-wing space battle, modern or late 20th century printings in plastic sleeves</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>$10-$42</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>5</v>
+      </c>
+      <c r="F47" t="n">
+        <v>5</v>
+      </c>
+      <c r="G47" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="H47" t="n">
+        <v>1</v>
+      </c>
+      <c r="I47" t="n">
+        <v>5</v>
+      </c>
+      <c r="J47" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-SEND</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>grounded_search</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEWQ3KozMXGkFyjrLE3htvM_W2QuZWfjrOHz5p63ksCgs4hcaLWp0F_SjhUfNzwrIxh9boSCroHPMZb90pnpjPdn7nfC8WAwp5VEJoL5gIzkc5uiT72clLIQ9RzFfj3PvvjVrfRoorcdDM9dKUyEGWEMNs1rIMoWO8zxUekaHFoXqqTU8-0BL_D4w==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEtVEkBfsnZYRK9v_MllgjhyaMqJ24wxBWvqfRELek02M7VPcYSKGHhb8B5gObCbLgsYgJG6F1OeLhg1BWAikiYsh4ci9UWbCouJf1so89Vuc7b_t67yefUE0Hn-atYEWU=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQEyPBWDS5Pl6fxzejLgR5kb0qqs6Cj3GiIirBb1v-2da2K8QEiAHE1C-RY7miBJxtYj6cPSBl2nr01HllZaFszm5_rMlwO2sMRn_m9bvkGzhp5MJCk6WtQkUdmvY3JYfS4=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFAqA8Nf4EuAi0Bjl44Lz0oIxVYn5U6SGAXcJ3O5YQYSvGyqliSG-Hfn_QMIuGK885q-Kd1RD7XQsIIr5ig9k3uQ-b-WHkTFBwJl3pQ2gWw4TV_0FNvp7u6cWvi2zZT0XY=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQFm824qkylnsSnHlrl2hYgSZ_YnfK1g1z3WKvpiw6GIURaNywbzAccvuqqt5bIvKfhQSke27iZA0hn2kKU0aDHfLnWEQqjZbf8BiNEiOB0qUIE-uNhWIyqZKw_a5wBhceXeEusLVFHiGseO6lyWih74w4FONR8=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGAwlH0GQtbivuWJMgbGeTf_ekEBqKSkARFMRDZdVFQNfAFy-nDd-OvD9J8_h7Tg6kUgjbMHC27WQqAOPnqoxxYdfEPAzfUav6iaApjBtlBjRsgin6QN7dQSllyFxKqyKI=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGhfg2uf5P0ecQRfkMukqEhHIhbHsXC0psfnLmmMJOEhFsYBfk86yM_TM36FkjbUB7uzVBQKzsM887slOk-5eQToelGJxux4S3seRWKGO7VyyjVYVawMt78rchUlQrQr8JMM6fkLLH0rd2rdgtzK4oglKKRs4E=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQGvfhUxm6BPCNH6fj87P38TJFxhF-MJ7oD5MYKX_2VTTOURqX4-F0scGbctXQP6uowUQql7u4BPy58S6vckid-GEndO8KgPZCcCVmxxGnLODdUeDX7IfcNczNmhlJpgtQY=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQH0XPKYFT8T4sDWGCixX3eS-jjht0R2NHe7TOdlKnDgiwErY1fVrma8yZL-8gf06Rjfz0i2_XjUVlEhayh9cXfU3B2eLNKKP1shHNh91jCJJkrmTGMNSaEjlyRVTGbFPZg=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHSFSkoCbBDsKBsoH8kJ_vnrMH20AiJzFD7MyyaWoGjGdMmS6hWAmF_YNP5663TqAvMdRV10F9fFaqRyUlGEB17EJuDrKCQelTL4lpvOExrwK0syfXkZZHXRkPXM5cnd2CiySShSZjtS2RNQsweLiFHzLzCdg==
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHZPi7ni-gi8ijfmdxjDS5d5OMPHgGKsbd7vzrVxCkCgi5T4LO8bfsA2v-kMOWfyTcVjPEtALSVXJjeiVuCEbj9u1SIZBVa4xe2Esj6aWkRIrYMOHrM9qajOFcI4LK_6Um5mnDS5Wit-L6ijCYaASYrLBrWM8twnTDpPDDsdy1AVJY=
+https://vertexaisearch.cloud.google.com/grounding-api-redirect/AUZIYQHd80I7oa1dEUWH_PIya2lmemtf2mowzcuWwH-K0DgkyKSyfZbAT4Eub4svXw3-MQH4ja5-byD2oxaQ_R5Eqfar6mATXG5v5Th4vqGIQUhjxIzux0Pys9XzHRX2k6FG3i0=</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr"/>
+      <c r="B48" t="inlineStr"/>
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="I11" s="3" t="n">
-        <v>275</v>
-      </c>
-      <c r="J11" s="3" t="n">
-        <v>316.25</v>
-      </c>
-      <c r="K11" t="inlineStr"/>
+      <c r="I48" s="3" t="n">
+        <v>520</v>
+      </c>
+      <c r="J48" s="3" t="n">
+        <v>598</v>
+      </c>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>